<commit_message>
docs(xlsx): catatan — original tidak memakai Open Data API (0 request di baseline)
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,6 +92,10 @@
       <b val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -154,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -231,6 +235,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -11108,14 +11113,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A3:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.88" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="22" t="inlineStr">
         <is>
@@ -11164,9 +11167,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="22" t="inlineStr">
         <is>
@@ -11191,9 +11191,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="22" t="inlineStr">
         <is>
@@ -11256,7 +11253,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="22" t="inlineStr">
         <is>
@@ -11288,7 +11284,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="22" t="inlineStr">
         <is>
@@ -11308,8 +11303,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="22" t="inlineStr">
         <is>
@@ -11340,7 +11333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -11697,7 +11690,26 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="38" t="inlineStr">
+        <is>
+          <t>CATATAN PENTING</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Web original (cuaca.bmkg.go.id) TIDAK memakai API Open Data ini sama sekali — dia memakai API internal ISDP-nya sendiri (hasil scraping 159 request, 0 request ke api.bmkg.go.id/data.bmkg.go.id). Bentuk data mirip karena berasal dari sistem produksi yang sama. Pemakaian Open Data di project ini = keputusan redesign kita sendiri (jalur resmi tanpa proxy), bukan meniru original.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A13:I15"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(xlsx): kolom Endpoint = full URL upstream (https://cuaca.bmkg.go.id/...) di semua baris
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -691,7 +691,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>/api/df/v1/forecast/coord</t>
+          <t>https://cuaca.bmkg.go.id/api/df/v1/forecast/coord</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>/api/df/v1/adm/coord</t>
+          <t>https://cuaca.bmkg.go.id/api/df/v1/adm/coord</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>/api/df/v1/amandemen/coord</t>
+          <t>https://cuaca.bmkg.go.id/api/df/v1/amandemen/coord</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>/api/presentwx/coord</t>
+          <t>https://cuaca.bmkg.go.id/api/presentwx/coord</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>/api/public/weather/warning</t>
+          <t>https://cuaca.bmkg.go.id/api/public/weather/warning</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>/api/public/weather/warning/cyclone</t>
+          <t>https://cuaca.bmkg.go.id/api/public/weather/warning/cyclone</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>/api/public/weather/weekly-temperature</t>
+          <t>https://cuaca.bmkg.go.id/api/public/weather/weekly-temperature</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>/api/public/weather/video-latest</t>
+          <t>https://cuaca.bmkg.go.id/api/public/weather/video-latest</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>/api/public/banners</t>
+          <t>https://cuaca.bmkg.go.id/api/public/banners</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/setting/find-code</t>
+          <t>https://cuaca.bmkg.go.id/api/v1/setting/find-code</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/sunset/json</t>
+          <t>https://cuaca.bmkg.go.id/api/v1/sunset/json</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/tcwc/cyclone/all</t>
+          <t>https://cuaca.bmkg.go.id/api/v1/tcwc/cyclone/all</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/public/maritim/nearest-location</t>
+          <t>https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/maritim/route</t>
+          <t>https://cuaca.bmkg.go.id/api/v1/maritim/route</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/maritim/water-area/water_area_point.geojson</t>
+          <t>https://cuaca.bmkg.go.id/api/v1/maritim/water-area/water_area_point.geojson</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/sus/modelrun</t>
+          <t>https://cuaca.bmkg.go.id/api/v1/sus/modelrun</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/api/signature/impact/public/list/&lt;YYYY-MM-DDT00:00:00Z&gt;</t>
+          <t>https://cuaca.bmkg.go.id/api/v1/api/signature/impact/public/list/&lt;YYYY-MM-DDT00:00:00Z&gt;</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/maps/{general,warning,maritim,aviation,tourism}/metadata/tiles</t>
+          <t>https://cuaca.bmkg.go.id/api/v1/maps/{general,warning,maritim,aviation,tourism}/metadata/tiles</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/tourism/tiles/data/tourism.json</t>
+          <t>https://cuaca.bmkg.go.id/api/v1/tourism/tiles/data/tourism.json</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/sus/tiles/data/suspoi.json</t>
+          <t>https://cuaca.bmkg.go.id/api/v1/sus/tiles/data/suspoi.json</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/spartan/pollution/{pol}/{lvl}/{t0}/{t1}/{z}/{x}/{y}.png</t>
+          <t>https://cuaca.bmkg.go.id/api/v1/spartan/pollution/{pol}/{lvl}/{t0}/{t1}/{z}/{x}/{y}.png</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/user/subscribe-type</t>
+          <t>https://cuaca.bmkg.go.id/api/v1/user/subscribe-type</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/developer/{login,register,token-management,token-management/services}</t>
+          <t>https://cuaca.bmkg.go.id/api/v1/developer/{login,register,token-management,token-management/services}</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>spartan.bmkg.go.id/map/modelrun</t>
+          <t>https://spartan.bmkg.go.id/map/modelrun</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>widis.bmkg.go.id/ndf/cgms/weather/forward</t>
+          <t>https://widis.bmkg.go.id/ndf/cgms/weather/forward</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>bmkg-sus.geo.id/windmap/ecmwf/1000</t>
+          <t>https://bmkg-sus.geo.id/windmap/ecmwf/1000</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>tiles.circlegeo.com/data/{indocg,administration}.json</t>
+          <t>https://tiles.circlegeo.com/data/{indocg,administration}.json</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>cuaca.bmkg.go.id/blog/wp-json/wp/v2/</t>
+          <t>https://cuaca.bmkg.go.id/blog/wp-json/wp/v2/</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>data.bmkg.go.id/DataMKG/TEWS/gempadirasakan.json</t>
+          <t>https://data.bmkg.go.id/DataMKG/TEWS/gempadirasakan.json</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>nominatim.openstreetmap.org (search/reverse)</t>
+          <t>https://nominatim.openstreetmap.org (search/reverse)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2491,7 +2491,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>overpass-api.de/api/interpreter</t>
+          <t>https://overpass-api.de/api/interpreter</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>router.project-osrm.org/route/v1/driving</t>
+          <t>https://router.project-osrm.org/route/v1/driving</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs: API Maritim public_api (perairan 232 + pelabuhan 294 + geojson + overview) & gempa terverifikasi — sample response tersimpan; api-reference & xlsx update
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -11333,7 +11333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -11592,7 +11592,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Belum dipakai</t>
+          <t>404 saat dicek (11 Sep 2026) — dinyatakan ada di halaman open data, path belum aktif; gempaterkini.json ✅ 200</t>
         </is>
       </c>
     </row>
@@ -11690,6 +11690,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="38" t="inlineStr">
         <is>
@@ -11704,8 +11705,241 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15"/>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Maritim: Cuaca Perairan</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>GET https://maritim.bmkg.go.id/public_api/perairan/{file}</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>file dari perairan_list (232 wilayah)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>4 slot: 12-12-24-24 jam</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>per rilis stasiun</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>weather, weather_desc (narasi), warning_desc (pd cuaca buruk), wave_cat/desc, wind_from/to/speed. Kode wilayah F.09 = sama dgn internal nearest-location → cocok card Pesisir &amp; Laut / Pelayaran / WaveRadarMap</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Maritim: index+list</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>GET https://maritim.bmkg.go.id/public_api/{perairan_list|pelabuhan_list}</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>232 perairan + 294 pelabuhan</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>per rilis</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Daftar file data; sample tersimpan di baseline/open-data/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Maritim: GeoJSON wilayah</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>GET https://maritim.bmkg.go.id/public_api/static/wilayah_perairan.json</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>GeoJSON</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>polygon 232 wilayah + kode</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>725 KB — untuk overlay peta + lookup code</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Maritim: Overview gelombang</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>GET https://maritim.bmkg.go.id/public_api/overview/gelombang.json</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>kategori gelombang per wilayah (today/tmr/h2/h3)</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>per rilis</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>ringkas utk badge peta</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Maritim: Cuaca Pelabuhan</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>GET https://maritim.bmkg.go.id/public_api/pelabuhan/{file}</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>file dari pelabuhan_list (294 pelabuhan)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2 rilis terakhir</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>per rilis</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>arus (current_*), visibility, rh, temp, PASUT low/high tide → card Pelayaran/Pelabuhan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A13:I15"/>

</xml_diff>

<commit_message>
docs(xlsx): sheet 'Temuan API Resmi' — list API resmi + contoh sample asli per endpoint (modal diskusi tim)
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Mapping" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Official Open Data" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Temuan API Resmi" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Official Open Data" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Mapping'!$A$1:$L$33</definedName>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -96,6 +97,25 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -158,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -236,6 +256,13 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2612,6 +2639,719 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>TEMUAN SCRAPPING API RESMI BMKG — 11 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>Sumber: daftar API resmi dari partner BMKG (Maritim/Cuaca/Cuaca Ekstrem; Penerbangan &amp; DWT menyusul) + halaman data.bmkg.go.id. Sample asli tersimpan: scrapping_cuaca-bmkg-go-id/baseline/open-data/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="41" t="inlineStr">
+        <is>
+          <t>Layanan</t>
+        </is>
+      </c>
+      <c r="C4" s="41" t="inlineStr">
+        <is>
+          <t>Endpoint (full URL)</t>
+        </is>
+      </c>
+      <c r="D4" s="41" t="inlineStr">
+        <is>
+          <t>Params</t>
+        </is>
+      </c>
+      <c r="E4" s="41" t="inlineStr">
+        <is>
+          <t>Field utama respons</t>
+        </is>
+      </c>
+      <c r="F4" s="41" t="inlineStr">
+        <is>
+          <t>Contoh value (dari sample ASLI)</t>
+        </is>
+      </c>
+      <c r="G4" s="41" t="inlineStr">
+        <is>
+          <t>Pemakaian di redesign</t>
+        </is>
+      </c>
+      <c r="H4" s="41" t="inlineStr">
+        <is>
+          <t>CORS/Akses</t>
+        </is>
+      </c>
+      <c r="I4" s="41" t="inlineStr">
+        <is>
+          <t>Sample file</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="42" t="inlineStr">
+        <is>
+          <t>A. PRAKIRAAN CUACA (api.bmkg.go.id) — resmi, 3 hari per 3 jam</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="43" t="inlineStr">
+        <is>
+          <t>Prakiraan Cuaca per desa</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://api.bmkg.go.id/publik/prakiraan-cuaca?adm4=31.71.03.1001</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>adm4 (kode Kemendagri tkt IV)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>t, hu, weather_desc, weather_desc_en, ws, wd, wd_deg, tcc, tp, vs_text, image</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>t=29°C, hu=70%, weather_desc="Cerah", ws=8.6 km/h, wd="SE", tcc=36%, tp=0.1mm</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Dashboard (3-harian hourly) — jalur DIRECT pengganti proxy</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>CORS * → DIRECT, 60 req/menit/IP</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>prakiraan-cuaca_adm4-31.71.03.1001.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="42" t="inlineStr">
+        <is>
+          <t>B. MARITIM (maritim.bmkg.go.id/public_api) — resmi, dari daftar partner</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="43" t="inlineStr">
+        <is>
+          <t>Cuaca Perairan (232 wilayah)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://maritim.bmkg.go.id/public_api/perairan/{file}  (list: /public_api/perairan_list)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>file (contoh F.09_Teluk Jakarta.json)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>weather, weather_desc (narasi), warning_desc, wave_cat, wave_desc, wind_from/to, wind_speed_min/max, area_remark</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>weather="Cerah Berawan", warning_desc="Waspada Angin Kencang", wave_cat="Rendah", wave_desc="0.5-1.25 m", wind 5-14 knot; 4 slot 12-12-24-24 jam</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Card Aktivitas Pesisir &amp; Laut, Pelayaran, WaveRadarMap</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>maritim_perairan_F.09_Teluk-Jakarta.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="43" t="inlineStr">
+        <is>
+          <t>Cuaca Pelabuhan (294 pelabuhan)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>https://maritim.bmkg.go.id/public_api/pelabuhan/{file}  (list: /public_api/pelabuhan_list)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>file (contoh 0088_Sintete.json)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>semua field perairan + current_from/to, current_speed, visibility, rh_min/max, temp_min/max, low/high_tide + jam</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>visibility=2111, rh 89-100%, temp 25°C, current 0.06-0.33 cm/s, low_tide=-0.79 (15:00 UTC), high_tide=0.65 (21:00 UTC)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Card Pelayaran/Pelabuhan + info pasut</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>maritim_pelabuhan_0088_Sintete.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="43" t="inlineStr">
+        <is>
+          <t>Peta wilayah perairan</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>https://maritim.bmkg.go.id/public_api/static/wilayah_perairan.json</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>GeoJSON FeatureCollection polygon 232 wilayah + kode</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>type=Polygon, koordinat teluk/ laut (725 KB)</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Overlay peta + lookup kode wilayah</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>maritim_wilayah_perairan.geojson</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="43" t="inlineStr">
+        <is>
+          <t>Overview gelombang</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>https://maritim.bmkg.go.id/public_api/overview/gelombang.json</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>per kode wilayah: issued, today, tomorrow, h2, h3</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>F.09: today="Rendah", tomorrow="Rendah" | U.04: "Tinggi" (11 Sep 2026)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Badge status gelombang di peta/list</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>maritim_overview_gelombang.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="42" t="inlineStr">
+        <is>
+          <t>C. GEMPABUMI (data.bmkg.go.id/DataMKG/TEWS) — resmi, sudah dipakai redesign</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="43" t="inlineStr">
+        <is>
+          <t>Gempa terbaru M5.0+</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>https://data.bmkg.go.id/DataMKG/TEWS/autogempa.json</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Tanggal, Jam, DateTime, Coordinates, Lintang, Bujur, Magnitude, Kedalaman, Wilayah, Potensi</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Magnitude=2.7, Kedalaman=4 km, Wilayah="...6 km barat laut Kab. Bener Meriah" (11 Sep 2026 13:00 WIB)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>EarthquakeActivity ✅ (sudah dipakai)</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>gempa_autogempa.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" s="43" t="inlineStr">
+        <is>
+          <t>Gempa M5.0+ terkini (15)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>https://data.bmkg.go.id/DataMKG/TEWS/gempaterkini.json</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>array gempa: field sama dengan autogempa</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Magnitude=5.2, "46 km Tenggara MALUKUBRTDAYA" (10 Sep 2026)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>EarthquakeHistory ✅</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>gempa_gempaterkini.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" s="43" t="inlineStr">
+        <is>
+          <t>Gempa Dirasakan</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>https://data.bmkg.go.id/DataMKG/TEWS/gempadirasakan.json</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>gempa + data dirasakan</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>(4.5 KB sample, beberapa peristiwa)</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>EarthquakeHistory ✅</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>gempa_gempadirasakan.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="43" t="inlineStr">
+        <is>
+          <t>Gempa Potensi Tsunami</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>https://data.bmkg.go.id/DataMKG/TEWS/tsunamiterkini.json</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>404 saat dicek (11 Sep 2026) — disebut di halaman open data tapi path belum aktif</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>(404)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="42" t="inlineStr">
+        <is>
+          <t>D. CUACA EKSTREM / PERINGATAN DINI (data.bmkg.go.id/peringatan-dini-cuaca) — resmi</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="43" t="inlineStr">
+        <is>
+          <t>Nowcast RSS (per provinsi)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bmkg.go.id/alerts/nowcast/id</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>RSS: title, link (CAP), description, pubDate</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>3 item: "Hujan Lebat disertai Petir di Sumatera Barat / Sulawesi Tengah / Aceh"</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Kandidat pengganti warning internal (butuh adapter RSS)</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT (perlu cek CORS)</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>nowcast_rss.xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="43" t="inlineStr">
+        <is>
+          <t>Nowcast CAP detail</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bmkg.go.id/alerts/nowcast/id/{kode_detail_cap}_alert.xml</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>kode_detail_cap dari RSS</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>CAP 1.2: event, severity, certainty, expires, description (kecamatan terdampak), areaDesc</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>event="Hujan Lebat dan Petir", severity=Moderate, kecamatan: Bungus Teluk Kabung, Koto Xi Tarusan, Padang Selatan, Siberut Barat Daya</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Alert detail s/d kecamatan</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>DIRECT (perlu cek CORS)</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>nowcast_cap_sumbab.xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="42" t="inlineStr">
+        <is>
+          <t>E. MENYUSUL (dari daftar partner — belum tersedia)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B21" s="43" t="inlineStr">
+        <is>
+          <t>API Penerbangan</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>menyusul</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Card Aktivitas Penerbangan</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>menunggu partner</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B22" s="43" t="inlineStr">
+        <is>
+          <t>API DWT (Digital Weather for Traffic)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>menyusul</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Card Weather for Traffic / TransportWeather</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>menunggu partner</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A7:I7"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A20:I20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2761,7 +3501,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11107,7 +11847,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11327,7 +12067,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11690,7 +12430,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="38" t="inlineStr">
         <is>
@@ -11705,100 +12444,8 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Maritim: Cuaca Perairan</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>GET https://maritim.bmkg.go.id/public_api/perairan/{file}</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>file dari perairan_list (232 wilayah)</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>JSON</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>4 slot: 12-12-24-24 jam</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>per rilis stasiun</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>DIRECT</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>weather, weather_desc (narasi), warning_desc (pd cuaca buruk), wave_cat/desc, wind_from/to/speed. Kode wilayah F.09 = sama dgn internal nearest-location → cocok card Pesisir &amp; Laut / Pelayaran / WaveRadarMap</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Maritim: index+list</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>GET https://maritim.bmkg.go.id/public_api/{perairan_list|pelabuhan_list}</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>JSON</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>232 perairan + 294 pelabuhan</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>per rilis</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>DIRECT</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>Daftar file data; sample tersimpan di baseline/open-data/</t>
-        </is>
-      </c>
-    </row>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(xlsx): header kolom A & judul sheet Temuan API Resmi tidak terbaca (font putih tanpa background)
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -116,6 +116,11 @@
       <color rgb="001F4E79"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="14"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -178,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -263,6 +268,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2654,7 +2663,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>TEMUAN SCRAPPING API RESMI BMKG — 11 Sep 2026</t>
         </is>
@@ -2668,7 +2677,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="39" t="inlineStr">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
fix(xlsx): normalisasi warna ARGB 00→FF (168 cell) — header transparan di WPS kini opaque
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="21">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -121,8 +121,52 @@
       <color rgb="001F4E79"/>
       <sz val="14"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1F4E79"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF006100"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF7F6000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF9C0006"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF9C6500"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1F4E79"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1F4E79"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -169,6 +213,46 @@
         <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBDD7EE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -183,7 +267,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -272,6 +356,49 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -655,62 +782,62 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="46" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="46" t="inlineStr">
         <is>
           <t>Family</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="46" t="inlineStr">
         <is>
           <t>Endpoint</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="46" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="46" t="inlineStr">
         <is>
           <t>Params</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="46" t="inlineStr">
         <is>
           <t>Auth</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="46" t="inlineStr">
         <is>
           <t>Akses (dev)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="46" t="inlineStr">
         <is>
           <t>Dipakai di Original (baseline)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="46" t="inlineStr">
         <is>
           <t>Komponen Redesign</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="46" t="inlineStr">
         <is>
           <t>Status Redesign</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="46" t="inlineStr">
         <is>
           <t>Sumber Pengganti (Redesign)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="46" t="inlineStr">
         <is>
           <t>Catatan / Response Shape</t>
         </is>
@@ -745,7 +872,7 @@
           <t>Referer+Origin</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="47" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -760,7 +887,7 @@
           <t>CurrentWeather.vue, ForecastPanel.vue, ForecastTemperatureChart.vue, ForecastPrecipitationChart.vue, ForecastAirQualityChart.vue</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="48" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
@@ -805,7 +932,7 @@
           <t>Referer+Origin</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="47" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -820,7 +947,7 @@
           <t>App.vue (geolocation handler)</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="48" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
@@ -865,7 +992,7 @@
           <t>Referer+Origin</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="47" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -880,7 +1007,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="49" t="inlineStr">
         <is>
           <t>SEBAGIAN</t>
         </is>
@@ -925,7 +1052,7 @@
           <t>Terbuka</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -940,7 +1067,7 @@
           <t>CurrentWeather.vue</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="48" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
@@ -985,7 +1112,7 @@
           <t>x-public-token</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="47" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -1000,7 +1127,7 @@
           <t>AlertsPanel.vue</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="48" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
@@ -1045,7 +1172,7 @@
           <t>x-public-token</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="47" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -1060,7 +1187,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J7" s="7" t="inlineStr">
+      <c r="J7" s="51" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -1105,7 +1232,7 @@
           <t>x-public-token</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="47" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -1120,7 +1247,7 @@
           <t>ForecastTemperatureChart.vue</t>
         </is>
       </c>
-      <c r="J8" s="7" t="inlineStr">
+      <c r="J8" s="51" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -1165,7 +1292,7 @@
           <t>x-public-token</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="47" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -1180,7 +1307,7 @@
           <t>NewsSection.vue</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J9" s="48" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
@@ -1225,7 +1352,7 @@
           <t>x-public-token</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="47" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -1240,7 +1367,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="J10" s="51" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -1285,7 +1412,7 @@
           <t>Terbuka</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="G11" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -1300,7 +1427,7 @@
           <t>src/data/cityThemes.ts</t>
         </is>
       </c>
-      <c r="J11" s="8" t="inlineStr">
+      <c r="J11" s="52" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -1345,7 +1472,7 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G12" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -1360,7 +1487,7 @@
           <t>CurrentWeather.vue (sunrise/sunset untuk day/night)</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J12" s="48" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
@@ -1405,7 +1532,7 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G13" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -1420,7 +1547,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J13" s="48" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
@@ -1465,7 +1592,7 @@
           <t>x-public-token</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="47" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -1480,7 +1607,7 @@
           <t>WaveRadarMap.vue / MaritimeAdvisorDrawer.vue</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="J14" s="49" t="inlineStr">
         <is>
           <t>SEBAGIAN</t>
         </is>
@@ -1525,7 +1652,7 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -1540,7 +1667,7 @@
           <t>TransportWeather.vue</t>
         </is>
       </c>
-      <c r="J15" s="8" t="inlineStr">
+      <c r="J15" s="52" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -1585,7 +1712,7 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="G16" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -1600,7 +1727,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr">
+      <c r="J16" s="51" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -1645,7 +1772,7 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G17" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -1660,7 +1787,7 @@
           <t>SatelliteMap.vue</t>
         </is>
       </c>
-      <c r="J17" s="8" t="inlineStr">
+      <c r="J17" s="52" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -1705,7 +1832,7 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G18" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -1720,7 +1847,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J18" s="7" t="inlineStr">
+      <c r="J18" s="51" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -1765,7 +1892,7 @@
           <t>campuran</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G19" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -1780,7 +1907,7 @@
           <t>SatelliteMap.vue, WaveRadarMap.vue</t>
         </is>
       </c>
-      <c r="J19" s="8" t="inlineStr">
+      <c r="J19" s="52" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -1825,7 +1952,7 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G20" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -1840,7 +1967,7 @@
           <t>LandBasedActivities.vue</t>
         </is>
       </c>
-      <c r="J20" s="8" t="inlineStr">
+      <c r="J20" s="52" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -1885,7 +2012,7 @@
           <t>X-API-KEY</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="G21" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -1900,7 +2027,7 @@
           <t>LandBasedActivities.vue</t>
         </is>
       </c>
-      <c r="J21" s="8" t="inlineStr">
+      <c r="J21" s="52" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -1945,7 +2072,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="G22" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -1960,7 +2087,7 @@
           <t>ForecastAirQualityChart.vue</t>
         </is>
       </c>
-      <c r="J22" s="7" t="inlineStr">
+      <c r="J22" s="51" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -2005,7 +2132,7 @@
           <t>x-public-token</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G23" s="47" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -2020,7 +2147,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J23" s="7" t="inlineStr">
+      <c r="J23" s="51" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -2065,7 +2192,7 @@
           <t>Akun dev</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="G24" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -2080,7 +2207,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J24" s="7" t="inlineStr">
+      <c r="J24" s="51" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -2125,7 +2252,7 @@
           <t>Terbuka</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="G25" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -2140,7 +2267,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J25" s="7" t="inlineStr">
+      <c r="J25" s="51" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -2185,7 +2312,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="G26" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -2200,7 +2327,7 @@
           <t>SatelliteMap.vue</t>
         </is>
       </c>
-      <c r="J26" s="8" t="inlineStr">
+      <c r="J26" s="52" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -2245,7 +2372,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="G27" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -2260,7 +2387,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J27" s="7" t="inlineStr">
+      <c r="J27" s="51" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -2305,7 +2432,7 @@
           <t>Terbuka</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="G28" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -2320,7 +2447,7 @@
           <t>SatelliteMap.vue</t>
         </is>
       </c>
-      <c r="J28" s="8" t="inlineStr">
+      <c r="J28" s="52" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -2365,7 +2492,7 @@
           <t>Terbuka</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G29" s="47" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -2380,7 +2507,7 @@
           <t>NewsSection.vue</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="J29" s="48" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
@@ -2425,7 +2552,7 @@
           <t>Terbuka</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="G30" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -2440,7 +2567,7 @@
           <t>EarthquakeActivity.vue, EarthquakeHistory.vue</t>
         </is>
       </c>
-      <c r="J30" s="9" t="inlineStr">
+      <c r="J30" s="53" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
@@ -2485,7 +2612,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="G31" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -2500,7 +2627,7 @@
           <t>App.vue, LandBasedActivities.vue</t>
         </is>
       </c>
-      <c r="J31" s="9" t="inlineStr">
+      <c r="J31" s="53" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
@@ -2545,7 +2672,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
+      <c r="G32" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -2560,7 +2687,7 @@
           <t>LandBasedActivities.vue</t>
         </is>
       </c>
-      <c r="J32" s="9" t="inlineStr">
+      <c r="J32" s="53" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
@@ -2605,7 +2732,7 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="G33" s="50" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -2620,7 +2747,7 @@
           <t>TransportWeather.vue</t>
         </is>
       </c>
-      <c r="J33" s="9" t="inlineStr">
+      <c r="J33" s="53" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
@@ -2663,7 +2790,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="45" t="inlineStr">
+      <c r="A1" s="54" t="inlineStr">
         <is>
           <t>TEMUAN SCRAPPING API RESMI BMKG — 11 Sep 2026</t>
         </is>
@@ -2676,55 +2803,56 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="A4" s="55" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B4" s="41" t="inlineStr">
+      <c r="B4" s="56" t="inlineStr">
         <is>
           <t>Layanan</t>
         </is>
       </c>
-      <c r="C4" s="41" t="inlineStr">
+      <c r="C4" s="56" t="inlineStr">
         <is>
           <t>Endpoint (full URL)</t>
         </is>
       </c>
-      <c r="D4" s="41" t="inlineStr">
+      <c r="D4" s="56" t="inlineStr">
         <is>
           <t>Params</t>
         </is>
       </c>
-      <c r="E4" s="41" t="inlineStr">
+      <c r="E4" s="56" t="inlineStr">
         <is>
           <t>Field utama respons</t>
         </is>
       </c>
-      <c r="F4" s="41" t="inlineStr">
+      <c r="F4" s="56" t="inlineStr">
         <is>
           <t>Contoh value (dari sample ASLI)</t>
         </is>
       </c>
-      <c r="G4" s="41" t="inlineStr">
+      <c r="G4" s="56" t="inlineStr">
         <is>
           <t>Pemakaian di redesign</t>
         </is>
       </c>
-      <c r="H4" s="41" t="inlineStr">
+      <c r="H4" s="56" t="inlineStr">
         <is>
           <t>CORS/Akses</t>
         </is>
       </c>
-      <c r="I4" s="41" t="inlineStr">
+      <c r="I4" s="56" t="inlineStr">
         <is>
           <t>Sample file</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="42" t="inlineStr">
+      <c r="A5" s="57" t="inlineStr">
         <is>
           <t>A. PRAKIRAAN CUACA (api.bmkg.go.id) — resmi, 3 hari per 3 jam</t>
         </is>
@@ -2776,7 +2904,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="42" t="inlineStr">
+      <c r="A7" s="57" t="inlineStr">
         <is>
           <t>B. MARITIM (maritim.bmkg.go.id/public_api) — resmi, dari daftar partner</t>
         </is>
@@ -2963,7 +3091,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="42" t="inlineStr">
+      <c r="A12" s="57" t="inlineStr">
         <is>
           <t>C. GEMPABUMI (data.bmkg.go.id/DataMKG/TEWS) — resmi, sudah dipakai redesign</t>
         </is>
@@ -3150,7 +3278,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="42" t="inlineStr">
+      <c r="A17" s="57" t="inlineStr">
         <is>
           <t>D. CUACA EKSTREM / PERINGATAN DINI (data.bmkg.go.id/peringatan-dini-cuaca) — resmi</t>
         </is>
@@ -3247,7 +3375,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="42" t="inlineStr">
+      <c r="A20" s="57" t="inlineStr">
         <is>
           <t>E. MENYUSUL (dari daftar partner — belum tersedia)</t>
         </is>
@@ -3376,6 +3504,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -3399,7 +3528,7 @@
       <c r="C4" s="11" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="58" t="inlineStr">
         <is>
           <t>TERIMPLEMENTASI</t>
         </is>
@@ -3414,7 +3543,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="59" t="inlineStr">
         <is>
           <t>SEBAGIAN</t>
         </is>
@@ -3429,7 +3558,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="60" t="inlineStr">
         <is>
           <t>BELUM</t>
         </is>
@@ -3444,7 +3573,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="61" t="inlineStr">
         <is>
           <t>BEDA-SUMBER</t>
         </is>
@@ -3459,7 +3588,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="62" t="inlineStr">
         <is>
           <t>REDESIGN-ONLY</t>
         </is>
@@ -3488,7 +3617,7 @@
       <c r="C11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="63" t="inlineStr">
         <is>
           <t>Endpoint original terimplementasi identik (pakai API yang sama)</t>
         </is>
@@ -3498,6 +3627,7 @@
       </c>
       <c r="C12" s="2" t="n"/>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
@@ -3546,22 +3676,22 @@
         </is>
       </c>
       <c r="F1" s="23" t="n"/>
-      <c r="G1" s="24" t="inlineStr">
+      <c r="G1" s="64" t="inlineStr">
         <is>
           <t>API READY</t>
         </is>
       </c>
-      <c r="H1" s="24" t="inlineStr">
+      <c r="H1" s="64" t="inlineStr">
         <is>
           <t>Endpoint BMKG (path)</t>
         </is>
       </c>
-      <c r="I1" s="24" t="inlineStr">
+      <c r="I1" s="64" t="inlineStr">
         <is>
           <t>Keterangan</t>
         </is>
       </c>
-      <c r="J1" s="24" t="inlineStr">
+      <c r="J1" s="64" t="inlineStr">
         <is>
           <t>Akses di Dev</t>
         </is>
@@ -3627,7 +3757,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G4" s="28" t="inlineStr">
+      <c r="G4" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -3642,7 +3772,7 @@
           <t>GPS → alamat admin; sudah dipakai redesign</t>
         </is>
       </c>
-      <c r="J4" s="30" t="inlineStr">
+      <c r="J4" s="66" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -3670,7 +3800,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G5" s="28" t="inlineStr">
+      <c r="G5" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -3685,7 +3815,7 @@
           <t>field lokasi.timezone (deteksi WIB/WITA/WIT)</t>
         </is>
       </c>
-      <c r="J5" s="30" t="inlineStr">
+      <c r="J5" s="66" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -3709,7 +3839,7 @@
         </is>
       </c>
       <c r="F6" s="23" t="n"/>
-      <c r="G6" s="28" t="inlineStr">
+      <c r="G6" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -3724,7 +3854,7 @@
           <t>observasi aktual kartu kondisi saat ini</t>
         </is>
       </c>
-      <c r="J6" s="31" t="inlineStr">
+      <c r="J6" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -3745,7 +3875,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G7" s="32" t="inlineStr">
+      <c r="G7" s="68" t="inlineStr">
         <is>
           <t>NO API</t>
         </is>
@@ -3788,7 +3918,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G8" s="32" t="inlineStr">
+      <c r="G8" s="68" t="inlineStr">
         <is>
           <t>NO API</t>
         </is>
@@ -3831,7 +3961,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G9" s="28" t="inlineStr">
+      <c r="G9" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -3846,7 +3976,7 @@
           <t>per koordinat kota</t>
         </is>
       </c>
-      <c r="J9" s="30" t="inlineStr">
+      <c r="J9" s="66" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -3874,7 +4004,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G10" s="34" t="inlineStr">
+      <c r="G10" s="69" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -3917,7 +4047,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G11" s="34" t="inlineStr">
+      <c r="G11" s="69" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -3932,7 +4062,7 @@
           <t>Tidak ada JSON AQI — hanya tile polusi untuk peta</t>
         </is>
       </c>
-      <c r="J11" s="31" t="inlineStr">
+      <c r="J11" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -3956,7 +4086,7 @@
         </is>
       </c>
       <c r="F12" s="23" t="n"/>
-      <c r="G12" s="28" t="inlineStr">
+      <c r="G12" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -3971,7 +4101,7 @@
           <t>sumber parameter: t, ws, wd, hu</t>
         </is>
       </c>
-      <c r="J12" s="31" t="inlineStr">
+      <c r="J12" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -3992,7 +4122,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G13" s="28" t="inlineStr">
+      <c r="G13" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4007,7 +4137,7 @@
           <t>field t (°C)</t>
         </is>
       </c>
-      <c r="J13" s="31" t="inlineStr">
+      <c r="J13" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -4028,7 +4158,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G14" s="28" t="inlineStr">
+      <c r="G14" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4043,7 +4173,7 @@
           <t>field ws (km/h)</t>
         </is>
       </c>
-      <c r="J14" s="31" t="inlineStr">
+      <c r="J14" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -4064,7 +4194,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G15" s="28" t="inlineStr">
+      <c r="G15" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4079,7 +4209,7 @@
           <t>field wd / wd_deg</t>
         </is>
       </c>
-      <c r="J15" s="31" t="inlineStr">
+      <c r="J15" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -4100,7 +4230,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G16" s="28" t="inlineStr">
+      <c r="G16" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4115,7 +4245,7 @@
           <t>field hu (%)</t>
         </is>
       </c>
-      <c r="J16" s="31" t="inlineStr">
+      <c r="J16" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -4143,7 +4273,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G17" s="32" t="inlineStr">
+      <c r="G17" s="68" t="inlineStr">
         <is>
           <t>NO API</t>
         </is>
@@ -4182,7 +4312,7 @@
         </is>
       </c>
       <c r="F18" s="23" t="n"/>
-      <c r="G18" s="28" t="inlineStr">
+      <c r="G18" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4197,7 +4327,7 @@
           <t>data[0].cuaca[0] = grup hourly</t>
         </is>
       </c>
-      <c r="J18" s="30" t="inlineStr">
+      <c r="J18" s="66" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -4218,7 +4348,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G19" s="28" t="inlineStr">
+      <c r="G19" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4233,7 +4363,7 @@
           <t>field t per jam</t>
         </is>
       </c>
-      <c r="J19" s="30" t="inlineStr">
+      <c r="J19" s="66" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -4254,7 +4384,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G20" s="28" t="inlineStr">
+      <c r="G20" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4269,7 +4399,7 @@
           <t>field tp (mm) per jam</t>
         </is>
       </c>
-      <c r="J20" s="30" t="inlineStr">
+      <c r="J20" s="66" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -4290,7 +4420,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G21" s="28" t="inlineStr">
+      <c r="G21" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4305,7 +4435,7 @@
           <t>field ws per jam</t>
         </is>
       </c>
-      <c r="J21" s="30" t="inlineStr">
+      <c r="J21" s="66" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -4326,7 +4456,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G22" s="28" t="inlineStr">
+      <c r="G22" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4341,7 +4471,7 @@
           <t>field hu per jam</t>
         </is>
       </c>
-      <c r="J22" s="30" t="inlineStr">
+      <c r="J22" s="66" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -4362,7 +4492,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G23" s="32" t="inlineStr">
+      <c r="G23" s="68" t="inlineStr">
         <is>
           <t>NO API</t>
         </is>
@@ -4401,7 +4531,7 @@
         </is>
       </c>
       <c r="F24" s="23" t="n"/>
-      <c r="G24" s="34" t="inlineStr">
+      <c r="G24" s="69" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -4437,7 +4567,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G25" s="32" t="inlineStr">
+      <c r="G25" s="68" t="inlineStr">
         <is>
           <t>NO API</t>
         </is>
@@ -4473,7 +4603,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G26" s="34" t="inlineStr">
+      <c r="G26" s="69" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -4488,7 +4618,7 @@
           <t>wilayah laut terdekat (code, name, wilpel, polygon)</t>
         </is>
       </c>
-      <c r="J26" s="30" t="inlineStr">
+      <c r="J26" s="66" t="inlineStr">
         <is>
           <t>PROXY</t>
         </is>
@@ -4509,7 +4639,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G27" s="28" t="inlineStr">
+      <c r="G27" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4524,7 +4654,7 @@
           <t>rute pelayaran + titik area laut</t>
         </is>
       </c>
-      <c r="J27" s="31" t="inlineStr">
+      <c r="J27" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -4545,7 +4675,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G28" s="28" t="inlineStr">
+      <c r="G28" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4560,7 +4690,7 @@
           <t>layer peta penerbangan + katalog run model</t>
         </is>
       </c>
-      <c r="J28" s="31" t="inlineStr">
+      <c r="J28" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -4584,7 +4714,7 @@
         </is>
       </c>
       <c r="F29" s="23" t="n"/>
-      <c r="G29" s="34" t="inlineStr">
+      <c r="G29" s="69" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -4599,7 +4729,7 @@
           <t>perlu reverse-engineering param; alternatif statis: inderaja HIMA</t>
         </is>
       </c>
-      <c r="J29" s="31" t="inlineStr">
+      <c r="J29" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -4620,7 +4750,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G30" s="34" t="inlineStr">
+      <c r="G30" s="69" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -4635,7 +4765,7 @@
           <t>belum ada endpoint JSON terdokumentasi</t>
         </is>
       </c>
-      <c r="J30" s="31" t="inlineStr">
+      <c r="J30" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -4656,7 +4786,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G31" s="34" t="inlineStr">
+      <c r="G31" s="69" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -4671,7 +4801,7 @@
           <t>citra awan via HIMA/widis</t>
         </is>
       </c>
-      <c r="J31" s="31" t="inlineStr">
+      <c r="J31" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -4692,7 +4822,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G32" s="34" t="inlineStr">
+      <c r="G32" s="69" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
@@ -4707,7 +4837,7 @@
           <t>tile curah hujan satelit</t>
         </is>
       </c>
-      <c r="J32" s="31" t="inlineStr">
+      <c r="J32" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -4728,7 +4858,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G33" s="28" t="inlineStr">
+      <c r="G33" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4743,7 +4873,7 @@
           <t>wind tiles ECMWF</t>
         </is>
       </c>
-      <c r="J33" s="31" t="inlineStr">
+      <c r="J33" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -4771,7 +4901,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G34" s="28" t="inlineStr">
+      <c r="G34" s="65" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
@@ -4786,7 +4916,7 @@
           <t>metadata layer peta (sources, layers, overlays)</t>
         </is>
       </c>
-      <c r="J34" s="31" t="inlineStr">
+      <c r="J34" s="67" t="inlineStr">
         <is>
           <t>DIRECT</t>
         </is>
@@ -4814,7 +4944,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G35" s="32" t="inlineStr">
+      <c r="G35" s="68" t="inlineStr">
         <is>
           <t>NO API</t>
         </is>
@@ -4857,7 +4987,7 @@
           <t>NOT YET</t>
         </is>
       </c>
-      <c r="G36" s="32" t="inlineStr">
+      <c r="G36" s="68" t="inlineStr">
         <is>
           <t>NO API</t>
         </is>
@@ -4892,7 +5022,7 @@
         </is>
       </c>
       <c r="F37" s="23" t="n"/>
-      <c r="G37" s="32" t="inlineStr">
+      <c r="G37" s="68" t="inlineStr">
         <is>
           <t>NO API</t>
         </is>
@@ -11862,12 +11992,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:H31"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.88" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="22" t="inlineStr">
         <is>
@@ -11916,6 +12048,9 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="22" t="inlineStr">
         <is>
@@ -11940,6 +12075,9 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="22" t="inlineStr">
         <is>
@@ -12002,6 +12140,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="22" t="inlineStr">
         <is>
@@ -12033,6 +12172,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="22" t="inlineStr">
         <is>
@@ -12052,6 +12192,8 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="22" t="inlineStr">
         <is>
@@ -12110,48 +12252,49 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
-      <c r="A4" s="37" t="inlineStr">
+      <c r="A4" s="70" t="inlineStr">
         <is>
           <t>Layanan</t>
         </is>
       </c>
-      <c r="B4" s="37" t="inlineStr">
+      <c r="B4" s="70" t="inlineStr">
         <is>
           <t>Endpoint</t>
         </is>
       </c>
-      <c r="C4" s="37" t="inlineStr">
+      <c r="C4" s="70" t="inlineStr">
         <is>
           <t>Params</t>
         </is>
       </c>
-      <c r="D4" s="37" t="inlineStr">
+      <c r="D4" s="70" t="inlineStr">
         <is>
           <t>Format</t>
         </is>
       </c>
-      <c r="E4" s="37" t="inlineStr">
+      <c r="E4" s="70" t="inlineStr">
         <is>
           <t>Coverage</t>
         </is>
       </c>
-      <c r="F4" s="37" t="inlineStr">
+      <c r="F4" s="70" t="inlineStr">
         <is>
           <t>Update</t>
         </is>
       </c>
-      <c r="G4" s="37" t="inlineStr">
+      <c r="G4" s="70" t="inlineStr">
         <is>
           <t>Limit</t>
         </is>
       </c>
-      <c r="H4" s="37" t="inlineStr">
+      <c r="H4" s="70" t="inlineStr">
         <is>
           <t>CORS</t>
         </is>
       </c>
-      <c r="I4" s="37" t="inlineStr">
+      <c r="I4" s="70" t="inlineStr">
         <is>
           <t>Keterangan</t>
         </is>
@@ -12439,6 +12582,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="38" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(xlsx): sheet 'Audit Content Card' — 22 item konten redesign dipetakan ke API knowledge base (10 LIVE, 7 READY, 3 PARTIAL, 4 TUNGGU)
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -8,10 +8,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Mapping" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Temuan API Resmi" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Official Open Data" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Content Card" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Official Open Data" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Mapping'!$A$1:$L$33</definedName>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="39">
+  <fonts count="44">
     <font>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -312,8 +313,31 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1F4E79"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="FF1F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF1F4E79"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="43">
+  <fills count="48">
     <fill>
       <patternFill/>
     </fill>
@@ -563,6 +587,31 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE699"/>
       </patternFill>
     </fill>
   </fills>
@@ -820,7 +869,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -903,6 +952,25 @@
     </xf>
     <xf numFmtId="0" fontId="37" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="42" fillId="43" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="44" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="45" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="47" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4221,6 +4289,839 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="44" t="inlineStr">
+        <is>
+          <t>AUDIT CONTENT WEB REDESIGN → SUMBER API (11 Sep 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="45" t="inlineStr">
+        <is>
+          <t>Pertanyaan audit: konten mana di web redesign yang bisa di-update valuenya dari hit API (knowledge base: internal BMKG + Open Data resmi + Maritim + DWT)?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="46" t="inlineStr">
+        <is>
+          <t>Status: ✅ LIVE = sudah terpasang  |  🔄 READY = API sudah kita pegang, tinggal pasang adapter  |  ⚠️ PARTIAL = separuh data/needs narasi  |  ⏳ TUNGGU = menunggu API partner / tidak ada</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="inlineStr">
+        <is>
+          <t>Card / Komponen</t>
+        </is>
+      </c>
+      <c r="C5" s="47" t="inlineStr">
+        <is>
+          <t>Konten (value yang tampil di UI)</t>
+        </is>
+      </c>
+      <c r="D5" s="47" t="inlineStr">
+        <is>
+          <t>Sumber sekarang</t>
+        </is>
+      </c>
+      <c r="E5" s="47" t="inlineStr">
+        <is>
+          <t>API dari knowledge base yang bisa supply</t>
+        </is>
+      </c>
+      <c r="F5" s="47" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G5" s="47" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="48" t="inlineStr">
+        <is>
+          <t>─ KOLOM HERO &amp; FORECAST ─</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="43" t="inlineStr">
+        <is>
+          <t>HeroWeatherCard</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Suhu, kondisi, hujan, angin, kelembapan, peluang hujan</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>liveHourly (useBmkgWeather) — fallback mock</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>internal df/forecast/coord</t>
+        </is>
+      </c>
+      <c r="F7" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="43" t="inlineStr">
+        <is>
+          <t>HeroWeatherCard</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Chart jam-an mini di hero</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>liveHourly</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>internal df/forecast/coord (7 hari)</t>
+        </is>
+      </c>
+      <c r="F8" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="43" t="inlineStr">
+        <is>
+          <t>CurrentWeather</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Card cuaca besar per kota terpilih</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>liveWeather</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>internal df/forecast/coord + adm/coord (geolokasi)</t>
+        </is>
+      </c>
+      <c r="F9" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="43" t="inlineStr">
+        <is>
+          <t>ForecastPanel</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Prakiraan 7 hari (panel forecast)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>liveHourly</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>internal df/forecast/coord</t>
+        </is>
+      </c>
+      <c r="F10" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Opsi pengurang beban proxy: official api.bmkg.go.id/publik/prakiraan-cuaca?adm4 (3 hari, DIRECT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="43" t="inlineStr">
+        <is>
+          <t>AlertsPanel</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Banner peringatan cuaca</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>liveAlerts (warning + cyclone internal)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>internal /api/public/weather/warning(+cyclone)</t>
+        </is>
+      </c>
+      <c r="F11" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Upgrade resmi: nowcast RSS/CAP (produk beda: 3-jam per kecamatan; item bisa stale)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="43" t="inlineStr">
+        <is>
+          <t>MajorCitiesCarousel</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Kondisi terkini antar kota (carousel)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>liveWeather per kota</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>internal df/forecast/coord</t>
+        </is>
+      </c>
+      <c r="F12" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="43" t="inlineStr">
+        <is>
+          <t>NewsSection</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Berita &amp; pengumuman</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>liveNews (WP BMKG) — fallback mock</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>blog WP BMKG (502 flaky)</t>
+        </is>
+      </c>
+      <c r="F13" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Upstream sering 502 — fallback mock jalan</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="43" t="inlineStr">
+        <is>
+          <t>EarthquakeActivity + History</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Gempa terbaru, dirasakan, riwayat</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>live TEWS</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>data.bmkg.go.id TEWS (autogempa/gempaterkini/gempadirasakan)</t>
+        </is>
+      </c>
+      <c r="F14" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="43" t="inlineStr">
+        <is>
+          <t>SatelliteMap</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Citra satelit Himawari-9</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>live internal</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>internal citra satelit</t>
+        </is>
+      </c>
+      <c r="F15" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="43" t="inlineStr">
+        <is>
+          <t>ComfortIndexCard</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Indeks kenyamanan</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>dihitung dari liveWeather</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>internal df/forecast/coord</t>
+        </is>
+      </c>
+      <c r="F16" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="48" t="inlineStr">
+        <is>
+          <t>─ KARTU AKTIVITAS (kolom 2) &amp; TRANSPORT ─</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B18" s="43" t="inlineStr">
+        <is>
+          <t>TransportWeather — Jalan Raya</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Status Aman/Waspada/Awas + narasi</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>MOCK transportStatusesMap</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>DWT apiDF_Darat: kode_cuaca, hujan, angin per kecamatan per jam UTC</t>
+        </is>
+      </c>
+      <c r="F18" s="50" t="inlineStr">
+        <is>
+          <t>🔄 READY</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Mapping: kode_cuaca 0-1→Aman, 3-7→Waspada, &gt;=10/AWS→Awas + narasi template</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B19" s="43" t="inlineStr">
+        <is>
+          <t>TransportWeather — Penerbangan</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Status bandara/sector udara</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>MOCK</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>API Penerbangan = menyusul (partner); sementara: tcc/vis dari df forecast</t>
+        </is>
+      </c>
+      <c r="F19" s="51" t="inlineStr">
+        <is>
+          <t>⏳ TUNGGU</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Partial jangka pendek pakai tcc dari forecast internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B20" s="43" t="inlineStr">
+        <is>
+          <t>TransportWeather — Maritim</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Status pelayaran + gelombang</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>MOCK</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>maritim public_api: perairan wave_cat/warning_desc; pelabuhan (pasut, arus)</t>
+        </is>
+      </c>
+      <c r="F20" s="50" t="inlineStr">
+        <is>
+          <t>🔄 READY</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Kode wilayah dari nearest-location internal sudah cocok (contoh F.09)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B21" s="43" t="inlineStr">
+        <is>
+          <t>TransportWeather — Kereta (slot baru)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Status jalur KAI</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>belum ada slot (kandidat tambahan)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>DWT apiDF_Kereta: 178 stasiun per jam UTC</t>
+        </is>
+      </c>
+      <c r="F21" s="50" t="inlineStr">
+        <is>
+          <t>🔄 READY</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Perlu slot UI baru kalau mau tampil</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B22" s="43" t="inlineStr">
+        <is>
+          <t>LandBasedActivities</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Cuaca per titik rute (aktivitas darat)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>MOCK hourlyForecastsMap (dipaksa match kota regional)</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>DWT apiDF_Darat: lat/lon kecamatan → match titik rute terdekat</t>
+        </is>
+      </c>
+      <c r="F22" s="50" t="inlineStr">
+        <is>
+          <t>🔄 READY</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Rute &amp; POI tetap Overpass OSM (bukan BMKG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B23" s="43" t="inlineStr">
+        <is>
+          <t>AroundActivityPanel</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Narasi analisis "Aktivitas Sekitar"</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>MOCK cityAnalysisMap (narasi fiktif per kota)</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>bisa disusun generator: df forecast + DWT darat + maritim</t>
+        </is>
+      </c>
+      <c r="F23" s="52" t="inlineStr">
+        <is>
+          <t>⚠️ PARTIAL</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Data ada semua, tapi perlu builder narasi; atau satukan konten faktual (suhu/hujan/angin) tanpa narasi fiktif</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B24" s="43" t="inlineStr">
+        <is>
+          <t>AirQualityCard</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>AQI, PM2.5, PM10, O3, NO2</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>PSEUDO: pm25 = f(temp)+seed — nilai fiktif</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>TIDAK ADA di knowledge base / daftar partner</t>
+        </is>
+      </c>
+      <c r="F24" s="51" t="inlineStr">
+        <is>
+          <t>⏳ TUNGGU</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Risiko etika UI: tampilan seperti data nyata padahal pseudo. Cari API ISPU BMKG (kualitas udara) terpisah atau tandai "ilustrasi"</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B25" s="43" t="inlineStr">
+        <is>
+          <t>WaveRadarMap</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Radar tinggi gelombang</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>MOCK (label "BMKG WaveWatch III")</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>maritim overview gelombang + perairan wave_cat/wave_desc</t>
+        </is>
+      </c>
+      <c r="F25" s="50" t="inlineStr">
+        <is>
+          <t>🔄 READY</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B26" s="43" t="inlineStr">
+        <is>
+          <t>WindMap + WeatherRadarMap</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Vektor angin, isobar, temperatur</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>SYNTHETIC generateIndonesiaGfsWindGrid (grid prosedural)</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>internal presentwx (family di baseline) / DWT angin per kecamatan</t>
+        </is>
+      </c>
+      <c r="F26" s="52" t="inlineStr">
+        <is>
+          <t>⚠️ PARTIAL</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Grid GFS asli tidak di knowledge base; DWT angin bisa jadi pengganti skala kecamatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B27" s="43" t="inlineStr">
+        <is>
+          <t>MaritimeAdvisorDrawer</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Sektor maritim: risiko, status cuaca, SOP, kontak</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>maritimeAdvisorData (static)</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>maritim perairan per wilayah (warning_desc, wave_cat)</t>
+        </is>
+      </c>
+      <c r="F27" s="50" t="inlineStr">
+        <is>
+          <t>🔄 READY</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>SOP checklist &amp; kontak memang by-design static</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B28" s="43" t="inlineStr">
+        <is>
+          <t>AviationAdvisorDrawer</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Sektor udara: pra-terbang, SOP, kontak</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>aviationAdvisorData (static)</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>API Penerbangan menyusul; sementara df forecast tcc</t>
+        </is>
+      </c>
+      <c r="F28" s="51" t="inlineStr">
+        <is>
+          <t>⏳ TUNGGU</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B29" s="43" t="inlineStr">
+        <is>
+          <t>MarineMap</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Peta maritim Indonesia</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>static indonesiaMapData + earthquakeData</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>maritim wilayah_perairan.geojson (polygon 232 wilayah)</t>
+        </is>
+      </c>
+      <c r="F29" s="50" t="inlineStr">
+        <is>
+          <t>🔄 READY (opsional)</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Layer polygon resmi per wilayah + kode</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A17:G17"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
@@ -4370,7 +5271,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12715,7 +13616,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12935,7 +13836,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs(xlsx): AirQualityCard ditandai PAUSED (keputusan diskusi)
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -337,7 +337,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="48">
+  <fills count="49">
     <fill>
       <patternFill/>
     </fill>
@@ -614,6 +614,11 @@
         <fgColor rgb="FFFFE699"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E6E6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="9">
     <border>
@@ -869,7 +874,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -971,6 +976,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="47" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4929,14 +4937,14 @@
           <t>TIDAK ADA di knowledge base / daftar partner</t>
         </is>
       </c>
-      <c r="F24" s="51" t="inlineStr">
-        <is>
-          <t>⏳ TUNGGU</t>
+      <c r="F24" s="53" t="inlineStr">
+        <is>
+          <t>⏸️ PAUSED (keputusan: urus nanti)</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>Risiko etika UI: tampilan seperti data nyata padahal pseudo. Cari API ISPU BMKG (kualitas udara) terpisah atau tandai "ilustrasi"</t>
+          <t>Risiko etika UI: tampilan seperti data nyata padahal pseudo. Cari API ISPU BMKG (kualitas udara) terpisah atau tandai "ilustrasi" — ⏸️ PAUSED sementara oleh keputusan (nilai pseudo dibiarkan sementara)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(xlsx): baris 12/16/19 sheet Audit Content Card belum ter-update (salah kolom match) — penerbangan PAUSED, narasi dinamis & DWT wind terpasang
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -4762,14 +4762,14 @@
           <t>API Penerbangan = menyusul (partner); sementara: tcc/vis dari df forecast</t>
         </is>
       </c>
-      <c r="F19" s="51" t="inlineStr">
-        <is>
-          <t>⏳ TUNGGU</t>
+      <c r="F19" s="53" t="inlineStr">
+        <is>
+          <t>⏸️ PAUSED (menunggu kesepakatan partner)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Partial jangka pendek pakai tcc dari forecast internal</t>
+          <t>Keputusan: di-pause, tunggu data dari partner; jangka pendek bisa derivasi tcc</t>
         </is>
       </c>
     </row>
@@ -4902,14 +4902,14 @@
           <t>bisa disusun generator: df forecast + DWT darat + maritim</t>
         </is>
       </c>
-      <c r="F23" s="52" t="inlineStr">
-        <is>
-          <t>⚠️ PARTIAL</t>
+      <c r="F23" s="49" t="inlineStr">
+        <is>
+          <t>✅ NARASI DINAMIS TERPASANG</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Data ada semua, tapi perlu builder narasi; atau satukan konten faktual (suhu/hujan/angin) tanpa narasi fiktif</t>
+          <t>buildCityAnalysis (analysisNarrative.ts): fakta cuaca → narasi per kondisi; fallback map statis</t>
         </is>
       </c>
     </row>
@@ -5003,14 +5003,14 @@
           <t>internal presentwx (family di baseline) / DWT angin per kecamatan</t>
         </is>
       </c>
-      <c r="F26" s="52" t="inlineStr">
-        <is>
-          <t>⚠️ PARTIAL</t>
+      <c r="F26" s="50" t="inlineStr">
+        <is>
+          <t>🔄 REAL DATA DWT TERPASANG</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Grid GFS asli tidak di knowledge base; DWT angin bisa jadi pengganti skala kecamatan</t>
+          <t>initDwtWindStations(): 1234 kecamatan DWT → IDW 3-titik di getGfsWindVectorAt; fallback sintetis bila gagal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement semua item READY — transport live (DWT jalan+kereta, maritim perairan), forecast per titik rute (df/coord), WaveRadarMap live (geojson+overview), advisor maritim live, overlay wilayah perairan di MarineMap; service openData.ts
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -4727,14 +4727,14 @@
           <t>DWT apiDF_Darat: kode_cuaca, hujan, angin per kecamatan per jam UTC</t>
         </is>
       </c>
-      <c r="F18" s="50" t="inlineStr">
-        <is>
-          <t>🔄 READY</t>
+      <c r="F18" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE (DWT kecamatan terdekat)</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Mapping: kode_cuaca 0-1→Aman, 3-7→Waspada, &gt;=10/AWS→Awas + narasi template</t>
+          <t>openData.dwtWeatherAt → status dari kode_cuaca + narasi suhu/kelembapan; fallback mock</t>
         </is>
       </c>
     </row>
@@ -4797,14 +4797,14 @@
           <t>maritim public_api: perairan wave_cat/warning_desc; pelabuhan (pasut, arus)</t>
         </is>
       </c>
-      <c r="F20" s="50" t="inlineStr">
-        <is>
-          <t>🔄 READY</t>
+      <c r="F20" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE (maritim perairan resmi)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Kode wilayah dari nearest-location internal sudah cocok (contoh F.09)</t>
+          <t>nearest-location code → perairan wave_desc/warning_desc → status + narasi; pasut nanti via pelabuhan</t>
         </is>
       </c>
     </row>
@@ -4832,14 +4832,14 @@
           <t>DWT apiDF_Kereta: 178 stasiun per jam UTC</t>
         </is>
       </c>
-      <c r="F21" s="50" t="inlineStr">
-        <is>
-          <t>🔄 READY</t>
+      <c r="F21" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE (DWT kereta)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Perlu slot UI baru kalau mau tampil</t>
+          <t>dwtKeretaAt (178 stasiun, jarak maks 0.5°) → baris Rail baru; di luar Jawa otomatis disembunyikan</t>
         </is>
       </c>
     </row>
@@ -4867,14 +4867,14 @@
           <t>DWT apiDF_Darat: lat/lon kecamatan → match titik rute terdekat</t>
         </is>
       </c>
-      <c r="F22" s="50" t="inlineStr">
-        <is>
-          <t>🔄 READY</t>
+      <c r="F22" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE (df/forecast/coord per titik rute)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Rute &amp; POI tetap Overpass OSM (bukan BMKG)</t>
+          <t>lokasi aktif → bmkg.forecast(lat,lng) internal → 7 hari per titik; fallback peta kota mock</t>
         </is>
       </c>
     </row>
@@ -4972,12 +4972,16 @@
           <t>maritim overview gelombang + perairan wave_cat/wave_desc</t>
         </is>
       </c>
-      <c r="F25" s="50" t="inlineStr">
-        <is>
-          <t>🔄 READY</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr"/>
+      <c r="F25" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE (geojson + overview maritim)</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>232 centroid wilayah (geojson resmi) + wave_cat overview → zone peta; wind mode ilustratif</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -5038,14 +5042,14 @@
           <t>maritim perairan per wilayah (warning_desc, wave_cat)</t>
         </is>
       </c>
-      <c r="F27" s="50" t="inlineStr">
-        <is>
-          <t>🔄 READY</t>
+      <c r="F27" s="49" t="inlineStr">
+        <is>
+          <t>✅ LIVE (parameter gelombang resmi)</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>SOP checklist &amp; kontak memang by-design static</t>
+          <t>maritimLive di-inject: parameter Tinggi Gelombang + riskLevel + advisory utk shipping/fishery</t>
         </is>
       </c>
     </row>
@@ -5104,14 +5108,14 @@
           <t>maritim wilayah_perairan.geojson (polygon 232 wilayah)</t>
         </is>
       </c>
-      <c r="F29" s="50" t="inlineStr">
-        <is>
-          <t>🔄 READY (opsional)</t>
+      <c r="F29" s="49" t="inlineStr">
+        <is>
+          <t>✅ TERPASANG (overlay wilayah perairan)</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Layer polygon resmi per wilayah + kode</t>
+          <t>L.geoJSON wilayah_perairan (232 polygon, CORS *) + popup nama/kode di MarineMap</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(xlsx): sheet 'Audit Card + Screenshot' — 17 kartu + gambar + API/query/sample
Sheet baru (setelah 'Audit Content Card') berisi per komponen:
- screenshot card (dengan border/chip API BOX MARKER: merah=live,
  amber=campuran, abu=mock — terekam otomatis dari deployment prod-sim)
- status LIVE/CAMPURAN/MOCK, daftar API dipakai, query/URL terakhir
  (+status HTTP), potongan sample response (1500 char), catatan per bagian

Infrastruktur regenerasi:
- apiMarker.ts: data-api-box attribute (locator) + window.__apiBox
  {cards, defs, calls, totals} untuk ekstraksi ke dokumentasi
- docs/artifacts/scripts/capture_card_screenshots.js — Playwright, termasuk
  membuka 3 drawer (Darat/Pelayaran/Penerbangan; urutan nth 0/1/3)
- docs/artifacts/scripts/build_card_audit_sheet.py — rakit sheet + embed
  gambar (resize JPEG 720px via Pillow; xlsx tetap ~900KB)
- docs/screenshots/cards/*.png + dump.json (raw hasil capture)
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -9,10 +9,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API Mapping" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Temuan API Resmi" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Content Card" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Official Open Data" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit Card + Screenshot" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Web" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mobile" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Official Open Data" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Mapping'!$A$1:$L$33</definedName>
@@ -24,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="44">
+  <fonts count="50">
     <font>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -336,8 +337,34 @@
       <color rgb="FF1F4E79"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="49">
+  <fills count="53">
     <fill>
       <patternFill/>
     </fill>
@@ -619,8 +646,28 @@
         <fgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -725,6 +772,20 @@
         <color theme="4"/>
       </bottom>
       <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D5DD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D5DD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D5DD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D5DD"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="49">
@@ -874,7 +935,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -980,6 +1041,32 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="49" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="50" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="51" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="52" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1103,6 +1190,436 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>4</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="4543425"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="2438400"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>6</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="4381500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>7</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="390525"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>8</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="6572250"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="8020050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="3390900"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="3933825"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="3067050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="9" name="Image 9" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="26165175"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="10" name="Image 10" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="5695950"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="11" name="Image 11" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="5553075"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="12" name="Image 12" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="2362200"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="5238750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="5238750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="5238750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>2</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6858000" cy="781050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4760,7 +5277,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="47" t="inlineStr">
         <is>
@@ -5709,6 +6225,889 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="110" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="54" t="inlineStr">
+        <is>
+          <t>AUDIT CONTENT CARD + SCREENSHOT — komponen, API yang dipakai, query, sample response</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="55" t="inlineStr">
+        <is>
+          <t>Screenshot diambil dari deployment prod (server.mjs + dist, data live) dengan API BOX MARKER aktif — border merah = live, amber = campuran, abu = mock (lihat kolom Status). Sumber screenshot: docs/screenshots/cards/ · skrip: docs/artifacts/scripts/capture_card_screenshots.js</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="56" t="inlineStr">
+        <is>
+          <t>Status: ✅ LIVE = nilai kartu dari API live  |  ⚠️ CAMPURAN = sebagian live/sebagian mock  |  🔌 MOCK = statis/estimasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="57" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="57" t="inlineStr">
+        <is>
+          <t>Komponen</t>
+        </is>
+      </c>
+      <c r="C4" s="57" t="inlineStr">
+        <is>
+          <t>Screenshot</t>
+        </is>
+      </c>
+      <c r="D4" s="57" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E4" s="57" t="inlineStr">
+        <is>
+          <t>API dipakai</t>
+        </is>
+      </c>
+      <c r="F4" s="57" t="inlineStr">
+        <is>
+          <t>Query / URL terakhir</t>
+        </is>
+      </c>
+      <c r="G4" s="57" t="inlineStr">
+        <is>
+          <t>Sample Response (potongan)</t>
+        </is>
+      </c>
+      <c r="H4" s="57" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="365.75" customHeight="1">
+      <c r="A5" s="58" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="59" t="inlineStr">
+        <is>
+          <t>Hero Weather Card — Cuaca Hari Ini
+(hero)</t>
+        </is>
+      </c>
+      <c r="C5" s="60" t="n"/>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="E5" s="59" t="inlineStr">
+        <is>
+          <t>• DF Forecast: prakiraan 10 hari + per jam
+• Present Weather: cuaca saat ini</t>
+        </is>
+      </c>
+      <c r="F5" s="62" t="inlineStr">
+        <is>
+          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-6.2804&amp;lon=106.9507
+[200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666</t>
+        </is>
+      </c>
+      <c r="G5" s="62" t="inlineStr">
+        <is>
+          <t>{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.94655786745837,"lat":-6.277639992667722,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.9465578675,"lat":-6.2776399927,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T06:00:00Z","t":34,"tcc":93,"tp":0,"weather":3,"weather_desc":"Berawan","weather_desc_en":"Mostly Cloudy","wd_deg":306,"wd":"W","wd_to":"E","ws":11.5,"hu":48,"vs":null,"vs_text":null,"time_index":"5-6","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan-am.svg","utc_datetime":"2026-09-22 06:00:00","local_datetime":"2026-09-22 13:00:00"},{"datetime":"2026-09-22T07:00:00Z","t":33,"tcc":50,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":290,"wd":"W","wd_to":"E","ws":14,"hu":48,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":30,"tcc":82,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":290,"wd":"W","wd_to":"E",
+… (dipotong)</t>
+        </is>
+      </c>
+      <c r="H5" s="63" t="inlineStr">
+        <is>
+          <t>Kartu 'Hari Ini' = kondisi live saat ini; strip 7 hari = slot pertama tiap grup (df-forecast). API tidak punya tmin/tmax &amp; probabilitas hujan → keduanya di-skip (badge % = tp×20, aproksimasi).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="200" customHeight="1">
+      <c r="A6" s="58" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="59" t="inlineStr">
+        <is>
+          <t>Kondisi Saat Ini (rincian)
+(current-weather)</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="n"/>
+      <c r="D6" s="61" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="E6" s="59" t="inlineStr">
+        <is>
+          <t>• DF Forecast: prakiraan 10 hari + per jam
+• DF Adm: resolve wilayah admin
+• Present Weather: cuaca saat ini
+• API v1: waktu matahari terbit/terbenam</t>
+        </is>
+      </c>
+      <c r="F6" s="62" t="inlineStr">
+        <is>
+          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-6.2804&amp;lon=106.9507
+[200] /api-bmkgapi/df/v1/adm/coord&amp;lat=-6.2&amp;lon=106.816666
+[200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666
+[200] https://cuaca.bmkg.go.id/api/v1/sunset/json?lat=-6.2&amp;lng=106.816666</t>
+        </is>
+      </c>
+      <c r="G6" s="62" t="inlineStr">
+        <is>
+          <t>{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.94655786745837,"lat":-6.277639992667722,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.9465578675,"lat":-6.2776399927,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T06:00:00Z","t":34,"tcc":93,"tp":0,"weather":3,"weather_desc":"Berawan","weather_desc_en":"Mostly Cloudy","wd_deg":306,"wd":"W","wd_to":"E","ws":11.5,"hu":48,"vs":null,"vs_text":null,"time_index":"5-6","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan-am.svg","utc_datetime":"2026-09-22 06:00:00","local_datetime":"2026-09-22 13:00:00"},{"datetime":"2026-09-22T07:00:00Z","t":33,"tcc":50,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":290,"wd":"W","wd_to":"E","ws":14,"hu":48,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":30,"tcc":82,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":290,"wd":"W","wd_to":"E",
+… (dipotong)</t>
+        </is>
+      </c>
+      <c r="H6" s="63" t="inlineStr">
+        <is>
+          <t>Info matahari (sunset API), wilayah (df/adm).
+– UV: proksi tcc (bukan UV asli) (est)
+– "Terasa seperti": rumus t + (hu-50)/10 (est)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="353" customHeight="1">
+      <c r="A7" s="58" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="59" t="inlineStr">
+        <is>
+          <t>Panel Prakiraan (Per Jam / Mingguan)
+(forecast-panel)</t>
+        </is>
+      </c>
+      <c r="C7" s="60" t="n"/>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="E7" s="59" t="inlineStr">
+        <is>
+          <t>• DF Forecast: prakiraan 10 hari + per jam
+• Open Data RESMI: prakiraan-cuaca (adm4)</t>
+        </is>
+      </c>
+      <c r="F7" s="62" t="inlineStr">
+        <is>
+          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-6.2804&amp;lon=106.9507
+(belum terekam saat capture) — Open Data RESMI: prakiraan-cuaca (adm4)</t>
+        </is>
+      </c>
+      <c r="G7" s="62" t="inlineStr">
+        <is>
+          <t>{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.94655786745837,"lat":-6.277639992667722,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.9465578675,"lat":-6.2776399927,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T06:00:00Z","t":34,"tcc":93,"tp":0,"weather":3,"weather_desc":"Berawan","weather_desc_en":"Mostly Cloudy","wd_deg":306,"wd":"W","wd_to":"E","ws":11.5,"hu":48,"vs":null,"vs_text":null,"time_index":"5-6","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan-am.svg","utc_datetime":"2026-09-22 06:00:00","local_datetime":"2026-09-22 13:00:00"},{"datetime":"2026-09-22T07:00:00Z","t":33,"tcc":50,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":290,"wd":"W","wd_to":"E","ws":14,"hu":48,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":30,"tcc":82,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":290,"wd":"W","wd_to":"E",
+… (dipotong)</t>
+        </is>
+      </c>
+      <c r="H7" s="63" t="inlineStr">
+        <is>
+          <t>Tab Suhu = satu suhu per hari (slot pertama, tanpa min/max). Fallback resmi open-data bila df kosong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="120" customHeight="1">
+      <c r="A8" s="58" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="59" t="inlineStr">
+        <is>
+          <t>Peringatan Dini (Alerts)
+(alerts)</t>
+        </is>
+      </c>
+      <c r="C8" s="60" t="n"/>
+      <c r="D8" s="61" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="E8" s="59" t="inlineStr">
+        <is>
+          <t>• Public API: peringatan cuaca
+• Public API: peringatan siklon
+• Peringatan Dini Nowcast (RSS resmi)</t>
+        </is>
+      </c>
+      <c r="F8" s="62" t="inlineStr">
+        <is>
+          <t>[200] /api-bmkgapi/public/weather/warning&amp;lat=-6.2&amp;long=106.816666
+(belum terekam saat capture) — Public API: peringatan siklon
+(belum terekam saat capture) — Peringatan Dini Nowcast (RSS resmi)</t>
+        </is>
+      </c>
+      <c r="G8" s="62" t="inlineStr">
+        <is>
+          <t>{"statusCode":200,"message":"OK!","data":{"today":{},"tomorrow":null}}</t>
+        </is>
+      </c>
+      <c r="H8" s="63" t="inlineStr">
+        <is>
+          <t>Nowcast (resmi, per provinsi) menang atas warning internal. Cyclone terdampak jarang (hanya saat ada siklon).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="525.5" customHeight="1">
+      <c r="A9" s="58" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="59" t="inlineStr">
+        <is>
+          <t>Berita &amp; Video (News Section)
+(news)</t>
+        </is>
+      </c>
+      <c r="C9" s="60" t="n"/>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="E9" s="59" t="inlineStr">
+        <is>
+          <t>• Berita WordPress BMKG (WP REST)
+• Public API: video berita</t>
+        </is>
+      </c>
+      <c r="F9" s="62" t="inlineStr">
+        <is>
+          <t>(belum terekam saat capture) — Berita WordPress BMKG (WP REST)
+[200] /api-bmkgapi/public/weather/video-latest&amp;hashtag=infobmkgpws</t>
+        </is>
+      </c>
+      <c r="G9" s="62" t="inlineStr">
+        <is>
+          <t>[{"title":"Prakiraan Cuaca Esok Hari, Selasa, 22 September 2026.","videoUrl":"https://www.youtube.com/watch?v=l6NWtkthnzU"},{"title":"Prakiraan Cuaca Esok Hari,  Senin, 21 September 2026.","videoUrl":"https://www.youtube.com/watch?v=GNIhEbJS8q4"},{"title":"Prakiraan Cuaca Esok Hari, Minggu, 20 September 2026","videoUrl":"https://www.youtube.com/watch?v=kCepZRm8uIQ"},{"title":"Prakiraan Cuaca Esok Hari, Sabtu, 19 September 2026.","videoUrl":"https://www.youtube.com/watch?v=9egb1zLG0PM"},{"title":"Prakiraan Cuaca Esok Hari, Jumat, 18 September 2026.","videoUrl":"https://www.youtube.com/watch?v=1Dy6sPbtzpc"},{"title":"Prakiraan Cuaca Esok Hari Kamis, 17 September 2026","videoUrl":"https://www.youtube.com/watch?v=Xx3Ddki3bHk"}]</t>
+        </is>
+      </c>
+      <c r="H9" s="63" t="inlineStr">
+        <is>
+          <t>– Fallback: artikel mock saat WP 502 (sering) (mock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="639.5" customHeight="1">
+      <c r="A10" s="58" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="59" t="inlineStr">
+        <is>
+          <t>Gempa Bumi (TEWS)
+(earthquake)</t>
+        </is>
+      </c>
+      <c r="C10" s="60" t="n"/>
+      <c r="D10" s="61" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="E10" s="59" t="inlineStr">
+        <is>
+          <t>• Open Data: gempa (TEWS)</t>
+        </is>
+      </c>
+      <c r="F10" s="62" t="inlineStr">
+        <is>
+          <t>(belum terekam saat capture) — Open Data: gempa (TEWS)</t>
+        </is>
+      </c>
+      <c r="G10" s="62" t="inlineStr">
+        <is>
+          <t>— (tidak ada response live)</t>
+        </is>
+      </c>
+      <c r="H10" s="63" t="inlineStr">
+        <is>
+          <t>autogempa + gempadirasakan, 2 endpoint TEWS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="275" customHeight="1">
+      <c r="A11" s="58" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="59" t="inlineStr">
+        <is>
+          <t>Citra Satelit Himawari-9
+(satellite)</t>
+        </is>
+      </c>
+      <c r="C11" s="60" t="n"/>
+      <c r="D11" s="61" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="E11" s="59" t="inlineStr">
+        <is>
+          <t>• Citra Satelit Himawari-9 (background-image, bukan fetch)</t>
+        </is>
+      </c>
+      <c r="F11" s="62" t="inlineStr">
+        <is>
+          <t>(belum terekam saat capture) — Citra Satelit Himawari-9 (background-image, bukan fetch)</t>
+        </is>
+      </c>
+      <c r="G11" s="62" t="inlineStr">
+        <is>
+          <t>— (tidak ada response live)</t>
+        </is>
+      </c>
+      <c r="H11" s="63" t="inlineStr">
+        <is>
+          <t>Gambar PNG inderaja.bmkg.go.id (background-image &lt;img&gt; → TIDAK terekam patch fetch).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="317.75" customHeight="1">
+      <c r="A12" s="58" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="59" t="inlineStr">
+        <is>
+          <t>Carousel Kota Besar (statis)
+(major-cities)</t>
+        </is>
+      </c>
+      <c r="C12" s="60" t="n"/>
+      <c r="D12" s="64" t="inlineStr">
+        <is>
+          <t>🔌 MOCK</t>
+        </is>
+      </c>
+      <c r="E12" s="59" t="inlineStr">
+        <is>
+          <t>— (tanpa API live)</t>
+        </is>
+      </c>
+      <c r="F12" s="62" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="62" t="inlineStr">
+        <is>
+          <t>— (tidak ada response live)</t>
+        </is>
+      </c>
+      <c r="H12" s="63" t="inlineStr">
+        <is>
+          <t>– Kartu statis: landmark + nama kota (auto-geser &amp; fetch sengaja dimatikan, 16 Sep) (mock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="249.5" customHeight="1">
+      <c r="A13" s="58" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="59" t="inlineStr">
+        <is>
+          <t>Transportasi (Jalan / Kereta / Maritim)
+(transport)</t>
+        </is>
+      </c>
+      <c r="C13" s="60" t="n"/>
+      <c r="D13" s="65" t="inlineStr">
+        <is>
+          <t>⚠️ CAMPURAN</t>
+        </is>
+      </c>
+      <c r="E13" s="59" t="inlineStr">
+        <is>
+          <t>• DWT: cuaca kecamatan/stasiun (jalan+kereta)
+• ISDP v1: wilayah laut terdekat
+• Maritim: detail cuaca/gelombang perairan</t>
+        </is>
+      </c>
+      <c r="F13" s="62" t="inlineStr">
+        <is>
+          <t>[200] /event/source/dwt/apiDF_Kereta/manifest_times.json
+[200] /api-bmkgapi/v1/public/maritim/nearest-location&amp;lat=-6.2&amp;long=106.816666
+[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+        </is>
+      </c>
+      <c r="G13" s="62" t="inlineStr">
+        <is>
+          <t>&lt;!doctype html&gt;
+&lt;html lang="id" class="dark"&gt;
+  &lt;head&gt;
+    &lt;meta charset="UTF-8" /&gt;
+    &lt;link rel="icon" type="image/svg+xml" href="/assets/logo-BenySzP1.svg" /&gt;
+    &lt;!-- Preconnect to Google Fonts to fetch fonts faster and prevent Flash of Unstyled Text (FOUT) --&gt;
+    &lt;link rel="preconnect" href="https://fonts.googleapis.com" /&gt;
+    &lt;link rel="preconnect" href="https://fonts.gstatic.com" crossorigin /&gt;
+    &lt;link href="https://fonts.googleapis.com/css2?family=Plus+Jakarta+Sans:wght@300;400;500;600;700;800&amp;display=swap" rel="stylesheet" /&gt;
+    &lt;meta name="viewport" content="width=device-width, initial-scale=1.0, viewport-fit=cover" /&gt;
+    &lt;meta name="color-scheme" content="dark" /&gt;
+    &lt;meta name="theme-color" content="#070c19" /&gt;
+    &lt;meta name="apple-mobile-web-app-capable" content="yes" /&gt;
+    &lt;meta name="apple-mobile-web-app-status-bar-style" content="black-translucent" /&gt;
+    &lt;meta name="description" content="Portal Redesign Digital Weather Info BMKG - Layanan Informasi Cuaca Publik, Penerbangan, Maritim, Peringatan Dini Angin &amp; Hujan, dan Satelit Cuaca Himawari-9." /&gt;
+    &lt;meta name="keywords" content="BMKG, Info BMKG, Cuaca Indonesia, Radar Cuaca, Satelit Himawari-9, Gempa Megathrust, Peringatan Dini" /&gt;
+    &lt;meta name="author" content="BMKG Indonesia" /&gt;
+    &lt;title&gt;BMKG | Portal Informasi Cuaca, Iklim &amp; Geofisika Indonesia&lt;/title&gt;
+    &lt;script&gt;
+      (function() {
+        try {
+          const theme = localStorage.getItem('bmkg-theme-v2');
+          const isDark =
+… (dipotong)</t>
+        </is>
+      </c>
+      <c r="H13" s="63" t="inlineStr">
+        <is>
+          <t>– Jalan Raya: DWT kecamatan terdekat (live)
+– Kereta: DWT stasiun terdekat (178 stasiun) (live)
+– Maritim: perairan resmi (fix currentSlot 15 Sep) (live)
+– Penerbangan: MOCK/PAUSED (menunggu data partner) (mock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="2068.25" customHeight="1">
+      <c r="A14" s="58" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="59" t="inlineStr">
+        <is>
+          <t>Panduan Aktivitas &amp; Analisis Cuaca
+(weather-activity)</t>
+        </is>
+      </c>
+      <c r="C14" s="60" t="n"/>
+      <c r="D14" s="65" t="inlineStr">
+        <is>
+          <t>⚠️ CAMPURAN</t>
+        </is>
+      </c>
+      <c r="E14" s="59" t="inlineStr">
+        <is>
+          <t>• DF Forecast: prakiraan 10 hari + per jam
+• ISDP v1: wilayah laut terdekat
+• Maritim: detail cuaca/gelombang perairan</t>
+        </is>
+      </c>
+      <c r="F14" s="62" t="inlineStr">
+        <is>
+          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-6.2804&amp;lon=106.9507
+[200] /api-bmkgapi/v1/public/maritim/nearest-location&amp;lat=-6.2&amp;long=106.816666
+[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+        </is>
+      </c>
+      <c r="G14" s="62" t="inlineStr">
+        <is>
+          <t>{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.94655786745837,"lat":-6.277639992667722,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.9465578675,"lat":-6.2776399927,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T06:00:00Z","t":34,"tcc":93,"tp":0,"weather":3,"weather_desc":"Berawan","weather_desc_en":"Mostly Cloudy","wd_deg":306,"wd":"W","wd_to":"E","ws":11.5,"hu":48,"vs":null,"vs_text":null,"time_index":"5-6","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan-am.svg","utc_datetime":"2026-09-22 06:00:00","local_datetime":"2026-09-22 13:00:00"},{"datetime":"2026-09-22T07:00:00Z","t":33,"tcc":50,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":290,"wd":"W","wd_to":"E","ws":14,"hu":48,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":30,"tcc":82,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":290,"wd":"W","wd_to":"E",
+… (dipotong)</t>
+        </is>
+      </c>
+      <c r="H14" s="63" t="inlineStr">
+        <is>
+          <t>– Aktivitas umum: forecast live (live)
+– Aktivitas pelayaran: gelombang perairan resmi (live)
+– ISPU/AQI: ESTIMASI sintetis (tidak ada sumber resmi) (est)
+– Indeks kenyamanan: label statis (mock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="456.5" customHeight="1">
+      <c r="A15" s="58" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="59" t="inlineStr">
+        <is>
+          <t>Peta Laut (Marine Map)
+(marine-map)</t>
+        </is>
+      </c>
+      <c r="C15" s="60" t="n"/>
+      <c r="D15" s="65" t="inlineStr">
+        <is>
+          <t>⚠️ CAMPURAN</t>
+        </is>
+      </c>
+      <c r="E15" s="59" t="inlineStr">
+        <is>
+          <t>• Maritim: overview tinggi gelombang (232 wilayah)
+• Maritim: polygon 232 wilayah perairan
+• Maritim: detail cuaca/gelombang perairan
+• DWT: cuaca kecamatan/stasiun (jalan+kereta)</t>
+        </is>
+      </c>
+      <c r="F15" s="62" t="inlineStr">
+        <is>
+          <t>(belum terekam saat capture) — Maritim: overview tinggi gelombang (232 wilayah)
+(belum terekam saat capture) — Maritim: polygon 232 wilayah perairan
+[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json
+[200] /event/source/dwt/apiDF_Kereta/manifest_times.json</t>
+        </is>
+      </c>
+      <c r="G15" s="62" t="inlineStr">
+        <is>
+          <t>{"code": "F.09", "name": "Teluk Jakarta", "issued": "2026-09-21 23:39 UTC", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "data": [{"valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "time_desc": "Hari ini", "weather": "Berawan", "weather_desc": "Hari ini untuk Teluk Jakarta diperkirakan berawan, dengan kecepatan angin pada umumnya 5 - 18 knot bertiup dari arah selatan, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": "Rendah", "wave_desc": "0.5 - 1.25 m", "wind_from": "Selatan", "wind_to": "Barat Daya", "wind_speed_min": 5, "wind_speed_max": 18}, {"valid_from": "2026-09-22 00:00 UTC", "valid_to": "2026-09-22 12:00 UTC", "time_desc": "Besok", "weather": "Hujan Ringan", "weather_desc": "Besok untuk Teluk Jakarta diperkirakan hujan ringan, dengan kecepatan angin pada umumnya 11 - 33 knot bertiup dari arah utara, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": "Rendah", "wave_desc": "0.5 - 1.25 m", "wind_from": "Utara", "wind_to": "Barat Daya", "wind_speed_min": 11, "wind_speed_max": 33}, {"valid_from": "2026-09-22 12:00 UTC", "valid_to": "2026-09-23 12:00 UTC", "time_desc": "H+2", "weather": "Hujan Ringan", "weather_desc": "Lusa untuk Teluk Jakarta diperkirakan hujan ringan, dengan kecepatan angin pada umumn
+… (dipotong)</t>
+        </is>
+      </c>
+      <c r="H15" s="63" t="inlineStr">
+        <is>
+          <t>– Gelombang: 232 wilayah resmi (warna/legend live), klik → detail live (live)
+– Layer angin/cuaca: SNAPSHOT statis (sectors.json) (mock)
+– Mode Pelabuhan: snapshot ports.json (294) — hanya pelabuhan TERDEKAT yang live (mock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="445.25" customHeight="1">
+      <c r="A16" s="58" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="59" t="inlineStr">
+        <is>
+          <t>Pelabuhan &amp; Pasut
+(port-tide)</t>
+        </is>
+      </c>
+      <c r="C16" s="60" t="n"/>
+      <c r="D16" s="61" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="E16" s="59" t="inlineStr">
+        <is>
+          <t>• Maritim: daftar pelabuhan (294)
+• Maritim: detail pelabuhan + pasut</t>
+        </is>
+      </c>
+      <c r="F16" s="62" t="inlineStr">
+        <is>
+          <t>[200] https://maritim.bmkg.go.id/public_api/pelabuhan_list
+[200] https://maritim.bmkg.go.id/public_api/pelabuhan/0101_Sunda%20Kelapa.json</t>
+        </is>
+      </c>
+      <c r="G16" s="62" t="inlineStr">
+        <is>
+          <t>{
+  "files": [
+    {
+      "coor": [
+        1.198331,
+        109.054462
+      ],
+      "file_date": "2026-09-21 23:47 UTC",
+      "kb": 1720,
+      "name": "0088_Sintete.json",
+      "portname": "Sintete",
+      "type": "utama"
+    },
+    {
+      "coor": [
+        0.00214,
+        109.285391
+      ],
+      "file_date": "2026-09-21 23:47 UTC",
+      "kb": 1713,
+      "name": "0310_PPP Sungai Rengas.json",
+      "portname": "PPP Sungai Rengas",
+      "type": "utama"
+    },
+    {
+      "coor": [
+        -2.531535,
+        110.21588
+      ],
+      "file_date": "2026-09-21 23:47 UTC",
+      "kb": 1692,
+      "name": "0092_Kendawangan.json",
+      "portname": "Kendawangan",
+      "type": "utama"
+    },
+    {
+      "coor": [
+        4.145037,
+        117.665883
+      ],
+      "file_date": "2026-09-21 23:47 UTC",
+      "kb": 1679,
+      "name": "0237_Nunukan.json",
+      "portname": "Nunukan",
+      "type": "utama"
+    },
+    {
+      "coor": [
+        -8.6679806,
+        115.261925
+      ],
+      "file_date": "2026-09-21 23:47 UTC",
+      "kb": 1646,
+      "name": "0603_Sanur.json",
+      "portname": "Sanur",
+      "type": "utama"
+    },
+    {
+      "coor": [
+        -5.35863269,
+        105.81975796
+      ],
+      "file_date": "2026-09-21 23:47 UTC",
+      "kb": 1670,
+      "name": "0325_PPP Labuhan Maringgai.json",
+      "portname": "PPP Labuhan Maringgai",
+      "type": "utama"
+    },
+    {
+      "coor": [
+        -8.67206,
+        115.55675
+      ],
+      "file_date": "2026-09-
+… (dipotong)</t>
+        </is>
+      </c>
+      <c r="H16" s="63" t="inlineStr">
+        <is>
+          <t>Pasut null di sebagian pelabuhan → blok disembunyikan. Kolom arus di-skip (satuan ambigu).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="194" customHeight="1">
+      <c r="A17" s="58" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="59" t="inlineStr">
+        <is>
+          <t>Aktivitas Sekitar (POI)
+(around-activity)</t>
+        </is>
+      </c>
+      <c r="C17" s="60" t="n"/>
+      <c r="D17" s="65" t="inlineStr">
+        <is>
+          <t>⚠️ CAMPURAN</t>
+        </is>
+      </c>
+      <c r="E17" s="59" t="inlineStr">
+        <is>
+          <t>• DF Forecast: prakiraan 10 hari + per jam
+• Overpass API: POI OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="F17" s="62" t="inlineStr">
+        <is>
+          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-6.2804&amp;lon=106.9507
+(belum terekam saat capture) — Overpass API: POI OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="G17" s="62" t="inlineStr">
+        <is>
+          <t>{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.94655786745837,"lat":-6.277639992667722,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.9465578675,"lat":-6.2776399927,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T06:00:00Z","t":34,"tcc":93,"tp":0,"weather":3,"weather_desc":"Berawan","weather_desc_en":"Mostly Cloudy","wd_deg":306,"wd":"W","wd_to":"E","ws":11.5,"hu":48,"vs":null,"vs_text":null,"time_index":"5-6","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan-am.svg","utc_datetime":"2026-09-22 06:00:00","local_datetime":"2026-09-22 13:00:00"},{"datetime":"2026-09-22T07:00:00Z","t":33,"tcc":50,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":290,"wd":"W","wd_to":"E","ws":14,"hu":48,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":30,"tcc":82,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":290,"wd":"W","wd_to":"E",
+… (dipotong)</t>
+        </is>
+      </c>
+      <c r="H17" s="63" t="inlineStr">
+        <is>
+          <t>Nilai cuaca per titik POI live (1 request df/coord per POI).
+– Daftar POI: kurasi statis (cityLandmarks) (mock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="420.5" customHeight="1">
+      <c r="A18" s="58" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="59" t="inlineStr">
+        <is>
+          <t>Aktivitas Darat (Drawer)
+(land-based)</t>
+        </is>
+      </c>
+      <c r="C18" s="60" t="n"/>
+      <c r="D18" s="65" t="inlineStr">
+        <is>
+          <t>⚠️ CAMPURAN</t>
+        </is>
+      </c>
+      <c r="E18" s="59" t="inlineStr">
+        <is>
+          <t>• DF Forecast: prakiraan 10 hari + per jam
+• DWT: cuaca kecamatan/stasiun (jalan+kereta)
+• Overpass API: POI OpenStreetMap
+• Nominatim: geocode OSM
+• OSRM: routing</t>
+        </is>
+      </c>
+      <c r="F18" s="62" t="inlineStr">
+        <is>
+          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-6.2804&amp;lon=106.9507
+[200] /event/source/dwt/apiDF_Kereta/manifest_times.json
+(belum terekam saat capture) — Overpass API: POI OpenStreetMap
+(belum terekam saat capture) — Nominatim: geocode OSM
+(belum terekam saat capture) — OSRM: routing</t>
+        </is>
+      </c>
+      <c r="G18" s="62" t="inlineStr">
+        <is>
+          <t>{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.94655786745837,"lat":-6.277639992667722,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.9465578675,"lat":-6.2776399927,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T06:00:00Z","t":34,"tcc":93,"tp":0,"weather":3,"weather_desc":"Berawan","weather_desc_en":"Mostly Cloudy","wd_deg":306,"wd":"W","wd_to":"E","ws":11.5,"hu":48,"vs":null,"vs_text":null,"time_index":"5-6","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan-am.svg","utc_datetime":"2026-09-22 06:00:00","local_datetime":"2026-09-22 13:00:00"},{"datetime":"2026-09-22T07:00:00Z","t":33,"tcc":50,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":290,"wd":"W","wd_to":"E","ws":14,"hu":48,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":30,"tcc":82,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":290,"wd":"W","wd_to":"E",
+… (dipotong)</t>
+        </is>
+      </c>
+      <c r="H18" s="63" t="inlineStr">
+        <is>
+          <t>Forecast per titik rute live; fallback mock saat API gagal.
+– Pilihan lokasi awal: daftar statis (mock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="420.5" customHeight="1">
+      <c r="A19" s="58" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="59" t="inlineStr">
+        <is>
+          <t>Konsultasi Pelayaran (Drawer)
+(maritime-advisor)</t>
+        </is>
+      </c>
+      <c r="C19" s="60" t="n"/>
+      <c r="D19" s="65" t="inlineStr">
+        <is>
+          <t>⚠️ CAMPURAN</t>
+        </is>
+      </c>
+      <c r="E19" s="59" t="inlineStr">
+        <is>
+          <t>• ISDP v1: wilayah laut terdekat
+• Maritim: detail cuaca/gelombang perairan</t>
+        </is>
+      </c>
+      <c r="F19" s="62" t="inlineStr">
+        <is>
+          <t>[200] /api-bmkgapi/v1/public/maritim/nearest-location&amp;lat=-6.2&amp;long=106.816666
+[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+        </is>
+      </c>
+      <c r="G19" s="62" t="inlineStr">
+        <is>
+          <t>{"statusCode":200,"message":"OK!","data":{"code":"F.09","name":"Teluk Jakarta","wilpel":"Stamar Tanjung Priok - Jakarta","geometry":{"type":"Polygon","coordinates":[[[106.68448229697637,-6.015114864033774],[106.68448229697637,-5.910111585789263],[107.03498697202032,-5.910111585789263],[106.99055680194432,-5.931987268756869],[107.01030354420033,-5.940737541943912],[107.02017691532832,-5.960425656614758],[107.01030354420033,-5.984488907879126],[106.98562011638033,-6.004177022549971],[106.99055680194432,-6.023865137220817],[107.02017691532832,-6.03480297870462],[107.02017691532832,-6.078554344639833],[106.99055680194432,-6.087304617826876],[106.91156983292034,-6.100430027607439],[106.87701303397235,-6.098242459310679],[106.85726629171634,-6.117930573981525],[106.82270949276835,-6.124493278871807],[106.79308937938436,-6.111367869091243],[106.74372252374437,-6.106992732497721],[106.72397578148836,-6.093867322717157],[106.70422903923236,-6.052303525078705],[106.71903909592436,-6.041365683594902],[106.68448229697637,-6.015114864033774]]]},"distance":0.07574819298420225,"coordinate":{"type":"Point","coordinates":[106.83985076208779,-6.019490000627295]},"type":"area"}}</t>
+        </is>
+      </c>
+      <c r="H19" s="63" t="inlineStr">
+        <is>
+          <t>Parameter gelombang resmi di-inject ke drawer.
+– Sisa konten drawer (jenis aktivitas, tabel): statis maritimeAdvisorData.ts (mock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="420.5" customHeight="1">
+      <c r="A20" s="58" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="59" t="inlineStr">
+        <is>
+          <t>Konsultasi Penerbangan (Drawer)
+(aviation-advisor)</t>
+        </is>
+      </c>
+      <c r="C20" s="60" t="n"/>
+      <c r="D20" s="64" t="inlineStr">
+        <is>
+          <t>🔌 MOCK</t>
+        </is>
+      </c>
+      <c r="E20" s="59" t="inlineStr">
+        <is>
+          <t>— (tanpa API live)</t>
+        </is>
+      </c>
+      <c r="F20" s="62" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G20" s="62" t="inlineStr">
+        <is>
+          <t>— (tidak ada response live)</t>
+        </is>
+      </c>
+      <c r="H20" s="63" t="inlineStr">
+        <is>
+          <t>– 100% statis (aviationAdvisorData.ts) — API penerbangan belum ada (mock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="120" customHeight="1">
+      <c r="A21" s="58" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="59" t="inlineStr">
+        <is>
+          <t>Pencarian Lokasi
+(location-search)</t>
+        </is>
+      </c>
+      <c r="C21" s="60" t="n"/>
+      <c r="D21" s="64" t="inlineStr">
+        <is>
+          <t>🔌 MOCK</t>
+        </is>
+      </c>
+      <c r="E21" s="59" t="inlineStr">
+        <is>
+          <t>— (tanpa API live)</t>
+        </is>
+      </c>
+      <c r="F21" s="62" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="62" t="inlineStr">
+        <is>
+          <t>— (tidak ada response live)</t>
+        </is>
+      </c>
+      <c r="H21" s="63" t="inlineStr">
+        <is>
+          <t>– POI statis (poiSearchData.ts) (mock)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
@@ -5896,7 +7295,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14241,7 +15640,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14461,7 +15860,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
style(xlsx): sheet audit card — gambar lebih kecil, kolom sample dipanjangkan
- gambar 720px -> 460px (kolom C 110 -> 70) — baris lebih pendek, mudah discan
- kolom Sample Response 60 -> 115 char — teks JSON lebih terbaca
- tinggi baris mengikuti konten terpanjang (gambar vs estimasi teks sample),
  dikunci di batas Excel 409,5pt
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -1201,7 +1201,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="4543425"/>
+    <ext cx="4381500" cy="2905125"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -1226,7 +1226,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="2438400"/>
+    <ext cx="4381500" cy="1552575"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -1251,7 +1251,7 @@
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="4381500"/>
+    <ext cx="4381500" cy="2800350"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -1276,7 +1276,7 @@
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="390525"/>
+    <ext cx="4381500" cy="247650"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -1301,7 +1301,7 @@
       <row>8</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="6572250"/>
+    <ext cx="4381500" cy="4200525"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -1326,7 +1326,7 @@
       <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="8020050"/>
+    <ext cx="4381500" cy="5124450"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -1351,7 +1351,7 @@
       <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="3390900"/>
+    <ext cx="4381500" cy="2162175"/>
     <pic>
       <nvPicPr>
         <cNvPr id="7" name="Image 7" descr="Picture"/>
@@ -1376,7 +1376,7 @@
       <row>11</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="3933825"/>
+    <ext cx="4381500" cy="2514600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="8" name="Image 8" descr="Picture"/>
@@ -1401,7 +1401,7 @@
       <row>12</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="3067050"/>
+    <ext cx="4381500" cy="1962150"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -1426,7 +1426,7 @@
       <row>13</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="26165175"/>
+    <ext cx="4381500" cy="16716375"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -1451,7 +1451,7 @@
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="5695950"/>
+    <ext cx="4381500" cy="3638550"/>
     <pic>
       <nvPicPr>
         <cNvPr id="11" name="Image 11" descr="Picture"/>
@@ -1476,7 +1476,7 @@
       <row>15</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="5553075"/>
+    <ext cx="4381500" cy="3552825"/>
     <pic>
       <nvPicPr>
         <cNvPr id="12" name="Image 12" descr="Picture"/>
@@ -1501,7 +1501,7 @@
       <row>16</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="2362200"/>
+    <ext cx="4381500" cy="1504950"/>
     <pic>
       <nvPicPr>
         <cNvPr id="13" name="Image 13" descr="Picture"/>
@@ -1526,7 +1526,7 @@
       <row>17</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="5238750"/>
+    <ext cx="4381500" cy="3343275"/>
     <pic>
       <nvPicPr>
         <cNvPr id="14" name="Image 14" descr="Picture"/>
@@ -1551,7 +1551,7 @@
       <row>18</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="5238750"/>
+    <ext cx="4381500" cy="3343275"/>
     <pic>
       <nvPicPr>
         <cNvPr id="15" name="Image 15" descr="Picture"/>
@@ -1576,7 +1576,7 @@
       <row>19</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="5238750"/>
+    <ext cx="4381500" cy="3343275"/>
     <pic>
       <nvPicPr>
         <cNvPr id="16" name="Image 16" descr="Picture"/>
@@ -1601,7 +1601,7 @@
       <row>20</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6858000" cy="781050"/>
+    <ext cx="4381500" cy="504825"/>
     <pic>
       <nvPicPr>
         <cNvPr id="17" name="Image 17" descr="Picture"/>
@@ -6230,11 +6230,11 @@
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="110" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="115" customWidth="1" min="7" max="7"/>
     <col width="44" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -6301,7 +6301,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="365.75" customHeight="1">
+    <row r="5" ht="236.75" customHeight="1">
       <c r="A5" s="58" t="n">
         <v>1</v>
       </c>
@@ -6341,7 +6341,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="200" customHeight="1">
+    <row r="6" ht="163.5" customHeight="1">
       <c r="A6" s="58" t="n">
         <v>2</v>
       </c>
@@ -6387,7 +6387,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="353" customHeight="1">
+    <row r="7" ht="228.5" customHeight="1">
       <c r="A7" s="58" t="n">
         <v>3</v>
       </c>
@@ -6427,7 +6427,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="120" customHeight="1">
+    <row r="8" ht="90" customHeight="1">
       <c r="A8" s="58" t="n">
         <v>4</v>
       </c>
@@ -6468,7 +6468,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="525.5" customHeight="1">
+    <row r="9" ht="338.75" customHeight="1">
       <c r="A9" s="58" t="n">
         <v>5</v>
       </c>
@@ -6507,7 +6507,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="639.5" customHeight="1">
+    <row r="10" ht="409" customHeight="1">
       <c r="A10" s="58" t="n">
         <v>6</v>
       </c>
@@ -6544,7 +6544,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="275" customHeight="1">
+    <row r="11" ht="178.25" customHeight="1">
       <c r="A11" s="58" t="n">
         <v>7</v>
       </c>
@@ -6581,7 +6581,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="317.75" customHeight="1">
+    <row r="12" ht="206" customHeight="1">
       <c r="A12" s="58" t="n">
         <v>8</v>
       </c>
@@ -6618,7 +6618,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="249.5" customHeight="1">
+    <row r="13" ht="310.5" customHeight="1">
       <c r="A13" s="58" t="n">
         <v>9</v>
       </c>
@@ -6685,7 +6685,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="2068.25" customHeight="1">
+    <row r="14" ht="409" customHeight="1">
       <c r="A14" s="58" t="n">
         <v>10</v>
       </c>
@@ -6730,7 +6730,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="456.5" customHeight="1">
+    <row r="15" ht="294.5" customHeight="1">
       <c r="A15" s="58" t="n">
         <v>11</v>
       </c>
@@ -6776,7 +6776,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="445.25" customHeight="1">
+    <row r="16" ht="409" customHeight="1">
       <c r="A16" s="58" t="n">
         <v>12</v>
       </c>
@@ -6889,7 +6889,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="194" customHeight="1">
+    <row r="17" ht="163.5" customHeight="1">
       <c r="A17" s="58" t="n">
         <v>13</v>
       </c>
@@ -6930,7 +6930,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="420.5" customHeight="1">
+    <row r="18" ht="271.25" customHeight="1">
       <c r="A18" s="58" t="n">
         <v>14</v>
       </c>
@@ -6977,7 +6977,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="420.5" customHeight="1">
+    <row r="19" ht="271.25" customHeight="1">
       <c r="A19" s="58" t="n">
         <v>15</v>
       </c>
@@ -7017,7 +7017,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="420.5" customHeight="1">
+    <row r="20" ht="271.25" customHeight="1">
       <c r="A20" s="58" t="n">
         <v>16</v>
       </c>
@@ -7054,7 +7054,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="120" customHeight="1">
+    <row r="21" ht="90" customHeight="1">
       <c r="A21" s="58" t="n">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
fix(dwt): cuaca DWT (jalan/kereta) kembali live di prod — jangan sampai balik index.html
Di dev aman (vite proxy /event → publik.bmkg.go.id), tapi di prod/Vercel
path /event/* tidak punya handler → jatuh ke SPA rewrite → response 200
text/html (index.html) → transport & land-based diam-diam pakai fallback
mock. Ketahuan dari sheet 'Audit Card + Screenshot' yang sample-nya HTML.

- api.ts: helper bmkgProxied(path) — satu titik konversi path → URL proxy
  (dev path-style, prod /api-bmkg?path=…); dipakai openData DWT
- api/bmkg.ts: routing event/* → https://publik.bmkg.go.id (setara proxy
  vite /event, tanpa header khusus)
- capture_card_screenshots.js pindah ke docs/scrapping_cuaca-bmkg-go-id/
  (import 'playwright' resolve ke node_modules lokal folder itu)
- screenshot + dump + sheet di-regenerate: sample DWT kini JSON row
  cuaca kecamatan/stasiun (bukan HTML)
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -1401,7 +1401,7 @@
       <row>12</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="1962150"/>
+    <ext cx="4381500" cy="4229100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -6248,7 +6248,7 @@
     <row r="2">
       <c r="A2" s="55" t="inlineStr">
         <is>
-          <t>Screenshot diambil dari deployment prod (server.mjs + dist, data live) dengan API BOX MARKER aktif — border merah = live, amber = campuran, abu = mock (lihat kolom Status). Sumber screenshot: docs/screenshots/cards/ · skrip: docs/artifacts/scripts/capture_card_screenshots.js</t>
+          <t>Screenshot diambil dari deployment prod (server.mjs + dist, data live) dengan API BOX MARKER aktif — border merah = live, amber = campuran, abu = mock (lihat kolom Status). Sumber screenshot: docs/screenshots/cards/ · skrip: docs/scrapping_cuaca-bmkg-go-id/capture_card_screenshots.js</t>
         </is>
       </c>
     </row>
@@ -6325,13 +6325,13 @@
       </c>
       <c r="F5" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-6.2804&amp;lon=106.9507
+          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-7.8385&amp;lon=110.3275
 [200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666</t>
         </is>
       </c>
       <c r="G5" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.94655786745837,"lat":-6.277639992667722,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.9465578675,"lat":-6.2776399927,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T06:00:00Z","t":34,"tcc":93,"tp":0,"weather":3,"weather_desc":"Berawan","weather_desc_en":"Mostly Cloudy","wd_deg":306,"wd":"W","wd_to":"E","ws":11.5,"hu":48,"vs":null,"vs_text":null,"time_index":"5-6","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan-am.svg","utc_datetime":"2026-09-22 06:00:00","local_datetime":"2026-09-22 13:00:00"},{"datetime":"2026-09-22T07:00:00Z","t":33,"tcc":50,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":290,"wd":"W","wd_to":"E","ws":14,"hu":48,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":30,"tcc":82,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":290,"wd":"W","wd_to":"E",
+          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,
 … (dipotong)</t>
         </is>
       </c>
@@ -6367,7 +6367,7 @@
       </c>
       <c r="F6" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-6.2804&amp;lon=106.9507
+          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-7.8385&amp;lon=110.3275
 [200] /api-bmkgapi/df/v1/adm/coord&amp;lat=-6.2&amp;lon=106.816666
 [200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666
 [200] https://cuaca.bmkg.go.id/api/v1/sunset/json?lat=-6.2&amp;lng=106.816666</t>
@@ -6375,7 +6375,7 @@
       </c>
       <c r="G6" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.94655786745837,"lat":-6.277639992667722,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.9465578675,"lat":-6.2776399927,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T06:00:00Z","t":34,"tcc":93,"tp":0,"weather":3,"weather_desc":"Berawan","weather_desc_en":"Mostly Cloudy","wd_deg":306,"wd":"W","wd_to":"E","ws":11.5,"hu":48,"vs":null,"vs_text":null,"time_index":"5-6","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan-am.svg","utc_datetime":"2026-09-22 06:00:00","local_datetime":"2026-09-22 13:00:00"},{"datetime":"2026-09-22T07:00:00Z","t":33,"tcc":50,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":290,"wd":"W","wd_to":"E","ws":14,"hu":48,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":30,"tcc":82,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":290,"wd":"W","wd_to":"E",
+          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,
 … (dipotong)</t>
         </is>
       </c>
@@ -6411,13 +6411,13 @@
       </c>
       <c r="F7" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-6.2804&amp;lon=106.9507
+          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-7.8385&amp;lon=110.3275
 (belum terekam saat capture) — Open Data RESMI: prakiraan-cuaca (adm4)</t>
         </is>
       </c>
       <c r="G7" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.94655786745837,"lat":-6.277639992667722,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.9465578675,"lat":-6.2776399927,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T06:00:00Z","t":34,"tcc":93,"tp":0,"weather":3,"weather_desc":"Berawan","weather_desc_en":"Mostly Cloudy","wd_deg":306,"wd":"W","wd_to":"E","ws":11.5,"hu":48,"vs":null,"vs_text":null,"time_index":"5-6","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan-am.svg","utc_datetime":"2026-09-22 06:00:00","local_datetime":"2026-09-22 13:00:00"},{"datetime":"2026-09-22T07:00:00Z","t":33,"tcc":50,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":290,"wd":"W","wd_to":"E","ws":14,"hu":48,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":30,"tcc":82,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":290,"wd":"W","wd_to":"E",
+          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,
 … (dipotong)</t>
         </is>
       </c>
@@ -6530,12 +6530,13 @@
       </c>
       <c r="F10" s="62" t="inlineStr">
         <is>
-          <t>(belum terekam saat capture) — Open Data: gempa (TEWS)</t>
+          <t>[200] https://data.bmkg.go.id/DataMKG/TEWS/gempadirasakan.json</t>
         </is>
       </c>
       <c r="G10" s="62" t="inlineStr">
         <is>
-          <t>— (tidak ada response live)</t>
+          <t>{"Infogempa":{"gempa":[{"Tanggal":"22 Sep 2026","Jam":"10:36:27 WIB","DateTime":"2026-09-22T03:36:27+00:00","Coordinates":"-8.43,121.44","Lintang":"8.43 LS","Bujur":"121.44 BT","Magnitude":"4.8","Kedalaman":"14 km","Wilayah":"Pusat gempa berada di laut 31 km timur laut Mbay, Nagekeo","Dirasakan":"IV Kab. Nagekeo, III Kab. Ngada, III Kab. Sikka, III Kab. Ende, II Kab. Manggarai"},{"Tanggal":"21 Sep 2026","Jam":"19:35:22 WIB","DateTime":"2026-09-21T12:35:22+00:00","Coordinates":"-0.52,99.37","Lintang":"0.52 LS","Bujur":"99.37 BT","Magnitude":"4.5","Kedalaman":"10 km","Wilayah":"Pusat gempa berada di laut 76 km Barat Daya Agam","Dirasakan":"III-IV Agam, II-III Kab. Padang Pariaman, II-III Kota Pariaman, II-III Kota Padang"},{"Tanggal":"21 Sep 2026","Jam":"14:31:07 WIB","DateTime":"2026-09-21T07:31:07+00:00","Coordinates":"-0.70,122.45","Lintang":"0.70 LS","Bujur":"122.45 BT","Magnitude":"5.3","Kedalaman":"10 km","Wilayah":"Pusat gempa berada di laut 26 km BaratDaya Pulau Puah","Dirasakan":"IV-V Luwuk, II-III Kab. Pohuwato"},{"Tanggal":"21 Sep 2026","Jam":"12:59:25 WIB","DateTime":"2026-09-21T05:59:25+00:00","Coordinates":"-8.28,120.57","Lintang":"8.28 LS","Bujur":"120.57 BT","Magnitude":"3.5","Kedalaman":"7 km","Wilayah":"Pusat gempa berada di laut 38 km utara Ruteng, Manggarai","Dirasakan":"II-III Manggarai"},{"Tanggal":"21 Sep 2026","Jam":"08:41:37 WIB","DateTime":"2026-09-21T01:41:37+00:00","Coordinates":"-8.33,120.59","Lintang":"8.33 LS","Bujur":"120.59 BT","Magnitude":"5.3"
+… (dipotong)</t>
         </is>
       </c>
       <c r="H10" s="63" t="inlineStr">
@@ -6618,7 +6619,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="310.5" customHeight="1">
+    <row r="13" ht="341" customHeight="1">
       <c r="A13" s="58" t="n">
         <v>9</v>
       </c>
@@ -6643,36 +6644,14 @@
       </c>
       <c r="F13" s="62" t="inlineStr">
         <is>
-          <t>[200] /event/source/dwt/apiDF_Kereta/manifest_times.json
+          <t>[200] /api-bmkgevent/source/dwt/apiDF_Kereta/202609101600.json
 [200] /api-bmkgapi/v1/public/maritim/nearest-location&amp;lat=-6.2&amp;long=106.816666
 [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
         </is>
       </c>
       <c r="G13" s="62" t="inlineStr">
         <is>
-          <t>&lt;!doctype html&gt;
-&lt;html lang="id" class="dark"&gt;
-  &lt;head&gt;
-    &lt;meta charset="UTF-8" /&gt;
-    &lt;link rel="icon" type="image/svg+xml" href="/assets/logo-BenySzP1.svg" /&gt;
-    &lt;!-- Preconnect to Google Fonts to fetch fonts faster and prevent Flash of Unstyled Text (FOUT) --&gt;
-    &lt;link rel="preconnect" href="https://fonts.googleapis.com" /&gt;
-    &lt;link rel="preconnect" href="https://fonts.gstatic.com" crossorigin /&gt;
-    &lt;link href="https://fonts.googleapis.com/css2?family=Plus+Jakarta+Sans:wght@300;400;500;600;700;800&amp;display=swap" rel="stylesheet" /&gt;
-    &lt;meta name="viewport" content="width=device-width, initial-scale=1.0, viewport-fit=cover" /&gt;
-    &lt;meta name="color-scheme" content="dark" /&gt;
-    &lt;meta name="theme-color" content="#070c19" /&gt;
-    &lt;meta name="apple-mobile-web-app-capable" content="yes" /&gt;
-    &lt;meta name="apple-mobile-web-app-status-bar-style" content="black-translucent" /&gt;
-    &lt;meta name="description" content="Portal Redesign Digital Weather Info BMKG - Layanan Informasi Cuaca Publik, Penerbangan, Maritim, Peringatan Dini Angin &amp; Hujan, dan Satelit Cuaca Himawari-9." /&gt;
-    &lt;meta name="keywords" content="BMKG, Info BMKG, Cuaca Indonesia, Radar Cuaca, Satelit Himawari-9, Gempa Megathrust, Peringatan Dini" /&gt;
-    &lt;meta name="author" content="BMKG Indonesia" /&gt;
-    &lt;title&gt;BMKG | Portal Informasi Cuaca, Iklim &amp; Geofisika Indonesia&lt;/title&gt;
-    &lt;script&gt;
-      (function() {
-        try {
-          const theme = localStorage.getItem('bmkg-theme-v2');
-          const isDark =
+          <t>[["","Kota Jakarta Pusat","Menteng ",-6.19809917164,106.84108701,"5005610","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.149180001,106.827000026,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.141079981,106.822740007,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Pusat","Senen ",-6.193899969,106.856519999,"5005611","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Pusat","Kemayoran ",-6.174619999,106.844179993,"5005614","2026-09-10 16:00:00",["83","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Barat","Cengkareng ",-6.158600003,106.756496988,"5005623","2026-09-10 16:00:00",["82","26","2","E","0.5"],"ndf"],["","Kota Tangerang","Batuceper",-6.169660008,106.681367978,"5008776","2026-09-10 16:00:00",["85","26","2","SE","2.4"],"ndf"],["","Kota Jakarta Barat","Grogol Petamburan ",-6.161280032,106.772031002,"5005620","2026-09-10 16:00:00",["82","26","2","E","0.5"],"ndf"],["","Kota Jakarta Barat","Tambora",-6.155889966,106.801510993,"5005621","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Timur","Jakarta Timur",-6.212939965,106.900340002,"501191","2026-09-10 16:00:00",["88","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Selatan","Tebet ",-6.225910038,106.858320013,"5005597","2026-09-10 16:00:00",["87","26","2","SE","2.5"],"ndf"],["","Kab. Karawang","Kotabaru",-6.406120034,107.458950011,"5009561"
 … (dipotong)</t>
         </is>
       </c>
@@ -6710,14 +6689,14 @@
       </c>
       <c r="F14" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-6.2804&amp;lon=106.9507
+          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-7.8385&amp;lon=110.3275
 [200] /api-bmkgapi/v1/public/maritim/nearest-location&amp;lat=-6.2&amp;long=106.816666
 [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
         </is>
       </c>
       <c r="G14" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.94655786745837,"lat":-6.277639992667722,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.9465578675,"lat":-6.2776399927,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T06:00:00Z","t":34,"tcc":93,"tp":0,"weather":3,"weather_desc":"Berawan","weather_desc_en":"Mostly Cloudy","wd_deg":306,"wd":"W","wd_to":"E","ws":11.5,"hu":48,"vs":null,"vs_text":null,"time_index":"5-6","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan-am.svg","utc_datetime":"2026-09-22 06:00:00","local_datetime":"2026-09-22 13:00:00"},{"datetime":"2026-09-22T07:00:00Z","t":33,"tcc":50,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":290,"wd":"W","wd_to":"E","ws":14,"hu":48,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":30,"tcc":82,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":290,"wd":"W","wd_to":"E",
+          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,
 … (dipotong)</t>
         </is>
       </c>
@@ -6756,15 +6735,15 @@
       </c>
       <c r="F15" s="62" t="inlineStr">
         <is>
-          <t>(belum terekam saat capture) — Maritim: overview tinggi gelombang (232 wilayah)
-(belum terekam saat capture) — Maritim: polygon 232 wilayah perairan
+          <t>[200] https://maritim.bmkg.go.id/public_api/overview/gelombang.json
+[200] https://maritim.bmkg.go.id/public_api/static/wilayah_perairan.json
 [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json
-[200] /event/source/dwt/apiDF_Kereta/manifest_times.json</t>
+[200] /api-bmkgevent/source/dwt/apiDF_Kereta/202609101600.json</t>
         </is>
       </c>
       <c r="G15" s="62" t="inlineStr">
         <is>
-          <t>{"code": "F.09", "name": "Teluk Jakarta", "issued": "2026-09-21 23:39 UTC", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "data": [{"valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "time_desc": "Hari ini", "weather": "Berawan", "weather_desc": "Hari ini untuk Teluk Jakarta diperkirakan berawan, dengan kecepatan angin pada umumnya 5 - 18 knot bertiup dari arah selatan, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": "Rendah", "wave_desc": "0.5 - 1.25 m", "wind_from": "Selatan", "wind_to": "Barat Daya", "wind_speed_min": 5, "wind_speed_max": 18}, {"valid_from": "2026-09-22 00:00 UTC", "valid_to": "2026-09-22 12:00 UTC", "time_desc": "Besok", "weather": "Hujan Ringan", "weather_desc": "Besok untuk Teluk Jakarta diperkirakan hujan ringan, dengan kecepatan angin pada umumnya 11 - 33 knot bertiup dari arah utara, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": "Rendah", "wave_desc": "0.5 - 1.25 m", "wind_from": "Utara", "wind_to": "Barat Daya", "wind_speed_min": 11, "wind_speed_max": 33}, {"valid_from": "2026-09-22 12:00 UTC", "valid_to": "2026-09-23 12:00 UTC", "time_desc": "H+2", "weather": "Hujan Ringan", "weather_desc": "Lusa untuk Teluk Jakarta diperkirakan hujan ringan, dengan kecepatan angin pada umumn
+          <t>{"U.04": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "U.02": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "U.01": {"issued": "2026-09-21 23:47 UTC", "today": "Rendah", "tomorrow": "Rendah", "h2": "Rendah", "h3": "Rendah"}, "U.03": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.09": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.05": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.12": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.02": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.08": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Tinggi"}, "B.03": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.07": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Tinggi"}, "B.04": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.06": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Seda
 … (dipotong)</t>
         </is>
       </c>
@@ -6913,13 +6892,13 @@
       </c>
       <c r="F17" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-6.2804&amp;lon=106.9507
+          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-7.8385&amp;lon=110.3275
 (belum terekam saat capture) — Overpass API: POI OpenStreetMap</t>
         </is>
       </c>
       <c r="G17" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.94655786745837,"lat":-6.277639992667722,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.9465578675,"lat":-6.2776399927,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T06:00:00Z","t":34,"tcc":93,"tp":0,"weather":3,"weather_desc":"Berawan","weather_desc_en":"Mostly Cloudy","wd_deg":306,"wd":"W","wd_to":"E","ws":11.5,"hu":48,"vs":null,"vs_text":null,"time_index":"5-6","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan-am.svg","utc_datetime":"2026-09-22 06:00:00","local_datetime":"2026-09-22 13:00:00"},{"datetime":"2026-09-22T07:00:00Z","t":33,"tcc":50,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":290,"wd":"W","wd_to":"E","ws":14,"hu":48,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":30,"tcc":82,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":290,"wd":"W","wd_to":"E",
+          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,
 … (dipotong)</t>
         </is>
       </c>
@@ -6957,8 +6936,8 @@
       </c>
       <c r="F18" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-6.2804&amp;lon=106.9507
-[200] /event/source/dwt/apiDF_Kereta/manifest_times.json
+          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-7.8385&amp;lon=110.3275
+[200] /api-bmkgevent/source/dwt/apiDF_Kereta/202609101600.json
 (belum terekam saat capture) — Overpass API: POI OpenStreetMap
 (belum terekam saat capture) — Nominatim: geocode OSM
 (belum terekam saat capture) — OSRM: routing</t>
@@ -6966,7 +6945,7 @@
       </c>
       <c r="G18" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.94655786745837,"lat":-6.277639992667722,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"32","adm2":"32.75","adm3":"32.75.09","adm4":"32.75.09.1003","provinsi":"Jawa Barat","kotkab":"Kota Bekasi","kecamatan":"Jatiasih","desa":"Jatikramat","lon":106.9465578675,"lat":-6.2776399927,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T06:00:00Z","t":34,"tcc":93,"tp":0,"weather":3,"weather_desc":"Berawan","weather_desc_en":"Mostly Cloudy","wd_deg":306,"wd":"W","wd_to":"E","ws":11.5,"hu":48,"vs":null,"vs_text":null,"time_index":"5-6","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan-am.svg","utc_datetime":"2026-09-22 06:00:00","local_datetime":"2026-09-22 13:00:00"},{"datetime":"2026-09-22T07:00:00Z","t":33,"tcc":50,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":290,"wd":"W","wd_to":"E","ws":14,"hu":48,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":30,"tcc":82,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":290,"wd":"W","wd_to":"E",
+          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,
 … (dipotong)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
style(xlsx): sample response dirapikan 1 baris (JSON pretty-print → spasi)
Pelabuhan & Pasut (port-tide) tadinya membentang 3.238 baris karena
pelabuhan_list pretty-print; marine-map 42 baris. Builder kini melipat
newline/whitespace jadi satu baris untuk semua row — tampilan seragam,
tinggi baris menyesuaikan otomatis.
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -6331,8 +6331,7 @@
       </c>
       <c r="G5" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,
-… (dipotong)</t>
+          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173, … (dipotong)</t>
         </is>
       </c>
       <c r="H5" s="63" t="inlineStr">
@@ -6341,7 +6340,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="163.5" customHeight="1">
+    <row r="6" ht="153" customHeight="1">
       <c r="A6" s="58" t="n">
         <v>2</v>
       </c>
@@ -6375,8 +6374,7 @@
       </c>
       <c r="G6" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,
-… (dipotong)</t>
+          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173, … (dipotong)</t>
         </is>
       </c>
       <c r="H6" s="63" t="inlineStr">
@@ -6417,8 +6415,7 @@
       </c>
       <c r="G7" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,
-… (dipotong)</t>
+          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173, … (dipotong)</t>
         </is>
       </c>
       <c r="H7" s="63" t="inlineStr">
@@ -6498,7 +6495,7 @@
       </c>
       <c r="G9" s="62" t="inlineStr">
         <is>
-          <t>[{"title":"Prakiraan Cuaca Esok Hari, Selasa, 22 September 2026.","videoUrl":"https://www.youtube.com/watch?v=l6NWtkthnzU"},{"title":"Prakiraan Cuaca Esok Hari,  Senin, 21 September 2026.","videoUrl":"https://www.youtube.com/watch?v=GNIhEbJS8q4"},{"title":"Prakiraan Cuaca Esok Hari, Minggu, 20 September 2026","videoUrl":"https://www.youtube.com/watch?v=kCepZRm8uIQ"},{"title":"Prakiraan Cuaca Esok Hari, Sabtu, 19 September 2026.","videoUrl":"https://www.youtube.com/watch?v=9egb1zLG0PM"},{"title":"Prakiraan Cuaca Esok Hari, Jumat, 18 September 2026.","videoUrl":"https://www.youtube.com/watch?v=1Dy6sPbtzpc"},{"title":"Prakiraan Cuaca Esok Hari Kamis, 17 September 2026","videoUrl":"https://www.youtube.com/watch?v=Xx3Ddki3bHk"}]</t>
+          <t>[{"title":"Prakiraan Cuaca Esok Hari, Selasa, 22 September 2026.","videoUrl":"https://www.youtube.com/watch?v=l6NWtkthnzU"},{"title":"Prakiraan Cuaca Esok Hari, Senin, 21 September 2026.","videoUrl":"https://www.youtube.com/watch?v=GNIhEbJS8q4"},{"title":"Prakiraan Cuaca Esok Hari, Minggu, 20 September 2026","videoUrl":"https://www.youtube.com/watch?v=kCepZRm8uIQ"},{"title":"Prakiraan Cuaca Esok Hari, Sabtu, 19 September 2026.","videoUrl":"https://www.youtube.com/watch?v=9egb1zLG0PM"},{"title":"Prakiraan Cuaca Esok Hari, Jumat, 18 September 2026.","videoUrl":"https://www.youtube.com/watch?v=1Dy6sPbtzpc"},{"title":"Prakiraan Cuaca Esok Hari Kamis, 17 September 2026","videoUrl":"https://www.youtube.com/watch?v=Xx3Ddki3bHk"}]</t>
         </is>
       </c>
       <c r="H9" s="63" t="inlineStr">
@@ -6535,8 +6532,7 @@
       </c>
       <c r="G10" s="62" t="inlineStr">
         <is>
-          <t>{"Infogempa":{"gempa":[{"Tanggal":"22 Sep 2026","Jam":"10:36:27 WIB","DateTime":"2026-09-22T03:36:27+00:00","Coordinates":"-8.43,121.44","Lintang":"8.43 LS","Bujur":"121.44 BT","Magnitude":"4.8","Kedalaman":"14 km","Wilayah":"Pusat gempa berada di laut 31 km timur laut Mbay, Nagekeo","Dirasakan":"IV Kab. Nagekeo, III Kab. Ngada, III Kab. Sikka, III Kab. Ende, II Kab. Manggarai"},{"Tanggal":"21 Sep 2026","Jam":"19:35:22 WIB","DateTime":"2026-09-21T12:35:22+00:00","Coordinates":"-0.52,99.37","Lintang":"0.52 LS","Bujur":"99.37 BT","Magnitude":"4.5","Kedalaman":"10 km","Wilayah":"Pusat gempa berada di laut 76 km Barat Daya Agam","Dirasakan":"III-IV Agam, II-III Kab. Padang Pariaman, II-III Kota Pariaman, II-III Kota Padang"},{"Tanggal":"21 Sep 2026","Jam":"14:31:07 WIB","DateTime":"2026-09-21T07:31:07+00:00","Coordinates":"-0.70,122.45","Lintang":"0.70 LS","Bujur":"122.45 BT","Magnitude":"5.3","Kedalaman":"10 km","Wilayah":"Pusat gempa berada di laut 26 km BaratDaya Pulau Puah","Dirasakan":"IV-V Luwuk, II-III Kab. Pohuwato"},{"Tanggal":"21 Sep 2026","Jam":"12:59:25 WIB","DateTime":"2026-09-21T05:59:25+00:00","Coordinates":"-8.28,120.57","Lintang":"8.28 LS","Bujur":"120.57 BT","Magnitude":"3.5","Kedalaman":"7 km","Wilayah":"Pusat gempa berada di laut 38 km utara Ruteng, Manggarai","Dirasakan":"II-III Manggarai"},{"Tanggal":"21 Sep 2026","Jam":"08:41:37 WIB","DateTime":"2026-09-21T01:41:37+00:00","Coordinates":"-8.33,120.59","Lintang":"8.33 LS","Bujur":"120.59 BT","Magnitude":"5.3"
-… (dipotong)</t>
+          <t>{"Infogempa":{"gempa":[{"Tanggal":"22 Sep 2026","Jam":"10:36:27 WIB","DateTime":"2026-09-22T03:36:27+00:00","Coordinates":"-8.43,121.44","Lintang":"8.43 LS","Bujur":"121.44 BT","Magnitude":"4.8","Kedalaman":"14 km","Wilayah":"Pusat gempa berada di laut 31 km timur laut Mbay, Nagekeo","Dirasakan":"IV Kab. Nagekeo, III Kab. Ngada, III Kab. Sikka, III Kab. Ende, II Kab. Manggarai"},{"Tanggal":"21 Sep 2026","Jam":"19:35:22 WIB","DateTime":"2026-09-21T12:35:22+00:00","Coordinates":"-0.52,99.37","Lintang":"0.52 LS","Bujur":"99.37 BT","Magnitude":"4.5","Kedalaman":"10 km","Wilayah":"Pusat gempa berada di laut 76 km Barat Daya Agam","Dirasakan":"III-IV Agam, II-III Kab. Padang Pariaman, II-III Kota Pariaman, II-III Kota Padang"},{"Tanggal":"21 Sep 2026","Jam":"14:31:07 WIB","DateTime":"2026-09-21T07:31:07+00:00","Coordinates":"-0.70,122.45","Lintang":"0.70 LS","Bujur":"122.45 BT","Magnitude":"5.3","Kedalaman":"10 km","Wilayah":"Pusat gempa berada di laut 26 km BaratDaya Pulau Puah","Dirasakan":"IV-V Luwuk, II-III Kab. Pohuwato"},{"Tanggal":"21 Sep 2026","Jam":"12:59:25 WIB","DateTime":"2026-09-21T05:59:25+00:00","Coordinates":"-8.28,120.57","Lintang":"8.28 LS","Bujur":"120.57 BT","Magnitude":"3.5","Kedalaman":"7 km","Wilayah":"Pusat gempa berada di laut 38 km utara Ruteng, Manggarai","Dirasakan":"II-III Manggarai"},{"Tanggal":"21 Sep 2026","Jam":"08:41:37 WIB","DateTime":"2026-09-21T01:41:37+00:00","Coordinates":"-8.33,120.59","Lintang":"8.33 LS","Bujur":"120.59 BT","Magnitude":"5.3" … (dipotong)</t>
         </is>
       </c>
       <c r="H10" s="63" t="inlineStr">
@@ -6651,8 +6647,7 @@
       </c>
       <c r="G13" s="62" t="inlineStr">
         <is>
-          <t>[["","Kota Jakarta Pusat","Menteng ",-6.19809917164,106.84108701,"5005610","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.149180001,106.827000026,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.141079981,106.822740007,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Pusat","Senen ",-6.193899969,106.856519999,"5005611","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Pusat","Kemayoran ",-6.174619999,106.844179993,"5005614","2026-09-10 16:00:00",["83","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Barat","Cengkareng ",-6.158600003,106.756496988,"5005623","2026-09-10 16:00:00",["82","26","2","E","0.5"],"ndf"],["","Kota Tangerang","Batuceper",-6.169660008,106.681367978,"5008776","2026-09-10 16:00:00",["85","26","2","SE","2.4"],"ndf"],["","Kota Jakarta Barat","Grogol Petamburan ",-6.161280032,106.772031002,"5005620","2026-09-10 16:00:00",["82","26","2","E","0.5"],"ndf"],["","Kota Jakarta Barat","Tambora",-6.155889966,106.801510993,"5005621","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Timur","Jakarta Timur",-6.212939965,106.900340002,"501191","2026-09-10 16:00:00",["88","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Selatan","Tebet ",-6.225910038,106.858320013,"5005597","2026-09-10 16:00:00",["87","26","2","SE","2.5"],"ndf"],["","Kab. Karawang","Kotabaru",-6.406120034,107.458950011,"5009561"
-… (dipotong)</t>
+          <t>[["","Kota Jakarta Pusat","Menteng ",-6.19809917164,106.84108701,"5005610","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.149180001,106.827000026,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.141079981,106.822740007,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Pusat","Senen ",-6.193899969,106.856519999,"5005611","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Pusat","Kemayoran ",-6.174619999,106.844179993,"5005614","2026-09-10 16:00:00",["83","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Barat","Cengkareng ",-6.158600003,106.756496988,"5005623","2026-09-10 16:00:00",["82","26","2","E","0.5"],"ndf"],["","Kota Tangerang","Batuceper",-6.169660008,106.681367978,"5008776","2026-09-10 16:00:00",["85","26","2","SE","2.4"],"ndf"],["","Kota Jakarta Barat","Grogol Petamburan ",-6.161280032,106.772031002,"5005620","2026-09-10 16:00:00",["82","26","2","E","0.5"],"ndf"],["","Kota Jakarta Barat","Tambora",-6.155889966,106.801510993,"5005621","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Timur","Jakarta Timur",-6.212939965,106.900340002,"501191","2026-09-10 16:00:00",["88","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Selatan","Tebet ",-6.225910038,106.858320013,"5005597","2026-09-10 16:00:00",["87","26","2","SE","2.5"],"ndf"],["","Kab. Karawang","Kotabaru",-6.406120034,107.458950011,"5009561" … (dipotong)</t>
         </is>
       </c>
       <c r="H13" s="63" t="inlineStr">
@@ -6696,8 +6691,7 @@
       </c>
       <c r="G14" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,
-… (dipotong)</t>
+          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173, … (dipotong)</t>
         </is>
       </c>
       <c r="H14" s="63" t="inlineStr">
@@ -6743,8 +6737,7 @@
       </c>
       <c r="G15" s="62" t="inlineStr">
         <is>
-          <t>{"U.04": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "U.02": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "U.01": {"issued": "2026-09-21 23:47 UTC", "today": "Rendah", "tomorrow": "Rendah", "h2": "Rendah", "h3": "Rendah"}, "U.03": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.09": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.05": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.12": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.02": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.08": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Tinggi"}, "B.03": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.07": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Tinggi"}, "B.04": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.06": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Seda
-… (dipotong)</t>
+          <t>{"U.04": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "U.02": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "U.01": {"issued": "2026-09-21 23:47 UTC", "today": "Rendah", "tomorrow": "Rendah", "h2": "Rendah", "h3": "Rendah"}, "U.03": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.09": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.05": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.12": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.02": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.08": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Tinggi"}, "B.03": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.07": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Tinggi"}, "B.04": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.06": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Seda … (dipotong)</t>
         </is>
       </c>
       <c r="H15" s="63" t="inlineStr">
@@ -6755,7 +6748,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="409" customHeight="1">
+    <row r="16" ht="287.75" customHeight="1">
       <c r="A16" s="58" t="n">
         <v>12</v>
       </c>
@@ -6785,81 +6778,7 @@
       </c>
       <c r="G16" s="62" t="inlineStr">
         <is>
-          <t>{
-  "files": [
-    {
-      "coor": [
-        1.198331,
-        109.054462
-      ],
-      "file_date": "2026-09-21 23:47 UTC",
-      "kb": 1720,
-      "name": "0088_Sintete.json",
-      "portname": "Sintete",
-      "type": "utama"
-    },
-    {
-      "coor": [
-        0.00214,
-        109.285391
-      ],
-      "file_date": "2026-09-21 23:47 UTC",
-      "kb": 1713,
-      "name": "0310_PPP Sungai Rengas.json",
-      "portname": "PPP Sungai Rengas",
-      "type": "utama"
-    },
-    {
-      "coor": [
-        -2.531535,
-        110.21588
-      ],
-      "file_date": "2026-09-21 23:47 UTC",
-      "kb": 1692,
-      "name": "0092_Kendawangan.json",
-      "portname": "Kendawangan",
-      "type": "utama"
-    },
-    {
-      "coor": [
-        4.145037,
-        117.665883
-      ],
-      "file_date": "2026-09-21 23:47 UTC",
-      "kb": 1679,
-      "name": "0237_Nunukan.json",
-      "portname": "Nunukan",
-      "type": "utama"
-    },
-    {
-      "coor": [
-        -8.6679806,
-        115.261925
-      ],
-      "file_date": "2026-09-21 23:47 UTC",
-      "kb": 1646,
-      "name": "0603_Sanur.json",
-      "portname": "Sanur",
-      "type": "utama"
-    },
-    {
-      "coor": [
-        -5.35863269,
-        105.81975796
-      ],
-      "file_date": "2026-09-21 23:47 UTC",
-      "kb": 1670,
-      "name": "0325_PPP Labuhan Maringgai.json",
-      "portname": "PPP Labuhan Maringgai",
-      "type": "utama"
-    },
-    {
-      "coor": [
-        -8.67206,
-        115.55675
-      ],
-      "file_date": "2026-09-
-… (dipotong)</t>
+          <t>{ "files": [ { "coor": [ 1.198331, 109.054462 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1720, "name": "0088_Sintete.json", "portname": "Sintete", "type": "utama" }, { "coor": [ 0.00214, 109.285391 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1713, "name": "0310_PPP Sungai Rengas.json", "portname": "PPP Sungai Rengas", "type": "utama" }, { "coor": [ -2.531535, 110.21588 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1692, "name": "0092_Kendawangan.json", "portname": "Kendawangan", "type": "utama" }, { "coor": [ 4.145037, 117.665883 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1679, "name": "0237_Nunukan.json", "portname": "Nunukan", "type": "utama" }, { "coor": [ -8.6679806, 115.261925 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1646, "name": "0603_Sanur.json", "portname": "Sanur", "type": "utama" }, { "coor": [ -5.35863269, 105.81975796 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1670, "name": "0325_PPP Labuhan Maringgai.json", "portname": "PPP Labuhan Maringgai", "type": "utama" }, { "coor": [ -8.67206, 115.55675 ], "file_date": "2026-09- … (dipotong)</t>
         </is>
       </c>
       <c r="H16" s="63" t="inlineStr">
@@ -6868,7 +6787,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="163.5" customHeight="1">
+    <row r="17" ht="153" customHeight="1">
       <c r="A17" s="58" t="n">
         <v>13</v>
       </c>
@@ -6898,8 +6817,7 @@
       </c>
       <c r="G17" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,
-… (dipotong)</t>
+          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173, … (dipotong)</t>
         </is>
       </c>
       <c r="H17" s="63" t="inlineStr">
@@ -6945,8 +6863,7 @@
       </c>
       <c r="G18" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,
-… (dipotong)</t>
+          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173, … (dipotong)</t>
         </is>
       </c>
       <c r="H18" s="63" t="inlineStr">

</xml_diff>

<commit_message>
docs(xlsx): sheet audit card — sample response per API + kolom field dipakai UI
- kolom 'Sample Response (per API, dipotong)': tiap API pada card kini punya
  blok sample sendiri (▸ nama + JSON 600 char, dirapikan 1 baris) — sebelumnya
  hanya sample API pertama yang tampil
- kolom baru 'Field dipakai UI + penjelasan': pemetaan response → nilai yang
  dirender UI per API (sumber kebenaran: src/services/bmkg/adapters.ts,
  openData.ts) + penjelasan singkat konversi/estimasi (tp×20, feels-like,
  UV dari tcc, dsb.) — 25 API terpetakan
- tinggi baris mengikuti konten terpanjang (G/H/I), batas Excel 409,5pt
- layout 9 kolom (A1:I…), file tetap ~560KB
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -6225,17 +6225,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="115" customWidth="1" min="7" max="7"/>
-    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="92" customWidth="1" min="7" max="7"/>
+    <col width="56" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6248,7 +6249,7 @@
     <row r="2">
       <c r="A2" s="55" t="inlineStr">
         <is>
-          <t>Screenshot diambil dari deployment prod (server.mjs + dist, data live) dengan API BOX MARKER aktif — border merah = live, amber = campuran, abu = mock (lihat kolom Status). Sumber screenshot: docs/screenshots/cards/ · skrip: docs/scrapping_cuaca-bmkg-go-id/capture_card_screenshots.js</t>
+          <t>Screenshot diambil dari deployment prod (server.mjs + dist, data live) dengan API BOX MARKER aktif — border merah = live, amber = campuran, abu = mock (lihat kolom Status). Kolom "Field dipakai UI" = pemetaan response → nilai yang dirender (sumber: src/services/bmkg/adapters.ts). Sumber screenshot: docs/screenshots/cards/ · skrip: docs/scrapping_cuaca-bmkg-go-id/capture_card_screenshots.js</t>
         </is>
       </c>
     </row>
@@ -6292,10 +6293,15 @@
       </c>
       <c r="G4" s="57" t="inlineStr">
         <is>
-          <t>Sample Response (potongan)</t>
+          <t>Sample Response (per API, dipotong)</t>
         </is>
       </c>
       <c r="H4" s="57" t="inlineStr">
+        <is>
+          <t>Field dipakai UI + penjelasan</t>
+        </is>
+      </c>
+      <c r="I4" s="57" t="inlineStr">
         <is>
           <t>Catatan</t>
         </is>
@@ -6331,16 +6337,27 @@
       </c>
       <c r="G5" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173, … (dipotong)</t>
-        </is>
-      </c>
-      <c r="H5" s="63" t="inlineStr">
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"w …
+▸ Present Weather: cuaca saat ini
+{"status":200,"data":{"lokasi":{"lon":106.81596823959143,"lat":-6.197052719903746,"adm1":"31","adm2":"31.71","adm3":"31.71.07","adm4":"31.71.07.1005","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Tanah Abang","desa":"Kebon Melati","distance":0},"cuaca":{"weather":4,"weather_desc":"Berawan Tebal","weather_desc_en":"Overcast","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan tebal-am.svg","datetime":"2026-09-22T06:00:00.000Z","local_datetime":"2026-09-22 13:00:00","t":33,"tcc":87,"wd_deg":21,"wd":"N","wd_to":"S","ws":10.2,"hu":46,"vs":null,"vs_text":null} …</t>
+        </is>
+      </c>
+      <c r="H5" s="59" t="inlineStr">
+        <is>
+          <t>▸ data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ data.t, hu, weather_desc, ws, tcc, vs, local_datetime
+  Kondisi terobservasi saat ini: suhu, status→ikon, "terasa seperti" = t+(hu-50)/10, UV estimasi dari tcc, jarak pandang vs m→km.</t>
+        </is>
+      </c>
+      <c r="I5" s="63" t="inlineStr">
         <is>
           <t>Kartu 'Hari Ini' = kondisi live saat ini; strip 7 hari = slot pertama tiap grup (df-forecast). API tidak punya tmin/tmax &amp; probabilitas hujan → keduanya di-skip (badge % = tp×20, aproksimasi).</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="153" customHeight="1">
+    <row r="6" ht="331.5" customHeight="1">
       <c r="A6" s="58" t="n">
         <v>2</v>
       </c>
@@ -6374,10 +6391,29 @@
       </c>
       <c r="G6" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173, … (dipotong)</t>
-        </is>
-      </c>
-      <c r="H6" s="63" t="inlineStr">
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"w …
+▸ DF Adm: resolve wilayah admin
+{"adm1":"31","adm2":"31.71","adm3":"31.71.07","adm4":"31.71.07.1005","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Tanah Abang","desa":"Kebon Melati","lon":106.81596823959143,"lat":-6.197052719903746,"distance":0}
+▸ Present Weather: cuaca saat ini
+{"status":200,"data":{"lokasi":{"lon":106.81596823959143,"lat":-6.197052719903746,"adm1":"31","adm2":"31.71","adm3":"31.71.07","adm4":"31.71.07.1005","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Tanah Abang","desa":"Kebon Melati","distance":0},"cuaca":{"weather":4,"weather_desc":"Berawan Tebal","weather_desc_en":"Overcast","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan tebal-am.svg","datetime":"2026-09-22T06:00:00.000Z","local_datetime":"2026-09-22 13:00:00","t":33,"tcc":87,"wd_deg":21,"wd":"N","wd_to":"S","ws":10.2,"hu":46,"vs":null,"vs_text":null} …
+▸ API v1: waktu matahari terbit/terbenam
+{"results":{"date":"2026-09-22","sunrise":"5:42:05 AM","sunset":"5:49:07 PM","first_light":"4:33:02 AM","last_light":"6:58:12 PM","dawn":"5:21:18 AM","dusk":"6:09:54 PM","solar_noon":"11:45:33 AM","golden_hour":"5:21:38 PM","day_length":"12:07:02","nautical_twilight_begin":"4:57:10 AM","nautical_twilight_end":"6:34:03 PM","timezone":"Asia/Jakarta","utc_offset":420,"sun_altitude":83.49,"sun_azimuth":0,"sunrise_azimuth":89.69,"sunset_azimuth":270.12,"moonrise":"2:19:27 PM","moonset":"2:15:11 AM","moon_illumination":80.06,"moon_phase":"Waxing Gibbous","moon_phase_value":0.35,"moon_always_up":fals …</t>
+        </is>
+      </c>
+      <c r="H6" s="59" t="inlineStr">
+        <is>
+          <t>▸ data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ provinsi, kotkab, kecamatan, desa
+  Resolusi koordinat → wilayah administratif; label lokasi kartu.
+▸ data.t, hu, weather_desc, ws, tcc, vs, local_datetime
+  Kondisi terobservasi saat ini: suhu, status→ikon, "terasa seperti" = t+(hu-50)/10, UV estimasi dari tcc, jarak pandang vs m→km.
+▸ sunrise, sunset (format 12-jam)
+  Dikonversi ke HH:mm → info matahari terbit/terbenam di CurrentWeather.</t>
+        </is>
+      </c>
+      <c r="I6" s="63" t="inlineStr">
         <is>
           <t>Info matahari (sunset API), wilayah (df/adm).
 – UV: proksi tcc (bukan UV asli) (est)
@@ -6415,16 +6451,27 @@
       </c>
       <c r="G7" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173, … (dipotong)</t>
-        </is>
-      </c>
-      <c r="H7" s="63" t="inlineStr">
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"w …
+▸ Open Data RESMI: prakiraan-cuaca (adm4)
+(tidak ada response live)</t>
+        </is>
+      </c>
+      <c r="H7" s="59" t="inlineStr">
+        <is>
+          <t>▸ data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ data[].cuaca[][] → t, hu, weather_desc, tp
+  Fallback prakiraan resmi (open-data) bila df kosong — bentuk item identik df.</t>
+        </is>
+      </c>
+      <c r="I7" s="63" t="inlineStr">
         <is>
           <t>Tab Suhu = satu suhu per hari (slot pertama, tanpa min/max). Fallback resmi open-data bila df kosong.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="90" customHeight="1">
+    <row r="8" ht="121.5" customHeight="1">
       <c r="A8" s="58" t="n">
         <v>4</v>
       </c>
@@ -6456,10 +6503,25 @@
       </c>
       <c r="G8" s="62" t="inlineStr">
         <is>
-          <t>{"statusCode":200,"message":"OK!","data":{"today":{},"tomorrow":null}}</t>
-        </is>
-      </c>
-      <c r="H8" s="63" t="inlineStr">
+          <t>▸ Public API: peringatan cuaca
+{"statusCode":200,"message":"OK!","data":{"today":{},"tomorrow":null}}
+▸ Public API: peringatan siklon
+(tidak ada response live)
+▸ Peringatan Dini Nowcast (RSS resmi)
+(tidak ada response live)</t>
+        </is>
+      </c>
+      <c r="H8" s="59" t="inlineStr">
+        <is>
+          <t>▸ data.today / data.tomorrow (warning_level, impact/description)
+  Peringatan hari ini/besok → severity Awas/Siaga/Waspada → AlertsPanel; kosong = tanpa peringatan.
+▸ data siklon terdampak
+  Peringatan siklon untuk wilayah — hanya muncul saat ada siklon aktif.
+▸ XML RSS: &lt;item&gt; per provinsi (title, description, pubDate)
+  Peringatan dini 3-6 jam resmi; difilter per provinsi; menang atas warning internal df.</t>
+        </is>
+      </c>
+      <c r="I8" s="63" t="inlineStr">
         <is>
           <t>Nowcast (resmi, per provinsi) menang atas warning internal. Cyclone terdampak jarang (hanya saat ada siklon).</t>
         </is>
@@ -6495,10 +6557,21 @@
       </c>
       <c r="G9" s="62" t="inlineStr">
         <is>
-          <t>[{"title":"Prakiraan Cuaca Esok Hari, Selasa, 22 September 2026.","videoUrl":"https://www.youtube.com/watch?v=l6NWtkthnzU"},{"title":"Prakiraan Cuaca Esok Hari, Senin, 21 September 2026.","videoUrl":"https://www.youtube.com/watch?v=GNIhEbJS8q4"},{"title":"Prakiraan Cuaca Esok Hari, Minggu, 20 September 2026","videoUrl":"https://www.youtube.com/watch?v=kCepZRm8uIQ"},{"title":"Prakiraan Cuaca Esok Hari, Sabtu, 19 September 2026.","videoUrl":"https://www.youtube.com/watch?v=9egb1zLG0PM"},{"title":"Prakiraan Cuaca Esok Hari, Jumat, 18 September 2026.","videoUrl":"https://www.youtube.com/watch?v=1Dy6sPbtzpc"},{"title":"Prakiraan Cuaca Esok Hari Kamis, 17 September 2026","videoUrl":"https://www.youtube.com/watch?v=Xx3Ddki3bHk"}]</t>
-        </is>
-      </c>
-      <c r="H9" s="63" t="inlineStr">
+          <t>▸ Berita WordPress BMKG (WP REST)
+(tidak ada response live)
+▸ Public API: video berita
+[{"title":"Prakiraan Cuaca Esok Hari, Selasa, 22 September 2026.","videoUrl":"https://www.youtube.com/watch?v=l6NWtkthnzU"},{"title":"Prakiraan Cuaca Esok Hari, Senin, 21 September 2026.","videoUrl":"https://www.youtube.com/watch?v=GNIhEbJS8q4"},{"title":"Prakiraan Cuaca Esok Hari, Minggu, 20 September 2026","videoUrl":"https://www.youtube.com/watch?v=kCepZRm8uIQ"},{"title":"Prakiraan Cuaca Esok Hari, Sabtu, 19 September 2026.","videoUrl":"https://www.youtube.com/watch?v=9egb1zLG0PM"},{"title":"Prakiraan Cuaca Esok Hari, Jumat, 18 September 2026.","videoUrl":"https://www.youtube.com/watch?v=1 …</t>
+        </is>
+      </c>
+      <c r="H9" s="59" t="inlineStr">
+        <is>
+          <t>▸ [].title.rendered, excerpt.rendered, link, _embedded (featured media)
+  Artikel berita WP → NewsSection; fallback mock saat upstream 502 (sering).
+▸ [].judul, video_url
+  Video berita terbaru (per hashtag) → tab video NewsSection.</t>
+        </is>
+      </c>
+      <c r="I9" s="63" t="inlineStr">
         <is>
           <t>– Fallback: artikel mock saat WP 502 (sering) (mock)</t>
         </is>
@@ -6532,10 +6605,17 @@
       </c>
       <c r="G10" s="62" t="inlineStr">
         <is>
-          <t>{"Infogempa":{"gempa":[{"Tanggal":"22 Sep 2026","Jam":"10:36:27 WIB","DateTime":"2026-09-22T03:36:27+00:00","Coordinates":"-8.43,121.44","Lintang":"8.43 LS","Bujur":"121.44 BT","Magnitude":"4.8","Kedalaman":"14 km","Wilayah":"Pusat gempa berada di laut 31 km timur laut Mbay, Nagekeo","Dirasakan":"IV Kab. Nagekeo, III Kab. Ngada, III Kab. Sikka, III Kab. Ende, II Kab. Manggarai"},{"Tanggal":"21 Sep 2026","Jam":"19:35:22 WIB","DateTime":"2026-09-21T12:35:22+00:00","Coordinates":"-0.52,99.37","Lintang":"0.52 LS","Bujur":"99.37 BT","Magnitude":"4.5","Kedalaman":"10 km","Wilayah":"Pusat gempa berada di laut 76 km Barat Daya Agam","Dirasakan":"III-IV Agam, II-III Kab. Padang Pariaman, II-III Kota Pariaman, II-III Kota Padang"},{"Tanggal":"21 Sep 2026","Jam":"14:31:07 WIB","DateTime":"2026-09-21T07:31:07+00:00","Coordinates":"-0.70,122.45","Lintang":"0.70 LS","Bujur":"122.45 BT","Magnitude":"5.3","Kedalaman":"10 km","Wilayah":"Pusat gempa berada di laut 26 km BaratDaya Pulau Puah","Dirasakan":"IV-V Luwuk, II-III Kab. Pohuwato"},{"Tanggal":"21 Sep 2026","Jam":"12:59:25 WIB","DateTime":"2026-09-21T05:59:25+00:00","Coordinates":"-8.28,120.57","Lintang":"8.28 LS","Bujur":"120.57 BT","Magnitude":"3.5","Kedalaman":"7 km","Wilayah":"Pusat gempa berada di laut 38 km utara Ruteng, Manggarai","Dirasakan":"II-III Manggarai"},{"Tanggal":"21 Sep 2026","Jam":"08:41:37 WIB","DateTime":"2026-09-21T01:41:37+00:00","Coordinates":"-8.33,120.59","Lintang":"8.33 LS","Bujur":"120.59 BT","Magnitude":"5.3" … (dipotong)</t>
-        </is>
-      </c>
-      <c r="H10" s="63" t="inlineStr">
+          <t>▸ Open Data: gempa (TEWS)
+{"Infogempa":{"gempa":[{"Tanggal":"22 Sep 2026","Jam":"10:36:27 WIB","DateTime":"2026-09-22T03:36:27+00:00","Coordinates":"-8.43,121.44","Lintang":"8.43 LS","Bujur":"121.44 BT","Magnitude":"4.8","Kedalaman":"14 km","Wilayah":"Pusat gempa berada di laut 31 km timur laut Mbay, Nagekeo","Dirasakan":"IV Kab. Nagekeo, III Kab. Ngada, III Kab. Sikka, III Kab. Ende, II Kab. Manggarai"},{"Tanggal":"21 Sep 2026","Jam":"19:35:22 WIB","DateTime":"2026-09-21T12:35:22+00:00","Coordinates":"-0.52,99.37","Lintang":"0.52 LS","Bujur":"99.37 BT","Magnitude":"4.5","Kedalaman":"10 km","Wilayah":"Pusat gempa berad …</t>
+        </is>
+      </c>
+      <c r="H10" s="59" t="inlineStr">
+        <is>
+          <t>▸ features[].properties (magnitude, kedalaman, wilayah, waktu)
+  Autogempa terkini + gempa dirasakan → EarthquakePanel.</t>
+        </is>
+      </c>
+      <c r="I10" s="63" t="inlineStr">
         <is>
           <t>autogempa + gempadirasakan, 2 endpoint TEWS.</t>
         </is>
@@ -6569,10 +6649,17 @@
       </c>
       <c r="G11" s="62" t="inlineStr">
         <is>
-          <t>— (tidak ada response live)</t>
-        </is>
-      </c>
-      <c r="H11" s="63" t="inlineStr">
+          <t>▸ Citra Satelit Himawari-9 (background-image, bukan fetch)
+(tidak ada response live)</t>
+        </is>
+      </c>
+      <c r="H11" s="59" t="inlineStr">
+        <is>
+          <t>▸ (PNG) inderaja.bmkg.go.id H08_*.png
+  Citra Himawari-9 → background panel satelit (bukan JSON; terekam sebagai request gambar).</t>
+        </is>
+      </c>
+      <c r="I11" s="63" t="inlineStr">
         <is>
           <t>Gambar PNG inderaja.bmkg.go.id (background-image &lt;img&gt; → TIDAK terekam patch fetch).</t>
         </is>
@@ -6609,7 +6696,12 @@
           <t>— (tidak ada response live)</t>
         </is>
       </c>
-      <c r="H12" s="63" t="inlineStr">
+      <c r="H12" s="59" t="inlineStr">
+        <is>
+          <t>— (kartu tanpa API live — 100% statis)</t>
+        </is>
+      </c>
+      <c r="I12" s="63" t="inlineStr">
         <is>
           <t>– Kartu statis: landmark + nama kota (auto-geser &amp; fetch sengaja dimatikan, 16 Sep) (mock)</t>
         </is>
@@ -6647,10 +6739,25 @@
       </c>
       <c r="G13" s="62" t="inlineStr">
         <is>
-          <t>[["","Kota Jakarta Pusat","Menteng ",-6.19809917164,106.84108701,"5005610","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.149180001,106.827000026,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.141079981,106.822740007,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Pusat","Senen ",-6.193899969,106.856519999,"5005611","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Pusat","Kemayoran ",-6.174619999,106.844179993,"5005614","2026-09-10 16:00:00",["83","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Barat","Cengkareng ",-6.158600003,106.756496988,"5005623","2026-09-10 16:00:00",["82","26","2","E","0.5"],"ndf"],["","Kota Tangerang","Batuceper",-6.169660008,106.681367978,"5008776","2026-09-10 16:00:00",["85","26","2","SE","2.4"],"ndf"],["","Kota Jakarta Barat","Grogol Petamburan ",-6.161280032,106.772031002,"5005620","2026-09-10 16:00:00",["82","26","2","E","0.5"],"ndf"],["","Kota Jakarta Barat","Tambora",-6.155889966,106.801510993,"5005621","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Timur","Jakarta Timur",-6.212939965,106.900340002,"501191","2026-09-10 16:00:00",["88","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Selatan","Tebet ",-6.225910038,106.858320013,"5005597","2026-09-10 16:00:00",["87","26","2","SE","2.5"],"ndf"],["","Kab. Karawang","Kotabaru",-6.406120034,107.458950011,"5009561" … (dipotong)</t>
-        </is>
-      </c>
-      <c r="H13" s="63" t="inlineStr">
+          <t>▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+[["","Kota Jakarta Pusat","Menteng ",-6.19809917164,106.84108701,"5005610","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.149180001,106.827000026,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.141079981,106.822740007,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Pusat","Senen ",-6.193899969,106.856519999,"5005611","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Pusat","Kemayoran ",-6.174619999,106.844179993,"5005614","2026-0 …
+▸ ISDP v1: wilayah laut terdekat
+{"statusCode":200,"message":"OK!","data":{"code":"F.09","name":"Teluk Jakarta","wilpel":"Stamar Tanjung Priok - Jakarta","geometry":{"type":"Polygon","coordinates":[[[106.68448229697637,-6.015114864033774],[106.68448229697637,-5.910111585789263],[107.03498697202032,-5.910111585789263],[106.99055680194432,-5.931987268756869],[107.01030354420033,-5.940737541943912],[107.02017691532832,-5.960425656614758],[107.01030354420033,-5.984488907879126],[106.98562011638033,-6.004177022549971],[106.99055680194432,-6.023865137220817],[107.02017691532832,-6.03480297870462],[107.02017691532832,-6.078554344639 …
+▸ Maritim: detail cuaca/gelombang perairan
+{"code": "F.09", "name": "Teluk Jakarta", "issued": "2026-09-21 23:39 UTC", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "data": [{"valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "time_desc": "Hari ini", "weather": "Berawan", "weather_desc": "Hari ini untuk Teluk Jakarta diperkirakan berawan, dengan kecepatan angin pada umumnya 5 - 18 knot bertiup dari arah selatan, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": …</t>
+        </is>
+      </c>
+      <c r="H13" s="59" t="inlineStr">
+        <is>
+          <t>▸ rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
+  Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.
+▸ code / nama wilayah laut terdekat
+  Anchor koordinat → wilayah perairan/pelabuhan resmi terdekat.
+▸ data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
+  Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.</t>
+        </is>
+      </c>
+      <c r="I13" s="63" t="inlineStr">
         <is>
           <t>– Jalan Raya: DWT kecamatan terdekat (live)
 – Kereta: DWT stasiun terdekat (178 stasiun) (live)
@@ -6691,10 +6798,25 @@
       </c>
       <c r="G14" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173, … (dipotong)</t>
-        </is>
-      </c>
-      <c r="H14" s="63" t="inlineStr">
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"w …
+▸ ISDP v1: wilayah laut terdekat
+{"statusCode":200,"message":"OK!","data":{"code":"F.09","name":"Teluk Jakarta","wilpel":"Stamar Tanjung Priok - Jakarta","geometry":{"type":"Polygon","coordinates":[[[106.68448229697637,-6.015114864033774],[106.68448229697637,-5.910111585789263],[107.03498697202032,-5.910111585789263],[106.99055680194432,-5.931987268756869],[107.01030354420033,-5.940737541943912],[107.02017691532832,-5.960425656614758],[107.01030354420033,-5.984488907879126],[106.98562011638033,-6.004177022549971],[106.99055680194432,-6.023865137220817],[107.02017691532832,-6.03480297870462],[107.02017691532832,-6.078554344639 …
+▸ Maritim: detail cuaca/gelombang perairan
+{"code": "F.09", "name": "Teluk Jakarta", "issued": "2026-09-21 23:39 UTC", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "data": [{"valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "time_desc": "Hari ini", "weather": "Berawan", "weather_desc": "Hari ini untuk Teluk Jakarta diperkirakan berawan, dengan kecepatan angin pada umumnya 5 - 18 knot bertiup dari arah selatan, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": …</t>
+        </is>
+      </c>
+      <c r="H14" s="59" t="inlineStr">
+        <is>
+          <t>▸ data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ code / nama wilayah laut terdekat
+  Anchor koordinat → wilayah perairan/pelabuhan resmi terdekat.
+▸ data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
+  Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.</t>
+        </is>
+      </c>
+      <c r="I14" s="63" t="inlineStr">
         <is>
           <t>– Aktivitas umum: forecast live (live)
 – Aktivitas pelayaran: gelombang perairan resmi (live)
@@ -6703,7 +6825,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="294.5" customHeight="1">
+    <row r="15" ht="373.5" customHeight="1">
       <c r="A15" s="58" t="n">
         <v>11</v>
       </c>
@@ -6737,10 +6859,29 @@
       </c>
       <c r="G15" s="62" t="inlineStr">
         <is>
-          <t>{"U.04": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "U.02": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "U.01": {"issued": "2026-09-21 23:47 UTC", "today": "Rendah", "tomorrow": "Rendah", "h2": "Rendah", "h3": "Rendah"}, "U.03": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.09": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.05": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.12": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.02": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.08": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Tinggi"}, "B.03": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.07": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Tinggi"}, "B.04": {"issued": "2026-09-21 23:47 UTC", "today": "Sedang", "tomorrow": "Sedang", "h2": "Sedang", "h3": "Sedang"}, "B.06": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Seda … (dipotong)</t>
-        </is>
-      </c>
-      <c r="H15" s="63" t="inlineStr">
+          <t>▸ Maritim: overview tinggi gelombang (232 wilayah)
+{"U.04": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "U.02": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "U.01": {"issued": "2026-09-21 23:47 UTC", "today": "Rendah", "tomorrow": "Rendah", "h2": "Rendah", "h3": "Rendah"}, "U.03": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.09": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.05": {"issu …
+▸ Maritim: polygon 232 wilayah perairan
+{"type":"FeatureCollection", "features": [ {"type":"Feature","geometry":{"type":"Polygon","coordinates":[[[106.16613031275644,-7.474222917973128],[106.15132025606444,-7.500473737534255],[106.15132025606444,-9.884923181003366],[105.85018243666048,-9.753669083197725],[104.9517056640126,-9.504286297367011],[104.1717093449007,-9.287717035987708],[103.32259942789281,-9.055834796531078],[102.82399418592888,-8.915830425538395],[102.41424928411693,-8.808639578997123],[102.39943922742495,-8.808639578997123],[105.08005948867658,-6.920768138892684],[105.12942634431657,-6.973269778014939],[105.42562747815 …
+▸ Maritim: detail cuaca/gelombang perairan
+{"code": "F.09", "name": "Teluk Jakarta", "issued": "2026-09-21 23:39 UTC", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "data": [{"valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "time_desc": "Hari ini", "weather": "Berawan", "weather_desc": "Hari ini untuk Teluk Jakarta diperkirakan berawan, dengan kecepatan angin pada umumnya 5 - 18 knot bertiup dari arah selatan, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": …
+▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+[["","Kota Jakarta Pusat","Menteng ",-6.19809917164,106.84108701,"5005610","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.149180001,106.827000026,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.141079981,106.822740007,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Pusat","Senen ",-6.193899969,106.856519999,"5005611","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Pusat","Kemayoran ",-6.174619999,106.844179993,"5005614","2026-0 …</t>
+        </is>
+      </c>
+      <c r="H15" s="59" t="inlineStr">
+        <is>
+          <t>▸ {code: issued, today, tomorrow, wave_desc}
+  Ringkasan 232 wilayah → warna peta laut + legend gelombang.
+▸ features[].geometry (polygon 232 wilayah)
+  Polygon GeoJSON → layer batas wilayah perairan di peta.
+▸ data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
+  Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.
+▸ rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
+  Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.</t>
+        </is>
+      </c>
+      <c r="I15" s="63" t="inlineStr">
         <is>
           <t>– Gelombang: 232 wilayah resmi (warna/legend live), klik → detail live (live)
 – Layer angin/cuaca: SNAPSHOT statis (sectors.json) (mock)
@@ -6778,16 +6919,27 @@
       </c>
       <c r="G16" s="62" t="inlineStr">
         <is>
-          <t>{ "files": [ { "coor": [ 1.198331, 109.054462 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1720, "name": "0088_Sintete.json", "portname": "Sintete", "type": "utama" }, { "coor": [ 0.00214, 109.285391 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1713, "name": "0310_PPP Sungai Rengas.json", "portname": "PPP Sungai Rengas", "type": "utama" }, { "coor": [ -2.531535, 110.21588 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1692, "name": "0092_Kendawangan.json", "portname": "Kendawangan", "type": "utama" }, { "coor": [ 4.145037, 117.665883 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1679, "name": "0237_Nunukan.json", "portname": "Nunukan", "type": "utama" }, { "coor": [ -8.6679806, 115.261925 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1646, "name": "0603_Sanur.json", "portname": "Sanur", "type": "utama" }, { "coor": [ -5.35863269, 105.81975796 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1670, "name": "0325_PPP Labuhan Maringgai.json", "portname": "PPP Labuhan Maringgai", "type": "utama" }, { "coor": [ -8.67206, 115.55675 ], "file_date": "2026-09- … (dipotong)</t>
-        </is>
-      </c>
-      <c r="H16" s="63" t="inlineStr">
+          <t>▸ Maritim: daftar pelabuhan (294)
+{ "files": [ { "coor": [ 1.198331, 109.054462 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1720, "name": "0088_Sintete.json", "portname": "Sintete", "type": "utama" }, { "coor": [ 0.00214, 109.285391 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1713, "name": "0310_PPP Sungai Rengas.json", "portname": "PPP Sungai Rengas", "type": "utama" }, { "coor": [ -2.531535, 110.21588 ], "file_date": "2026-09-21 23:47 UTC", "kb": …
+▸ Maritim: detail pelabuhan + pasut
+{"port_id": "0101", "name": "Sunda Kelapa", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "latitude": -6.11664888, "longitude": 106.80830956, "type": "utama", "data": [{"issued": "2026-09-21 23:47 UTC", "valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "weather": "Berawan", "weather_desc": "Untuk area Sunda Kelapa diperkirakan berawan, dengan kecepatan angin pada umumnya 2 - 14 knot bertiup dari arah timur", "warning_desc": "NIL", "wind_from": "Timur", "wind_to": "Utara", "wind_speed_min": 2, "wind_speed_max": 1 …</t>
+        </is>
+      </c>
+      <c r="H16" s="59" t="inlineStr">
+        <is>
+          <t>▸ files[].coor, file
+  Koordinat 294 pelabuhan → pilih terdekat → fetch detail.
+▸ detail pelabuhan + data pasut
+  Pasut (UTC → zona waktu pelabuhan) → PortTideCard; pasut null → blok disembunyikan.</t>
+        </is>
+      </c>
+      <c r="I16" s="63" t="inlineStr">
         <is>
           <t>Pasut null di sebagian pelabuhan → blok disembunyikan. Kolom arus di-skip (satuan ambigu).</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="153" customHeight="1">
+    <row r="17" ht="126.5" customHeight="1">
       <c r="A17" s="58" t="n">
         <v>13</v>
       </c>
@@ -6817,17 +6969,28 @@
       </c>
       <c r="G17" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173, … (dipotong)</t>
-        </is>
-      </c>
-      <c r="H17" s="63" t="inlineStr">
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"w …
+▸ Overpass API: POI OpenStreetMap
+(tidak ada response live)</t>
+        </is>
+      </c>
+      <c r="H17" s="59" t="inlineStr">
+        <is>
+          <t>▸ data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ elements[].lat/lon/tags
+  POI OpenStreetMap sekitar pengguna → AroundActivity.</t>
+        </is>
+      </c>
+      <c r="I17" s="63" t="inlineStr">
         <is>
           <t>Nilai cuaca per titik POI live (1 request df/coord per POI).
 – Daftar POI: kurasi statis (cityLandmarks) (mock)</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="271.25" customHeight="1">
+    <row r="18" ht="279" customHeight="1">
       <c r="A18" s="58" t="n">
         <v>14</v>
       </c>
@@ -6863,10 +7026,33 @@
       </c>
       <c r="G18" s="62" t="inlineStr">
         <is>
-          <t>{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":49,"vs":null,"vs_text":null,"time_index":"6-7","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah-am.svg","utc_datetime":"2026-09-22 07:00:00","local_datetime":"2026-09-22 14:00:00"},{"datetime":"2026-09-22T08:00:00Z","t":29,"tcc":60,"tp":0,"weather":2,"weather_desc":"Cerah Berawan","weather_desc_en":"Partly Cloudy","wd_deg":173,"wd":"SE","wd_to":"NW","ws":14.4,"hu":56,"vs":null,"vs_text":null,"time_index":"7-8","analysis_date":"2026-09-22T00:00:00","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/cerah berawan-am.svg","utc_datetime":"2026-09-22 08:00:00","local_datetime":"2026-09-22 15:00:00"},{"datetime":"2026-09-22T09:00:00Z","t":27,"tcc":52,"tp":0,"weather":1,"weather_desc":"Cerah","weather_desc_en":"Sunny","wd_deg":173, … (dipotong)</t>
-        </is>
-      </c>
-      <c r="H18" s="63" t="inlineStr">
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"w …
+▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+[["","Kota Jakarta Pusat","Menteng ",-6.19809917164,106.84108701,"5005610","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.149180001,106.827000026,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.141079981,106.822740007,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Pusat","Senen ",-6.193899969,106.856519999,"5005611","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Pusat","Kemayoran ",-6.174619999,106.844179993,"5005614","2026-0 …
+▸ Overpass API: POI OpenStreetMap
+(tidak ada response live)
+▸ Nominatim: geocode OSM
+(tidak ada response live)
+▸ OSRM: routing
+(tidak ada response live)</t>
+        </is>
+      </c>
+      <c r="H18" s="59" t="inlineStr">
+        <is>
+          <t>▸ data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
+  Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.
+▸ elements[].lat/lon/tags
+  POI OpenStreetMap sekitar pengguna → AroundActivity.
+▸ [].lat/lon/display_name
+  Geocode nama tempat → koordinat.
+▸ routes[].geometry, duration, distance
+  Rute antar titik → panel aktivitas darat.</t>
+        </is>
+      </c>
+      <c r="I18" s="63" t="inlineStr">
         <is>
           <t>Forecast per titik rute live; fallback mock saat API gagal.
 – Pilihan lokasi awal: daftar statis (mock)</t>
@@ -6903,10 +7089,21 @@
       </c>
       <c r="G19" s="62" t="inlineStr">
         <is>
-          <t>{"statusCode":200,"message":"OK!","data":{"code":"F.09","name":"Teluk Jakarta","wilpel":"Stamar Tanjung Priok - Jakarta","geometry":{"type":"Polygon","coordinates":[[[106.68448229697637,-6.015114864033774],[106.68448229697637,-5.910111585789263],[107.03498697202032,-5.910111585789263],[106.99055680194432,-5.931987268756869],[107.01030354420033,-5.940737541943912],[107.02017691532832,-5.960425656614758],[107.01030354420033,-5.984488907879126],[106.98562011638033,-6.004177022549971],[106.99055680194432,-6.023865137220817],[107.02017691532832,-6.03480297870462],[107.02017691532832,-6.078554344639833],[106.99055680194432,-6.087304617826876],[106.91156983292034,-6.100430027607439],[106.87701303397235,-6.098242459310679],[106.85726629171634,-6.117930573981525],[106.82270949276835,-6.124493278871807],[106.79308937938436,-6.111367869091243],[106.74372252374437,-6.106992732497721],[106.72397578148836,-6.093867322717157],[106.70422903923236,-6.052303525078705],[106.71903909592436,-6.041365683594902],[106.68448229697637,-6.015114864033774]]]},"distance":0.07574819298420225,"coordinate":{"type":"Point","coordinates":[106.83985076208779,-6.019490000627295]},"type":"area"}}</t>
-        </is>
-      </c>
-      <c r="H19" s="63" t="inlineStr">
+          <t>▸ ISDP v1: wilayah laut terdekat
+{"statusCode":200,"message":"OK!","data":{"code":"F.09","name":"Teluk Jakarta","wilpel":"Stamar Tanjung Priok - Jakarta","geometry":{"type":"Polygon","coordinates":[[[106.68448229697637,-6.015114864033774],[106.68448229697637,-5.910111585789263],[107.03498697202032,-5.910111585789263],[106.99055680194432,-5.931987268756869],[107.01030354420033,-5.940737541943912],[107.02017691532832,-5.960425656614758],[107.01030354420033,-5.984488907879126],[106.98562011638033,-6.004177022549971],[106.99055680194432,-6.023865137220817],[107.02017691532832,-6.03480297870462],[107.02017691532832,-6.078554344639 …
+▸ Maritim: detail cuaca/gelombang perairan
+{"code": "F.09", "name": "Teluk Jakarta", "issued": "2026-09-21 23:39 UTC", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "data": [{"valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "time_desc": "Hari ini", "weather": "Berawan", "weather_desc": "Hari ini untuk Teluk Jakarta diperkirakan berawan, dengan kecepatan angin pada umumnya 5 - 18 knot bertiup dari arah selatan, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": …</t>
+        </is>
+      </c>
+      <c r="H19" s="59" t="inlineStr">
+        <is>
+          <t>▸ code / nama wilayah laut terdekat
+  Anchor koordinat → wilayah perairan/pelabuhan resmi terdekat.
+▸ data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
+  Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.</t>
+        </is>
+      </c>
+      <c r="I19" s="63" t="inlineStr">
         <is>
           <t>Parameter gelombang resmi di-inject ke drawer.
 – Sisa konten drawer (jenis aktivitas, tabel): statis maritimeAdvisorData.ts (mock)</t>
@@ -6944,7 +7141,12 @@
           <t>— (tidak ada response live)</t>
         </is>
       </c>
-      <c r="H20" s="63" t="inlineStr">
+      <c r="H20" s="59" t="inlineStr">
+        <is>
+          <t>— (kartu tanpa API live — 100% statis)</t>
+        </is>
+      </c>
+      <c r="I20" s="63" t="inlineStr">
         <is>
           <t>– 100% statis (aviationAdvisorData.ts) — API penerbangan belum ada (mock)</t>
         </is>
@@ -6981,7 +7183,12 @@
           <t>— (tidak ada response live)</t>
         </is>
       </c>
-      <c r="H21" s="63" t="inlineStr">
+      <c r="H21" s="59" t="inlineStr">
+        <is>
+          <t>— (kartu tanpa API live — 100% statis)</t>
+        </is>
+      </c>
+      <c r="I21" s="63" t="inlineStr">
         <is>
           <t>– POI statis (poiSearchData.ts) (mock)</t>
         </is>
@@ -6989,9 +7196,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
docs(xlsx): kolom query/url = URL upstream asli + marker *(proxy) merah
Capture kini decode URL proxy (/api/bmkg/…, path-style dev) → URL upstream
asli per kartu, dengan routing host yang benar (alerts→www., event/DWT→
publik., sisanya→cuaca.) + flag proxied. Builder menampilkan URL asli dan
menambah ' *(proxy)' merah tebal (rich-text openpyxl) pada API yang butuh
proxy/alias untuk ambil response-nya (CORS / header khusus) — API direct
tanpa marker.

Bug timpal: const URL (target deploy) di capture script menimpa global URL
→ new URL() selalu throw → semua masuk catch (proxied:false). Fix via
globalThis.URL + strip prefix api/bmkg sebelum routing host.

Terverifikasi: 14 call proxied ter-decode benar; sheet diregenerasi.
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -1426,7 +1426,7 @@
       <row>13</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4381500" cy="16716375"/>
+    <ext cx="4381500" cy="15887700"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -6249,7 +6249,7 @@
     <row r="2">
       <c r="A2" s="55" t="inlineStr">
         <is>
-          <t>Screenshot diambil dari deployment prod (server.mjs + dist, data live) dengan API BOX MARKER aktif — border merah = live, amber = campuran, abu = mock (lihat kolom Status). Kolom "Field dipakai UI" = pemetaan response → nilai yang dirender (sumber: src/services/bmkg/adapters.ts). Sumber screenshot: docs/screenshots/cards/ · skrip: docs/scrapping_cuaca-bmkg-go-id/capture_card_screenshots.js</t>
+          <t>Screenshot diambil dari deployment prod (server.mjs + dist, data live) dengan API BOX MARKER aktif — border merah = live, amber = campuran, abu = mock (lihat kolom Status). Kolom "Field dipakai UI" = pemetaan response → nilai yang dirender (sumber: src/services/bmkg/adapters.ts). *(proxy) merah = API tidak bisa diakses langsung dari browser (CORS / header khusus) — harus lewat proxy/alias untuk ambil response-nya. Sumber screenshot: docs/screenshots/cards/ · skrip: docs/scrapping_cuaca-bmkg-go-id/capture_card_screenshots.js</t>
         </is>
       </c>
     </row>
@@ -6331,16 +6331,41 @@
       </c>
       <c r="F5" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-7.8385&amp;lon=110.3275
-[200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666</t>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666</t>
+          </r>
         </is>
       </c>
       <c r="G5" s="62" t="inlineStr">
         <is>
           <t>▸ DF Forecast: prakiraan 10 hari + per jam
-{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"w …
+{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.82670735619568,"lat":-6.176384269281675,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.8267073562,"lat":-6.1763842693,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T09:00:00Z","t":28,"tcc":90,"tp":0,"weathe …
 ▸ Present Weather: cuaca saat ini
-{"status":200,"data":{"lokasi":{"lon":106.81596823959143,"lat":-6.197052719903746,"adm1":"31","adm2":"31.71","adm3":"31.71.07","adm4":"31.71.07.1005","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Tanah Abang","desa":"Kebon Melati","distance":0},"cuaca":{"weather":4,"weather_desc":"Berawan Tebal","weather_desc_en":"Overcast","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan tebal-am.svg","datetime":"2026-09-22T06:00:00.000Z","local_datetime":"2026-09-22 13:00:00","t":33,"tcc":87,"wd_deg":21,"wd":"N","wd_to":"S","ws":10.2,"hu":46,"vs":null,"vs_text":null} …</t>
+{"status":200,"data":{"lokasi":{"lon":106.81596823959143,"lat":-6.197052719903746,"adm1":"31","adm2":"31.71","adm3":"31.71.07","adm4":"31.71.07.1005","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Tanah Abang","desa":"Kebon Melati","distance":0},"cuaca":{"weather":4,"weather_desc":"Berawan Tebal","weather_desc_en":"Overcast","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan tebal-am.svg","datetime":"2026-09-22T08:20:00.000Z","local_datetime":"2026-09-22 15:20:00","t":29,"tcc":89,"wd_deg":275,"wd":"W","wd_to":"E","ws":6.5,"hu":67,"vs":null,"vs_text":null} …</t>
         </is>
       </c>
       <c r="H5" s="59" t="inlineStr">
@@ -6383,22 +6408,76 @@
       </c>
       <c r="F6" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-7.8385&amp;lon=110.3275
-[200] /api-bmkgapi/df/v1/adm/coord&amp;lat=-6.2&amp;lon=106.816666
-[200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666
-[200] https://cuaca.bmkg.go.id/api/v1/sunset/json?lat=-6.2&amp;lng=106.816666</t>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/df/v1/adm/coord?lat=-6.2&amp;lon=106.816666</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/v1/sunset/json?lat=-6.2&amp;lng=106.816666</t>
+          </r>
         </is>
       </c>
       <c r="G6" s="62" t="inlineStr">
         <is>
           <t>▸ DF Forecast: prakiraan 10 hari + per jam
-{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"w …
+{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.82670735619568,"lat":-6.176384269281675,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.8267073562,"lat":-6.1763842693,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T09:00:00Z","t":28,"tcc":90,"tp":0,"weathe …
 ▸ DF Adm: resolve wilayah admin
 {"adm1":"31","adm2":"31.71","adm3":"31.71.07","adm4":"31.71.07.1005","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Tanah Abang","desa":"Kebon Melati","lon":106.81596823959143,"lat":-6.197052719903746,"distance":0}
 ▸ Present Weather: cuaca saat ini
-{"status":200,"data":{"lokasi":{"lon":106.81596823959143,"lat":-6.197052719903746,"adm1":"31","adm2":"31.71","adm3":"31.71.07","adm4":"31.71.07.1005","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Tanah Abang","desa":"Kebon Melati","distance":0},"cuaca":{"weather":4,"weather_desc":"Berawan Tebal","weather_desc_en":"Overcast","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan tebal-am.svg","datetime":"2026-09-22T06:00:00.000Z","local_datetime":"2026-09-22 13:00:00","t":33,"tcc":87,"wd_deg":21,"wd":"N","wd_to":"S","ws":10.2,"hu":46,"vs":null,"vs_text":null} …
+{"status":200,"data":{"lokasi":{"lon":106.81596823959143,"lat":-6.197052719903746,"adm1":"31","adm2":"31.71","adm3":"31.71.07","adm4":"31.71.07.1005","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Tanah Abang","desa":"Kebon Melati","distance":0},"cuaca":{"weather":4,"weather_desc":"Berawan Tebal","weather_desc_en":"Overcast","image":"https://api-apps.bmkg.go.id/storage/icon/cuaca/berawan tebal-am.svg","datetime":"2026-09-22T08:20:00.000Z","local_datetime":"2026-09-22 15:20:00","t":29,"tcc":89,"wd_deg":275,"wd":"W","wd_to":"E","ws":6.5,"hu":67,"vs":null,"vs_text":null} …
 ▸ API v1: waktu matahari terbit/terbenam
-{"results":{"date":"2026-09-22","sunrise":"5:42:05 AM","sunset":"5:49:07 PM","first_light":"4:33:02 AM","last_light":"6:58:12 PM","dawn":"5:21:18 AM","dusk":"6:09:54 PM","solar_noon":"11:45:33 AM","golden_hour":"5:21:38 PM","day_length":"12:07:02","nautical_twilight_begin":"4:57:10 AM","nautical_twilight_end":"6:34:03 PM","timezone":"Asia/Jakarta","utc_offset":420,"sun_altitude":83.49,"sun_azimuth":0,"sunrise_azimuth":89.69,"sunset_azimuth":270.12,"moonrise":"2:19:27 PM","moonset":"2:15:11 AM","moon_illumination":80.06,"moon_phase":"Waxing Gibbous","moon_phase_value":0.35,"moon_always_up":fals …</t>
+{"results":{"date":"2026-09-22","sunrise":"5:42:05 AM","sunset":"5:49:07 PM","first_light":"4:33:02 AM","last_light":"6:58:12 PM","dawn":"5:21:18 AM","dusk":"6:09:54 PM","solar_noon":"11:45:33 AM","golden_hour":"5:21:38 PM","day_length":"12:07:02","nautical_twilight_begin":"4:57:10 AM","nautical_twilight_end":"6:34:03 PM","timezone":"Asia/Jakarta","utc_offset":420,"sun_altitude":83.49,"sun_azimuth":0,"sunrise_azimuth":89.69,"sunset_azimuth":270.12,"moonrise":"2:19:27 PM","moonset":"2:15:11 AM","moon_illumination":81.03,"moon_phase":"Waxing Gibbous","moon_phase_value":0.36,"moon_always_up":fals …</t>
         </is>
       </c>
       <c r="H6" s="59" t="inlineStr">
@@ -6445,14 +6524,39 @@
       </c>
       <c r="F7" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-7.8385&amp;lon=110.3275
-(belum terekam saat capture) — Open Data RESMI: prakiraan-cuaca (adm4)</t>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>(belum terekam saat capture) — Open Data RESMI: prakiraan-cuaca (adm4)</t>
+          </r>
         </is>
       </c>
       <c r="G7" s="62" t="inlineStr">
         <is>
           <t>▸ DF Forecast: prakiraan 10 hari + per jam
-{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"w …
+{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.82670735619568,"lat":-6.176384269281675,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.8267073562,"lat":-6.1763842693,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T09:00:00Z","t":28,"tcc":90,"tp":0,"weathe …
 ▸ Open Data RESMI: prakiraan-cuaca (adm4)
 (tidak ada response live)</t>
         </is>
@@ -6471,7 +6575,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="121.5" customHeight="1">
+    <row r="8" ht="142.5" customHeight="1">
       <c r="A8" s="58" t="n">
         <v>4</v>
       </c>
@@ -6496,9 +6600,53 @@
       </c>
       <c r="F8" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgapi/public/weather/warning&amp;lat=-6.2&amp;long=106.816666
-(belum terekam saat capture) — Public API: peringatan siklon
-(belum terekam saat capture) — Peringatan Dini Nowcast (RSS resmi)</t>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/public/weather/warning?lat=-6.2&amp;long=106.816666</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>(belum terekam saat capture) — Public API: peringatan siklon</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://www.bmkg.go.id/alerts/nowcast/id</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
         </is>
       </c>
       <c r="G8" s="62" t="inlineStr">
@@ -6508,7 +6656,7 @@
 ▸ Public API: peringatan siklon
 (tidak ada response live)
 ▸ Peringatan Dini Nowcast (RSS resmi)
-(tidak ada response live)</t>
+&lt;?xml version="1.0" encoding="UTF-8"?&gt; &lt;?xml-stylesheet type="text/xsl" href="/cap/nowcast-rss-style.xsl"?&gt; &lt;rss version="2.0" xmlns:atom="http://www.w3.org/2005/Atom"&gt; &lt;channel&gt; &lt;title&gt;Peringatan Dini Cuaca BMKG&lt;/title&gt; &lt;link&gt;https://www.bmkg.go.id/alerts/nowcast/id/rss.xml&lt;/link&gt; &lt;description&gt;Peringatan Dini Cuaca dari BMKG (Badan Meteorologi, Klimatologi, dan Geofisika)&lt;/description&gt; &lt;atom:link href="https://www.bmkg.go.id/alerts/nowcast/id/rss.xml" rel="self" type="application/rss+xml"/&gt; &lt;language&gt;id&lt;/language&gt; …</t>
         </is>
       </c>
       <c r="H8" s="59" t="inlineStr">
@@ -6551,14 +6699,48 @@
       </c>
       <c r="F9" s="62" t="inlineStr">
         <is>
-          <t>(belum terekam saat capture) — Berita WordPress BMKG (WP REST)
-[200] /api-bmkgapi/public/weather/video-latest&amp;hashtag=infobmkgpws</t>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[502] https://cuaca.bmkg.go.id/blog/wp-json/wp/v2/posts?per_page=4&amp;_embed=1</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/public/weather/video-latest?hashtag=infobmkgpws</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
         </is>
       </c>
       <c r="G9" s="62" t="inlineStr">
         <is>
           <t>▸ Berita WordPress BMKG (WP REST)
-(tidak ada response live)
+{"type":"https://developers.cloudflare.com/support/troubleshooting/http-status-codes/cloudflare-5xx-errors/error-502/","title":"Error 502: Bad gateway","status":502,"detail":"The origin web server returned an invalid or incomplete response to Cloudflare. This typically indicates the origin is overloaded or misconfigured.","instance":"a3eff3f4cb3cfd32","error_code":502,"error_name":"origin_bad_gateway","error_category":"origin","ray_id":"a3eff3f4cb3cfd32","timestamp":"2026-09-22T08:31:22Z","zone":"cuaca.bmkg.go.id","cloudflare_error":true,"retryable":true,"retry_after":60,"owner_action_required …
 ▸ Public API: video berita
 [{"title":"Prakiraan Cuaca Esok Hari, Selasa, 22 September 2026.","videoUrl":"https://www.youtube.com/watch?v=l6NWtkthnzU"},{"title":"Prakiraan Cuaca Esok Hari, Senin, 21 September 2026.","videoUrl":"https://www.youtube.com/watch?v=GNIhEbJS8q4"},{"title":"Prakiraan Cuaca Esok Hari, Minggu, 20 September 2026","videoUrl":"https://www.youtube.com/watch?v=kCepZRm8uIQ"},{"title":"Prakiraan Cuaca Esok Hari, Sabtu, 19 September 2026.","videoUrl":"https://www.youtube.com/watch?v=9egb1zLG0PM"},{"title":"Prakiraan Cuaca Esok Hari, Jumat, 18 September 2026.","videoUrl":"https://www.youtube.com/watch?v=1 …</t>
         </is>
@@ -6600,13 +6782,13 @@
       </c>
       <c r="F10" s="62" t="inlineStr">
         <is>
-          <t>[200] https://data.bmkg.go.id/DataMKG/TEWS/gempadirasakan.json</t>
+          <t>(belum terekam saat capture) — Open Data: gempa (TEWS)</t>
         </is>
       </c>
       <c r="G10" s="62" t="inlineStr">
         <is>
           <t>▸ Open Data: gempa (TEWS)
-{"Infogempa":{"gempa":[{"Tanggal":"22 Sep 2026","Jam":"10:36:27 WIB","DateTime":"2026-09-22T03:36:27+00:00","Coordinates":"-8.43,121.44","Lintang":"8.43 LS","Bujur":"121.44 BT","Magnitude":"4.8","Kedalaman":"14 km","Wilayah":"Pusat gempa berada di laut 31 km timur laut Mbay, Nagekeo","Dirasakan":"IV Kab. Nagekeo, III Kab. Ngada, III Kab. Sikka, III Kab. Ende, II Kab. Manggarai"},{"Tanggal":"21 Sep 2026","Jam":"19:35:22 WIB","DateTime":"2026-09-21T12:35:22+00:00","Coordinates":"-0.52,99.37","Lintang":"0.52 LS","Bujur":"99.37 BT","Magnitude":"4.5","Kedalaman":"10 km","Wilayah":"Pusat gempa berad …</t>
+(tidak ada response live)</t>
         </is>
       </c>
       <c r="H10" s="59" t="inlineStr">
@@ -6732,15 +6914,59 @@
       </c>
       <c r="F13" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgevent/source/dwt/apiDF_Kereta/202609101600.json
-[200] /api-bmkgapi/v1/public/maritim/nearest-location&amp;lat=-6.2&amp;long=106.816666
-[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://publik.bmkg.go.id/event/source/dwt/apiDF_Darat/202609101600.json</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location?lat=-6.2&amp;long=106.816666</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+          </r>
         </is>
       </c>
       <c r="G13" s="62" t="inlineStr">
         <is>
           <t>▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
-[["","Kota Jakarta Pusat","Menteng ",-6.19809917164,106.84108701,"5005610","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.149180001,106.827000026,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.141079981,106.822740007,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Pusat","Senen ",-6.193899969,106.856519999,"5005611","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Pusat","Kemayoran ",-6.174619999,106.844179993,"5005614","2026-0 …
+[["lampung","Kab. Lampung Tengah","Terusan Nunyai",-4.699604904679063,105.20665965569867,"5013584","2026-09-10 16:00:00",["78","26","1","SE","9.5"],"ndf"],["lampung","Kab. Lampung Tengah","Seputih Agung",-4.89787745875816,105.05458830281606,"5013578","2026-09-10 16:00:00",["80","26","3","SE","9.2"],"ndf"],["lampung","Kab. Lampung Utara","Kotabumi",-4.846956993233334,104.85804482373453,"501378","2026-09-10 16:00:00",["81","26","1","SE","11.7"],"ndf"],["lampung","Kab. Lampung Utara","Abung Barat",-4.865040896877758,104.69148255332641,"5013612","2026-09-10 16:00:00",["87","24","1","SE","5.5"],"nd …
 ▸ ISDP v1: wilayah laut terdekat
 {"statusCode":200,"message":"OK!","data":{"code":"F.09","name":"Teluk Jakarta","wilpel":"Stamar Tanjung Priok - Jakarta","geometry":{"type":"Polygon","coordinates":[[[106.68448229697637,-6.015114864033774],[106.68448229697637,-5.910111585789263],[107.03498697202032,-5.910111585789263],[106.99055680194432,-5.931987268756869],[107.01030354420033,-5.940737541943912],[107.02017691532832,-5.960425656614758],[107.01030354420033,-5.984488907879126],[106.98562011638033,-6.004177022549971],[106.99055680194432,-6.023865137220817],[107.02017691532832,-6.03480297870462],[107.02017691532832,-6.078554344639 …
 ▸ Maritim: detail cuaca/gelombang perairan
@@ -6791,15 +7017,59 @@
       </c>
       <c r="F14" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-7.8385&amp;lon=110.3275
-[200] /api-bmkgapi/v1/public/maritim/nearest-location&amp;lat=-6.2&amp;long=106.816666
-[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location?lat=-6.2&amp;long=106.816666</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+          </r>
         </is>
       </c>
       <c r="G14" s="62" t="inlineStr">
         <is>
           <t>▸ DF Forecast: prakiraan 10 hari + per jam
-{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"w …
+{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.82670735619568,"lat":-6.176384269281675,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.8267073562,"lat":-6.1763842693,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T09:00:00Z","t":28,"tcc":90,"tp":0,"weathe …
 ▸ ISDP v1: wilayah laut terdekat
 {"statusCode":200,"message":"OK!","data":{"code":"F.09","name":"Teluk Jakarta","wilpel":"Stamar Tanjung Priok - Jakarta","geometry":{"type":"Polygon","coordinates":[[[106.68448229697637,-6.015114864033774],[106.68448229697637,-5.910111585789263],[107.03498697202032,-5.910111585789263],[106.99055680194432,-5.931987268756869],[107.01030354420033,-5.940737541943912],[107.02017691532832,-5.960425656614758],[107.01030354420033,-5.984488907879126],[106.98562011638033,-6.004177022549971],[106.99055680194432,-6.023865137220817],[107.02017691532832,-6.03480297870462],[107.02017691532832,-6.078554344639 …
 ▸ Maritim: detail cuaca/gelombang perairan
@@ -6825,7 +7095,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="373.5" customHeight="1">
+    <row r="15" ht="294.5" customHeight="1">
       <c r="A15" s="58" t="n">
         <v>11</v>
       </c>
@@ -6851,22 +7121,67 @@
       </c>
       <c r="F15" s="62" t="inlineStr">
         <is>
-          <t>[200] https://maritim.bmkg.go.id/public_api/overview/gelombang.json
-[200] https://maritim.bmkg.go.id/public_api/static/wilayah_perairan.json
-[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json
-[200] /api-bmkgevent/source/dwt/apiDF_Kereta/202609101600.json</t>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>(belum terekam saat capture) — Maritim: overview tinggi gelombang (232 wilayah)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>(belum terekam saat capture) — Maritim: polygon 232 wilayah perairan</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://publik.bmkg.go.id/event/source/dwt/apiDF_Darat/202609101600.json</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
         </is>
       </c>
       <c r="G15" s="62" t="inlineStr">
         <is>
           <t>▸ Maritim: overview tinggi gelombang (232 wilayah)
-{"U.04": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "U.02": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "U.01": {"issued": "2026-09-21 23:47 UTC", "today": "Rendah", "tomorrow": "Rendah", "h2": "Rendah", "h3": "Rendah"}, "U.03": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.09": {"issued": "2026-09-21 23:47 UTC", "today": "Tinggi", "tomorrow": "Sedang", "h2": "Tinggi", "h3": "Tinggi"}, "B.05": {"issu …
+(tidak ada response live)
 ▸ Maritim: polygon 232 wilayah perairan
-{"type":"FeatureCollection", "features": [ {"type":"Feature","geometry":{"type":"Polygon","coordinates":[[[106.16613031275644,-7.474222917973128],[106.15132025606444,-7.500473737534255],[106.15132025606444,-9.884923181003366],[105.85018243666048,-9.753669083197725],[104.9517056640126,-9.504286297367011],[104.1717093449007,-9.287717035987708],[103.32259942789281,-9.055834796531078],[102.82399418592888,-8.915830425538395],[102.41424928411693,-8.808639578997123],[102.39943922742495,-8.808639578997123],[105.08005948867658,-6.920768138892684],[105.12942634431657,-6.973269778014939],[105.42562747815 …
+(tidak ada response live)
 ▸ Maritim: detail cuaca/gelombang perairan
 {"code": "F.09", "name": "Teluk Jakarta", "issued": "2026-09-21 23:39 UTC", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "data": [{"valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "time_desc": "Hari ini", "weather": "Berawan", "weather_desc": "Hari ini untuk Teluk Jakarta diperkirakan berawan, dengan kecepatan angin pada umumnya 5 - 18 knot bertiup dari arah selatan, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": …
 ▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
-[["","Kota Jakarta Pusat","Menteng ",-6.19809917164,106.84108701,"5005610","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.149180001,106.827000026,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.141079981,106.822740007,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Pusat","Senen ",-6.193899969,106.856519999,"5005611","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Pusat","Kemayoran ",-6.174619999,106.844179993,"5005614","2026-0 …</t>
+[["lampung","Kab. Lampung Tengah","Terusan Nunyai",-4.699604904679063,105.20665965569867,"5013584","2026-09-10 16:00:00",["78","26","1","SE","9.5"],"ndf"],["lampung","Kab. Lampung Tengah","Seputih Agung",-4.89787745875816,105.05458830281606,"5013578","2026-09-10 16:00:00",["80","26","3","SE","9.2"],"ndf"],["lampung","Kab. Lampung Utara","Kotabumi",-4.846956993233334,104.85804482373453,"501378","2026-09-10 16:00:00",["81","26","1","SE","11.7"],"ndf"],["lampung","Kab. Lampung Utara","Abung Barat",-4.865040896877758,104.69148255332641,"5013612","2026-09-10 16:00:00",["87","24","1","SE","5.5"],"nd …</t>
         </is>
       </c>
       <c r="H15" s="59" t="inlineStr">
@@ -6963,14 +7278,39 @@
       </c>
       <c r="F17" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-7.8385&amp;lon=110.3275
-(belum terekam saat capture) — Overpass API: POI OpenStreetMap</t>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>(belum terekam saat capture) — Overpass API: POI OpenStreetMap</t>
+          </r>
         </is>
       </c>
       <c r="G17" s="62" t="inlineStr">
         <is>
           <t>▸ DF Forecast: prakiraan 10 hari + per jam
-{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"w …
+{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.82670735619568,"lat":-6.176384269281675,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.8267073562,"lat":-6.1763842693,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T09:00:00Z","t":28,"tcc":90,"tp":0,"weathe …
 ▸ Overpass API: POI OpenStreetMap
 (tidak ada response live)</t>
         </is>
@@ -7017,19 +7357,83 @@
       </c>
       <c r="F18" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgapi/df/v1/forecast/coord&amp;lat=-7.8385&amp;lon=110.3275
-[200] /api-bmkgevent/source/dwt/apiDF_Kereta/202609101600.json
-(belum terekam saat capture) — Overpass API: POI OpenStreetMap
-(belum terekam saat capture) — Nominatim: geocode OSM
-(belum terekam saat capture) — OSRM: routing</t>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://publik.bmkg.go.id/event/source/dwt/apiDF_Darat/202609101600.json</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>(belum terekam saat capture) — Overpass API: POI OpenStreetMap</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>(belum terekam saat capture) — Nominatim: geocode OSM</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>(belum terekam saat capture) — OSRM: routing</t>
+          </r>
         </is>
       </c>
       <c r="G18" s="62" t="inlineStr">
         <is>
           <t>▸ DF Forecast: prakiraan 10 hari + per jam
-{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.31087740815543,"lat":-7.841634455002868,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"34","adm2":"34.02","adm3":"34.02.16","adm4":"34.02.16.2001","provinsi":"Daerah Istimewa Yogyakarta","kotkab":"Bantul","kecamatan":"Kasihan","desa":"Bangunjiwo","lon":110.3108774082,"lat":-7.841634455,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T07:00:00Z","t":30,"tcc":39,"tp":0,"w …
+{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.82670735619568,"lat":-6.176384269281675,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.8267073562,"lat":-6.1763842693,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T09:00:00Z","t":28,"tcc":90,"tp":0,"weathe …
 ▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
-[["","Kota Jakarta Pusat","Menteng ",-6.19809917164,106.84108701,"5005610","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.149180001,106.827000026,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Barat","Taman Sari",-6.141079981,106.822740007,"5005622","2026-09-10 16:00:00",["81","26","2","E","0.5"],"ndf"],["","Kota Jakarta Pusat","Senen ",-6.193899969,106.856519999,"5005611","2026-09-10 16:00:00",["85","26","2","SE","2.5"],"ndf"],["","Kota Jakarta Pusat","Kemayoran ",-6.174619999,106.844179993,"5005614","2026-0 …
+[["lampung","Kab. Lampung Tengah","Terusan Nunyai",-4.699604904679063,105.20665965569867,"5013584","2026-09-10 16:00:00",["78","26","1","SE","9.5"],"ndf"],["lampung","Kab. Lampung Tengah","Seputih Agung",-4.89787745875816,105.05458830281606,"5013578","2026-09-10 16:00:00",["80","26","3","SE","9.2"],"ndf"],["lampung","Kab. Lampung Utara","Kotabumi",-4.846956993233334,104.85804482373453,"501378","2026-09-10 16:00:00",["81","26","1","SE","11.7"],"ndf"],["lampung","Kab. Lampung Utara","Abung Barat",-4.865040896877758,104.69148255332641,"5013612","2026-09-10 16:00:00",["87","24","1","SE","5.5"],"nd …
 ▸ Overpass API: POI OpenStreetMap
 (tidak ada response live)
 ▸ Nominatim: geocode OSM
@@ -7083,8 +7487,33 @@
       </c>
       <c r="F19" s="62" t="inlineStr">
         <is>
-          <t>[200] /api-bmkgapi/v1/public/maritim/nearest-location&amp;lat=-6.2&amp;long=106.816666
-[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location?lat=-6.2&amp;long=106.816666</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+          </r>
         </is>
       </c>
       <c r="G19" s="62" t="inlineStr">

</xml_diff>

<commit_message>
style(xlsx): kolom 'API dipakai' pakai bullet ▸ (seragam dgn kolom sample/field)
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -6325,8 +6325,8 @@
       </c>
       <c r="E5" s="59" t="inlineStr">
         <is>
-          <t>• DF Forecast: prakiraan 10 hari + per jam
-• Present Weather: cuaca saat ini</t>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+▸ Present Weather: cuaca saat ini</t>
         </is>
       </c>
       <c r="F5" s="62" t="inlineStr">
@@ -6400,10 +6400,10 @@
       </c>
       <c r="E6" s="59" t="inlineStr">
         <is>
-          <t>• DF Forecast: prakiraan 10 hari + per jam
-• DF Adm: resolve wilayah admin
-• Present Weather: cuaca saat ini
-• API v1: waktu matahari terbit/terbenam</t>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+▸ DF Adm: resolve wilayah admin
+▸ Present Weather: cuaca saat ini
+▸ API v1: waktu matahari terbit/terbenam</t>
         </is>
       </c>
       <c r="F6" s="62" t="inlineStr">
@@ -6518,8 +6518,8 @@
       </c>
       <c r="E7" s="59" t="inlineStr">
         <is>
-          <t>• DF Forecast: prakiraan 10 hari + per jam
-• Open Data RESMI: prakiraan-cuaca (adm4)</t>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+▸ Open Data RESMI: prakiraan-cuaca (adm4)</t>
         </is>
       </c>
       <c r="F7" s="62" t="inlineStr">
@@ -6593,9 +6593,9 @@
       </c>
       <c r="E8" s="59" t="inlineStr">
         <is>
-          <t>• Public API: peringatan cuaca
-• Public API: peringatan siklon
-• Peringatan Dini Nowcast (RSS resmi)</t>
+          <t>▸ Public API: peringatan cuaca
+▸ Public API: peringatan siklon
+▸ Peringatan Dini Nowcast (RSS resmi)</t>
         </is>
       </c>
       <c r="F8" s="62" t="inlineStr">
@@ -6693,8 +6693,8 @@
       </c>
       <c r="E9" s="59" t="inlineStr">
         <is>
-          <t>• Berita WordPress BMKG (WP REST)
-• Public API: video berita</t>
+          <t>▸ Berita WordPress BMKG (WP REST)
+▸ Public API: video berita</t>
         </is>
       </c>
       <c r="F9" s="62" t="inlineStr">
@@ -6777,7 +6777,7 @@
       </c>
       <c r="E10" s="59" t="inlineStr">
         <is>
-          <t>• Open Data: gempa (TEWS)</t>
+          <t>▸ Open Data: gempa (TEWS)</t>
         </is>
       </c>
       <c r="F10" s="62" t="inlineStr">
@@ -6821,7 +6821,7 @@
       </c>
       <c r="E11" s="59" t="inlineStr">
         <is>
-          <t>• Citra Satelit Himawari-9 (background-image, bukan fetch)</t>
+          <t>▸ Citra Satelit Himawari-9 (background-image, bukan fetch)</t>
         </is>
       </c>
       <c r="F11" s="62" t="inlineStr">
@@ -6907,9 +6907,9 @@
       </c>
       <c r="E13" s="59" t="inlineStr">
         <is>
-          <t>• DWT: cuaca kecamatan/stasiun (jalan+kereta)
-• ISDP v1: wilayah laut terdekat
-• Maritim: detail cuaca/gelombang perairan</t>
+          <t>▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+▸ ISDP v1: wilayah laut terdekat
+▸ Maritim: detail cuaca/gelombang perairan</t>
         </is>
       </c>
       <c r="F13" s="62" t="inlineStr">
@@ -7010,9 +7010,9 @@
       </c>
       <c r="E14" s="59" t="inlineStr">
         <is>
-          <t>• DF Forecast: prakiraan 10 hari + per jam
-• ISDP v1: wilayah laut terdekat
-• Maritim: detail cuaca/gelombang perairan</t>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+▸ ISDP v1: wilayah laut terdekat
+▸ Maritim: detail cuaca/gelombang perairan</t>
         </is>
       </c>
       <c r="F14" s="62" t="inlineStr">
@@ -7113,10 +7113,10 @@
       </c>
       <c r="E15" s="59" t="inlineStr">
         <is>
-          <t>• Maritim: overview tinggi gelombang (232 wilayah)
-• Maritim: polygon 232 wilayah perairan
-• Maritim: detail cuaca/gelombang perairan
-• DWT: cuaca kecamatan/stasiun (jalan+kereta)</t>
+          <t>▸ Maritim: overview tinggi gelombang (232 wilayah)
+▸ Maritim: polygon 232 wilayah perairan
+▸ Maritim: detail cuaca/gelombang perairan
+▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)</t>
         </is>
       </c>
       <c r="F15" s="62" t="inlineStr">
@@ -7222,8 +7222,8 @@
       </c>
       <c r="E16" s="59" t="inlineStr">
         <is>
-          <t>• Maritim: daftar pelabuhan (294)
-• Maritim: detail pelabuhan + pasut</t>
+          <t>▸ Maritim: daftar pelabuhan (294)
+▸ Maritim: detail pelabuhan + pasut</t>
         </is>
       </c>
       <c r="F16" s="62" t="inlineStr">
@@ -7272,8 +7272,8 @@
       </c>
       <c r="E17" s="59" t="inlineStr">
         <is>
-          <t>• DF Forecast: prakiraan 10 hari + per jam
-• Overpass API: POI OpenStreetMap</t>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+▸ Overpass API: POI OpenStreetMap</t>
         </is>
       </c>
       <c r="F17" s="62" t="inlineStr">
@@ -7348,11 +7348,11 @@
       </c>
       <c r="E18" s="59" t="inlineStr">
         <is>
-          <t>• DF Forecast: prakiraan 10 hari + per jam
-• DWT: cuaca kecamatan/stasiun (jalan+kereta)
-• Overpass API: POI OpenStreetMap
-• Nominatim: geocode OSM
-• OSRM: routing</t>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+▸ Overpass API: POI OpenStreetMap
+▸ Nominatim: geocode OSM
+▸ OSRM: routing</t>
         </is>
       </c>
       <c r="F18" s="62" t="inlineStr">
@@ -7481,8 +7481,8 @@
       </c>
       <c r="E19" s="59" t="inlineStr">
         <is>
-          <t>• ISDP v1: wilayah laut terdekat
-• Maritim: detail cuaca/gelombang perairan</t>
+          <t>▸ ISDP v1: wilayah laut terdekat
+▸ Maritim: detail cuaca/gelombang perairan</t>
         </is>
       </c>
       <c r="F19" s="62" t="inlineStr">

</xml_diff>

<commit_message>
docs(xlsx): kolom F/H/I lebih jelas
- F 'Query / URL terakhir': tiap baris API pakai bullet ▸ ([status] URL *(proxy))
- H 'Field dipakai UI': per blok sekarang sebut nama API + 'Dipakai:' field
  + '→' penjelasan — mudah dipadankan dengan kolom E/F/G
- I 'Catatan': bullet ▸ + status bahasa eksplisit per komponen
  ('data asli dari API' / 'estimasi/konversi dari API' / 'data statis
  (belum ada endpoint)')
- A2: legend arti live/estimasi/mock + arti marker *(proxy)
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -6249,7 +6249,7 @@
     <row r="2">
       <c r="A2" s="55" t="inlineStr">
         <is>
-          <t>Screenshot diambil dari deployment prod (server.mjs + dist, data live) dengan API BOX MARKER aktif — border merah = live, amber = campuran, abu = mock (lihat kolom Status). Kolom "Field dipakai UI" = pemetaan response → nilai yang dirender (sumber: src/services/bmkg/adapters.ts). *(proxy) merah = API tidak bisa diakses langsung dari browser (CORS / header khusus) — harus lewat proxy/alias untuk ambil response-nya. Sumber screenshot: docs/screenshots/cards/ · skrip: docs/scrapping_cuaca-bmkg-go-id/capture_card_screenshots.js</t>
+          <t>Screenshot diambil dari deployment prod (server.mjs + dist, data live) dengan API BOX MARKER aktif — border merah = live, amber = campuran, abu = mock (lihat kolom Status). Kolom "Field dipakai UI" = pemetaan response → nilai yang dirender (sumber: src/services/bmkg/adapters.ts). *(proxy) merah = API tidak bisa diakses langsung dari browser (CORS / header khusus) — harus lewat proxy/alias untuk ambil response-nya. live = respon asli API · estimasi = nilai turunan/konversi dari API · mock = data statis (endpoint belum tersedia). Sumber screenshot: docs/screenshots/cards/ · skrip: docs/scrapping_cuaca-bmkg-go-id/capture_card_screenshots.js</t>
         </is>
       </c>
     </row>
@@ -6336,7 +6336,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
           </r>
           <r>
             <rPr>
@@ -6356,7 +6356,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666</t>
           </r>
         </is>
       </c>
@@ -6370,10 +6370,12 @@
       </c>
       <c r="H5" s="59" t="inlineStr">
         <is>
-          <t>▸ data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
-  Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
-▸ data.t, hu, weather_desc, ws, tcc, vs, local_datetime
-  Kondisi terobservasi saat ini: suhu, status→ikon, "terasa seperti" = t+(hu-50)/10, UV estimasi dari tcc, jarak pandang vs m→km.</t>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+  Dipakai: data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  → Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ Present Weather: cuaca saat ini
+  Dipakai: data.t, hu, weather_desc, ws, tcc, vs, local_datetime
+  → Kondisi terobservasi saat ini: suhu, status→ikon, "terasa seperti" = t+(hu-50)/10, UV estimasi dari tcc, jarak pandang vs m→km.</t>
         </is>
       </c>
       <c r="I5" s="63" t="inlineStr">
@@ -6413,7 +6415,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
           </r>
           <r>
             <rPr>
@@ -6433,7 +6435,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/df/v1/adm/coord?lat=-6.2&amp;lon=106.816666</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/df/v1/adm/coord?lat=-6.2&amp;lon=106.816666</t>
           </r>
           <r>
             <rPr>
@@ -6453,7 +6455,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666</t>
           </r>
           <r>
             <t>
@@ -6464,7 +6466,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/v1/sunset/json?lat=-6.2&amp;lng=106.816666</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/v1/sunset/json?lat=-6.2&amp;lng=106.816666</t>
           </r>
         </is>
       </c>
@@ -6482,21 +6484,25 @@
       </c>
       <c r="H6" s="59" t="inlineStr">
         <is>
-          <t>▸ data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
-  Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
-▸ provinsi, kotkab, kecamatan, desa
-  Resolusi koordinat → wilayah administratif; label lokasi kartu.
-▸ data.t, hu, weather_desc, ws, tcc, vs, local_datetime
-  Kondisi terobservasi saat ini: suhu, status→ikon, "terasa seperti" = t+(hu-50)/10, UV estimasi dari tcc, jarak pandang vs m→km.
-▸ sunrise, sunset (format 12-jam)
-  Dikonversi ke HH:mm → info matahari terbit/terbenam di CurrentWeather.</t>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+  Dipakai: data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  → Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ DF Adm: resolve wilayah admin
+  Dipakai: provinsi, kotkab, kecamatan, desa
+  → Resolusi koordinat → wilayah administratif; label lokasi kartu.
+▸ Present Weather: cuaca saat ini
+  Dipakai: data.t, hu, weather_desc, ws, tcc, vs, local_datetime
+  → Kondisi terobservasi saat ini: suhu, status→ikon, "terasa seperti" = t+(hu-50)/10, UV estimasi dari tcc, jarak pandang vs m→km.
+▸ API v1: waktu matahari terbit/terbenam
+  Dipakai: sunrise, sunset (format 12-jam)
+  → Dikonversi ke HH:mm → info matahari terbit/terbenam di CurrentWeather.</t>
         </is>
       </c>
       <c r="I6" s="63" t="inlineStr">
         <is>
           <t>Info matahari (sunset API), wilayah (df/adm).
-– UV: proksi tcc (bukan UV asli) (est)
-– "Terasa seperti": rumus t + (hu-50)/10 (est)</t>
+▸ UV: proksi tcc (bukan UV asli) — estimasi/konversi dari API
+▸ "Terasa seperti": rumus t + (hu-50)/10 — estimasi/konversi dari API</t>
         </is>
       </c>
     </row>
@@ -6529,7 +6535,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
           </r>
           <r>
             <rPr>
@@ -6549,7 +6555,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>(belum terekam saat capture) — Open Data RESMI: prakiraan-cuaca (adm4)</t>
+            <t>▸ Open Data RESMI: prakiraan-cuaca (adm4) — (belum terekam saat capture)</t>
           </r>
         </is>
       </c>
@@ -6563,10 +6569,12 @@
       </c>
       <c r="H7" s="59" t="inlineStr">
         <is>
-          <t>▸ data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
-  Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
-▸ data[].cuaca[][] → t, hu, weather_desc, tp
-  Fallback prakiraan resmi (open-data) bila df kosong — bentuk item identik df.</t>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+  Dipakai: data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  → Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ Open Data RESMI: prakiraan-cuaca (adm4)
+  Dipakai: data[].cuaca[][] → t, hu, weather_desc, tp
+  → Fallback prakiraan resmi (open-data) bila df kosong — bentuk item identik df.</t>
         </is>
       </c>
       <c r="I7" s="63" t="inlineStr">
@@ -6575,7 +6583,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="142.5" customHeight="1">
+    <row r="8" ht="153" customHeight="1">
       <c r="A8" s="58" t="n">
         <v>4</v>
       </c>
@@ -6605,7 +6613,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/public/weather/warning?lat=-6.2&amp;long=106.816666</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/public/weather/warning?lat=-6.2&amp;long=106.816666</t>
           </r>
           <r>
             <rPr>
@@ -6625,7 +6633,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>(belum terekam saat capture) — Public API: peringatan siklon</t>
+            <t>▸ Public API: peringatan siklon — (belum terekam saat capture)</t>
           </r>
           <r>
             <t>
@@ -6636,7 +6644,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://www.bmkg.go.id/alerts/nowcast/id</t>
+            <t>▸ [200] https://www.bmkg.go.id/alerts/nowcast/id</t>
           </r>
           <r>
             <rPr>
@@ -6661,12 +6669,15 @@
       </c>
       <c r="H8" s="59" t="inlineStr">
         <is>
-          <t>▸ data.today / data.tomorrow (warning_level, impact/description)
-  Peringatan hari ini/besok → severity Awas/Siaga/Waspada → AlertsPanel; kosong = tanpa peringatan.
-▸ data siklon terdampak
-  Peringatan siklon untuk wilayah — hanya muncul saat ada siklon aktif.
-▸ XML RSS: &lt;item&gt; per provinsi (title, description, pubDate)
-  Peringatan dini 3-6 jam resmi; difilter per provinsi; menang atas warning internal df.</t>
+          <t>▸ Public API: peringatan cuaca
+  Dipakai: data.today / data.tomorrow (warning_level, impact/description)
+  → Peringatan hari ini/besok → severity Awas/Siaga/Waspada → AlertsPanel; kosong = tanpa peringatan.
+▸ Public API: peringatan siklon
+  Dipakai: data siklon terdampak
+  → Peringatan siklon untuk wilayah — hanya muncul saat ada siklon aktif.
+▸ Peringatan Dini Nowcast (RSS resmi)
+  Dipakai: XML RSS: &lt;item&gt; per provinsi (title, description, pubDate)
+  → Peringatan dini 3-6 jam resmi; difilter per provinsi; menang atas warning internal df.</t>
         </is>
       </c>
       <c r="I8" s="63" t="inlineStr">
@@ -6704,7 +6715,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[502] https://cuaca.bmkg.go.id/blog/wp-json/wp/v2/posts?per_page=4&amp;_embed=1</t>
+            <t>▸ [502] https://cuaca.bmkg.go.id/blog/wp-json/wp/v2/posts?per_page=4&amp;_embed=1</t>
           </r>
           <r>
             <rPr>
@@ -6724,7 +6735,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/public/weather/video-latest?hashtag=infobmkgpws</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/public/weather/video-latest?hashtag=infobmkgpws</t>
           </r>
           <r>
             <rPr>
@@ -6747,15 +6758,17 @@
       </c>
       <c r="H9" s="59" t="inlineStr">
         <is>
-          <t>▸ [].title.rendered, excerpt.rendered, link, _embedded (featured media)
-  Artikel berita WP → NewsSection; fallback mock saat upstream 502 (sering).
-▸ [].judul, video_url
-  Video berita terbaru (per hashtag) → tab video NewsSection.</t>
+          <t>▸ Berita WordPress BMKG (WP REST)
+  Dipakai: [].title.rendered, excerpt.rendered, link, _embedded (featured media)
+  → Artikel berita WP → NewsSection; fallback mock saat upstream 502 (sering).
+▸ Public API: video berita
+  Dipakai: [].judul, video_url
+  → Video berita terbaru (per hashtag) → tab video NewsSection.</t>
         </is>
       </c>
       <c r="I9" s="63" t="inlineStr">
         <is>
-          <t>– Fallback: artikel mock saat WP 502 (sering) (mock)</t>
+          <t>▸ Fallback: artikel mock saat WP 502 (sering) — data statis (belum ada endpoint)</t>
         </is>
       </c>
     </row>
@@ -6782,7 +6795,7 @@
       </c>
       <c r="F10" s="62" t="inlineStr">
         <is>
-          <t>(belum terekam saat capture) — Open Data: gempa (TEWS)</t>
+          <t>▸ Open Data: gempa (TEWS) — (belum terekam saat capture)</t>
         </is>
       </c>
       <c r="G10" s="62" t="inlineStr">
@@ -6793,8 +6806,9 @@
       </c>
       <c r="H10" s="59" t="inlineStr">
         <is>
-          <t>▸ features[].properties (magnitude, kedalaman, wilayah, waktu)
-  Autogempa terkini + gempa dirasakan → EarthquakePanel.</t>
+          <t>▸ Open Data: gempa (TEWS)
+  Dipakai: features[].properties (magnitude, kedalaman, wilayah, waktu)
+  → Autogempa terkini + gempa dirasakan → EarthquakePanel.</t>
         </is>
       </c>
       <c r="I10" s="63" t="inlineStr">
@@ -6826,7 +6840,7 @@
       </c>
       <c r="F11" s="62" t="inlineStr">
         <is>
-          <t>(belum terekam saat capture) — Citra Satelit Himawari-9 (background-image, bukan fetch)</t>
+          <t>▸ Citra Satelit Himawari-9 (background-image, bukan fetch) — (belum terekam saat capture)</t>
         </is>
       </c>
       <c r="G11" s="62" t="inlineStr">
@@ -6837,8 +6851,9 @@
       </c>
       <c r="H11" s="59" t="inlineStr">
         <is>
-          <t>▸ (PNG) inderaja.bmkg.go.id H08_*.png
-  Citra Himawari-9 → background panel satelit (bukan JSON; terekam sebagai request gambar).</t>
+          <t>▸ Citra Satelit Himawari-9 (background-image, bukan fetch)
+  Dipakai: (PNG) inderaja.bmkg.go.id H08_*.png
+  → Citra Himawari-9 → background panel satelit (bukan JSON; terekam sebagai request gambar).</t>
         </is>
       </c>
       <c r="I11" s="63" t="inlineStr">
@@ -6885,7 +6900,7 @@
       </c>
       <c r="I12" s="63" t="inlineStr">
         <is>
-          <t>– Kartu statis: landmark + nama kota (auto-geser &amp; fetch sengaja dimatikan, 16 Sep) (mock)</t>
+          <t>▸ Kartu statis: landmark + nama kota (auto-geser &amp; fetch sengaja dimatikan, 16 Sep) — data statis (belum ada endpoint)</t>
         </is>
       </c>
     </row>
@@ -6919,7 +6934,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://publik.bmkg.go.id/event/source/dwt/apiDF_Darat/202609101600.json</t>
+            <t>▸ [200] https://publik.bmkg.go.id/event/source/dwt/apiDF_Darat/202609101600.json</t>
           </r>
           <r>
             <rPr>
@@ -6939,7 +6954,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location?lat=-6.2&amp;long=106.816666</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location?lat=-6.2&amp;long=106.816666</t>
           </r>
           <r>
             <rPr>
@@ -6959,7 +6974,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+            <t>▸ [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
           </r>
         </is>
       </c>
@@ -6975,20 +6990,23 @@
       </c>
       <c r="H13" s="59" t="inlineStr">
         <is>
-          <t>▸ rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
-  Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.
-▸ code / nama wilayah laut terdekat
-  Anchor koordinat → wilayah perairan/pelabuhan resmi terdekat.
-▸ data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
-  Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.</t>
+          <t>▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+  Dipakai: rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
+  → Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.
+▸ ISDP v1: wilayah laut terdekat
+  Dipakai: code / nama wilayah laut terdekat
+  → Anchor koordinat → wilayah perairan/pelabuhan resmi terdekat.
+▸ Maritim: detail cuaca/gelombang perairan
+  Dipakai: data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
+  → Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.</t>
         </is>
       </c>
       <c r="I13" s="63" t="inlineStr">
         <is>
-          <t>– Jalan Raya: DWT kecamatan terdekat (live)
-– Kereta: DWT stasiun terdekat (178 stasiun) (live)
-– Maritim: perairan resmi (fix currentSlot 15 Sep) (live)
-– Penerbangan: MOCK/PAUSED (menunggu data partner) (mock)</t>
+          <t>▸ Jalan Raya: DWT kecamatan terdekat — data asli dari API
+▸ Kereta: DWT stasiun terdekat (178 stasiun) — data asli dari API
+▸ Maritim: perairan resmi (fix currentSlot 15 Sep) — data asli dari API
+▸ Penerbangan: MOCK/PAUSED (menunggu data partner) — data statis (belum ada endpoint)</t>
         </is>
       </c>
     </row>
@@ -7022,7 +7040,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
           </r>
           <r>
             <rPr>
@@ -7042,7 +7060,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location?lat=-6.2&amp;long=106.816666</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location?lat=-6.2&amp;long=106.816666</t>
           </r>
           <r>
             <rPr>
@@ -7062,7 +7080,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+            <t>▸ [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
           </r>
         </is>
       </c>
@@ -7078,20 +7096,23 @@
       </c>
       <c r="H14" s="59" t="inlineStr">
         <is>
-          <t>▸ data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
-  Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
-▸ code / nama wilayah laut terdekat
-  Anchor koordinat → wilayah perairan/pelabuhan resmi terdekat.
-▸ data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
-  Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.</t>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+  Dipakai: data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  → Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ ISDP v1: wilayah laut terdekat
+  Dipakai: code / nama wilayah laut terdekat
+  → Anchor koordinat → wilayah perairan/pelabuhan resmi terdekat.
+▸ Maritim: detail cuaca/gelombang perairan
+  Dipakai: data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
+  → Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.</t>
         </is>
       </c>
       <c r="I14" s="63" t="inlineStr">
         <is>
-          <t>– Aktivitas umum: forecast live (live)
-– Aktivitas pelayaran: gelombang perairan resmi (live)
-– ISPU/AQI: ESTIMASI sintetis (tidak ada sumber resmi) (est)
-– Indeks kenyamanan: label statis (mock)</t>
+          <t>▸ Aktivitas umum: forecast live — data asli dari API
+▸ Aktivitas pelayaran: gelombang perairan resmi — data asli dari API
+▸ ISPU/AQI: ESTIMASI sintetis (tidak ada sumber resmi) — estimasi/konversi dari API
+▸ Indeks kenyamanan: label statis — data statis (belum ada endpoint)</t>
         </is>
       </c>
     </row>
@@ -7126,7 +7147,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>(belum terekam saat capture) — Maritim: overview tinggi gelombang (232 wilayah)</t>
+            <t>▸ Maritim: overview tinggi gelombang (232 wilayah) — (belum terekam saat capture)</t>
           </r>
           <r>
             <t>
@@ -7137,7 +7158,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>(belum terekam saat capture) — Maritim: polygon 232 wilayah perairan</t>
+            <t>▸ Maritim: polygon 232 wilayah perairan — (belum terekam saat capture)</t>
           </r>
           <r>
             <t>
@@ -7148,7 +7169,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+            <t>▸ [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
           </r>
           <r>
             <t>
@@ -7159,7 +7180,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://publik.bmkg.go.id/event/source/dwt/apiDF_Darat/202609101600.json</t>
+            <t>▸ [200] https://publik.bmkg.go.id/event/source/dwt/apiDF_Darat/202609101600.json</t>
           </r>
           <r>
             <rPr>
@@ -7186,21 +7207,25 @@
       </c>
       <c r="H15" s="59" t="inlineStr">
         <is>
-          <t>▸ {code: issued, today, tomorrow, wave_desc}
-  Ringkasan 232 wilayah → warna peta laut + legend gelombang.
-▸ features[].geometry (polygon 232 wilayah)
-  Polygon GeoJSON → layer batas wilayah perairan di peta.
-▸ data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
-  Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.
-▸ rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
-  Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.</t>
+          <t>▸ Maritim: overview tinggi gelombang (232 wilayah)
+  Dipakai: {code: issued, today, tomorrow, wave_desc}
+  → Ringkasan 232 wilayah → warna peta laut + legend gelombang.
+▸ Maritim: polygon 232 wilayah perairan
+  Dipakai: features[].geometry (polygon 232 wilayah)
+  → Polygon GeoJSON → layer batas wilayah perairan di peta.
+▸ Maritim: detail cuaca/gelombang perairan
+  Dipakai: data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
+  → Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.
+▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+  Dipakai: rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
+  → Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.</t>
         </is>
       </c>
       <c r="I15" s="63" t="inlineStr">
         <is>
-          <t>– Gelombang: 232 wilayah resmi (warna/legend live), klik → detail live (live)
-– Layer angin/cuaca: SNAPSHOT statis (sectors.json) (mock)
-– Mode Pelabuhan: snapshot ports.json (294) — hanya pelabuhan TERDEKAT yang live (mock)</t>
+          <t>▸ Gelombang: 232 wilayah resmi (warna/legend live), klik → detail live — data asli dari API
+▸ Layer angin/cuaca: SNAPSHOT statis (sectors.json) — data statis (belum ada endpoint)
+▸ Mode Pelabuhan: snapshot ports.json (294) — hanya pelabuhan TERDEKAT yang live — data statis (belum ada endpoint)</t>
         </is>
       </c>
     </row>
@@ -7228,8 +7253,8 @@
       </c>
       <c r="F16" s="62" t="inlineStr">
         <is>
-          <t>[200] https://maritim.bmkg.go.id/public_api/pelabuhan_list
-[200] https://maritim.bmkg.go.id/public_api/pelabuhan/0101_Sunda%20Kelapa.json</t>
+          <t>▸ [200] https://maritim.bmkg.go.id/public_api/pelabuhan_list
+▸ [200] https://maritim.bmkg.go.id/public_api/pelabuhan/0101_Sunda%20Kelapa.json</t>
         </is>
       </c>
       <c r="G16" s="62" t="inlineStr">
@@ -7242,10 +7267,12 @@
       </c>
       <c r="H16" s="59" t="inlineStr">
         <is>
-          <t>▸ files[].coor, file
-  Koordinat 294 pelabuhan → pilih terdekat → fetch detail.
-▸ detail pelabuhan + data pasut
-  Pasut (UTC → zona waktu pelabuhan) → PortTideCard; pasut null → blok disembunyikan.</t>
+          <t>▸ Maritim: daftar pelabuhan (294)
+  Dipakai: files[].coor, file
+  → Koordinat 294 pelabuhan → pilih terdekat → fetch detail.
+▸ Maritim: detail pelabuhan + pasut
+  Dipakai: detail pelabuhan + data pasut
+  → Pasut (UTC → zona waktu pelabuhan) → PortTideCard; pasut null → blok disembunyikan.</t>
         </is>
       </c>
       <c r="I16" s="63" t="inlineStr">
@@ -7283,7 +7310,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
           </r>
           <r>
             <rPr>
@@ -7303,7 +7330,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>(belum terekam saat capture) — Overpass API: POI OpenStreetMap</t>
+            <t>▸ Overpass API: POI OpenStreetMap — (belum terekam saat capture)</t>
           </r>
         </is>
       </c>
@@ -7317,16 +7344,18 @@
       </c>
       <c r="H17" s="59" t="inlineStr">
         <is>
-          <t>▸ data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
-  Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
-▸ elements[].lat/lon/tags
-  POI OpenStreetMap sekitar pengguna → AroundActivity.</t>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+  Dipakai: data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  → Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ Overpass API: POI OpenStreetMap
+  Dipakai: elements[].lat/lon/tags
+  → POI OpenStreetMap sekitar pengguna → AroundActivity.</t>
         </is>
       </c>
       <c r="I17" s="63" t="inlineStr">
         <is>
           <t>Nilai cuaca per titik POI live (1 request df/coord per POI).
-– Daftar POI: kurasi statis (cityLandmarks) (mock)</t>
+▸ Daftar POI: kurasi statis (cityLandmarks) — data statis (belum ada endpoint)</t>
         </is>
       </c>
     </row>
@@ -7362,7 +7391,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
           </r>
           <r>
             <rPr>
@@ -7382,7 +7411,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://publik.bmkg.go.id/event/source/dwt/apiDF_Darat/202609101600.json</t>
+            <t>▸ [200] https://publik.bmkg.go.id/event/source/dwt/apiDF_Darat/202609101600.json</t>
           </r>
           <r>
             <rPr>
@@ -7402,7 +7431,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>(belum terekam saat capture) — Overpass API: POI OpenStreetMap</t>
+            <t>▸ Overpass API: POI OpenStreetMap — (belum terekam saat capture)</t>
           </r>
           <r>
             <t>
@@ -7413,7 +7442,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>(belum terekam saat capture) — Nominatim: geocode OSM</t>
+            <t>▸ Nominatim: geocode OSM — (belum terekam saat capture)</t>
           </r>
           <r>
             <t>
@@ -7424,7 +7453,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>(belum terekam saat capture) — OSRM: routing</t>
+            <t>▸ OSRM: routing — (belum terekam saat capture)</t>
           </r>
         </is>
       </c>
@@ -7444,22 +7473,27 @@
       </c>
       <c r="H18" s="59" t="inlineStr">
         <is>
-          <t>▸ data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
-  Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
-▸ rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
-  Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.
-▸ elements[].lat/lon/tags
-  POI OpenStreetMap sekitar pengguna → AroundActivity.
-▸ [].lat/lon/display_name
-  Geocode nama tempat → koordinat.
-▸ routes[].geometry, duration, distance
-  Rute antar titik → panel aktivitas darat.</t>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+  Dipakai: data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  → Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+  Dipakai: rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
+  → Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.
+▸ Overpass API: POI OpenStreetMap
+  Dipakai: elements[].lat/lon/tags
+  → POI OpenStreetMap sekitar pengguna → AroundActivity.
+▸ Nominatim: geocode OSM
+  Dipakai: [].lat/lon/display_name
+  → Geocode nama tempat → koordinat.
+▸ OSRM: routing
+  Dipakai: routes[].geometry, duration, distance
+  → Rute antar titik → panel aktivitas darat.</t>
         </is>
       </c>
       <c r="I18" s="63" t="inlineStr">
         <is>
           <t>Forecast per titik rute live; fallback mock saat API gagal.
-– Pilihan lokasi awal: daftar statis (mock)</t>
+▸ Pilihan lokasi awal: daftar statis — data statis (belum ada endpoint)</t>
         </is>
       </c>
     </row>
@@ -7492,7 +7526,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location?lat=-6.2&amp;long=106.816666</t>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location?lat=-6.2&amp;long=106.816666</t>
           </r>
           <r>
             <rPr>
@@ -7512,7 +7546,7 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>[200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+            <t>▸ [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
           </r>
         </is>
       </c>
@@ -7526,16 +7560,18 @@
       </c>
       <c r="H19" s="59" t="inlineStr">
         <is>
-          <t>▸ code / nama wilayah laut terdekat
-  Anchor koordinat → wilayah perairan/pelabuhan resmi terdekat.
-▸ data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
-  Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.</t>
+          <t>▸ ISDP v1: wilayah laut terdekat
+  Dipakai: code / nama wilayah laut terdekat
+  → Anchor koordinat → wilayah perairan/pelabuhan resmi terdekat.
+▸ Maritim: detail cuaca/gelombang perairan
+  Dipakai: data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
+  → Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.</t>
         </is>
       </c>
       <c r="I19" s="63" t="inlineStr">
         <is>
           <t>Parameter gelombang resmi di-inject ke drawer.
-– Sisa konten drawer (jenis aktivitas, tabel): statis maritimeAdvisorData.ts (mock)</t>
+▸ Sisa konten drawer (jenis aktivitas, tabel): statis maritimeAdvisorData.ts — data statis (belum ada endpoint)</t>
         </is>
       </c>
     </row>
@@ -7577,7 +7613,7 @@
       </c>
       <c r="I20" s="63" t="inlineStr">
         <is>
-          <t>– 100% statis (aviationAdvisorData.ts) — API penerbangan belum ada (mock)</t>
+          <t>▸ 100% statis (aviationAdvisorData.ts) — API penerbangan belum ada — data statis (belum ada endpoint)</t>
         </is>
       </c>
     </row>
@@ -7619,7 +7655,7 @@
       </c>
       <c r="I21" s="63" t="inlineStr">
         <is>
-          <t>– POI statis (poiSearchData.ts) (mock)</t>
+          <t>▸ POI statis (poiSearchData.ts) — data statis (belum ada endpoint)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(xlsx): enter baris di kolom F (rich-text) benar-benar tersimpan
Newline antar API di sel rich-text sebelumnya berupa string polos terpisah
— Excel memotong <t> tanpa format → daftar tampak menyatu 1 baris. Kini
newline ikut dalam TextBlock berfont (run <r><rPr> dengan <t>\n</t>) +
tinggi baris ikut menghitung kolom F.
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -6348,6 +6348,10 @@
             <t xml:space="preserve"> *(proxy)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -6427,6 +6431,10 @@
             <t xml:space="preserve"> *(proxy)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -6447,6 +6455,10 @@
             <t xml:space="preserve"> *(proxy)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -6458,6 +6470,10 @@
             <t>▸ [200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -6547,6 +6563,10 @@
             <t xml:space="preserve"> *(proxy)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -6625,6 +6645,10 @@
             <t xml:space="preserve"> *(proxy)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -6636,6 +6660,10 @@
             <t>▸ Public API: peringatan siklon — (belum terekam saat capture)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -6727,6 +6755,10 @@
             <t xml:space="preserve"> *(proxy)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -6946,6 +6978,10 @@
             <t xml:space="preserve"> *(proxy)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -6966,6 +7002,10 @@
             <t xml:space="preserve"> *(proxy)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -7052,6 +7092,10 @@
             <t xml:space="preserve"> *(proxy)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -7072,6 +7116,10 @@
             <t xml:space="preserve"> *(proxy)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -7150,6 +7198,10 @@
             <t>▸ Maritim: overview tinggi gelombang (232 wilayah) — (belum terekam saat capture)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -7161,6 +7213,10 @@
             <t>▸ Maritim: polygon 232 wilayah perairan — (belum terekam saat capture)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -7172,6 +7228,10 @@
             <t>▸ [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -7322,6 +7382,10 @@
             <t xml:space="preserve"> *(proxy)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -7403,6 +7467,10 @@
             <t xml:space="preserve"> *(proxy)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -7423,6 +7491,10 @@
             <t xml:space="preserve"> *(proxy)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -7434,6 +7506,10 @@
             <t>▸ Overpass API: POI OpenStreetMap — (belum terekam saat capture)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -7445,6 +7521,10 @@
             <t>▸ Nominatim: geocode OSM — (belum terekam saat capture)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>
@@ -7538,6 +7618,10 @@
             <t xml:space="preserve"> *(proxy)</t>
           </r>
           <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
             <t>
 </t>
           </r>

</xml_diff>

<commit_message>
fix(xlsx): newline kolom F digabung ke run teks berikutnya (xml:space=preserve)
Run berisi '\n' saja tetap di-drop renderer — diperbaiki mengikuti pola
file Excel asli: '\n' menempel di awal teks baris berikutnya dalam run
yang sama dengan xml:space="preserve". Terverifikasi di XML:
<t xml:space="preserve">
&#9656; [200] https://…</t>
</commit_message>
<xml_diff>
--- a/docs/bmkg-api-mapping.xlsx
+++ b/docs/bmkg-api-mapping.xlsx
@@ -6352,15 +6352,8 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666</t>
+            <t xml:space="preserve">
+▸ [200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666</t>
           </r>
         </is>
       </c>
@@ -6435,15 +6428,8 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://cuaca.bmkg.go.id/api/df/v1/adm/coord?lat=-6.2&amp;lon=106.816666</t>
+            <t xml:space="preserve">
+▸ [200] https://cuaca.bmkg.go.id/api/df/v1/adm/coord?lat=-6.2&amp;lon=106.816666</t>
           </r>
           <r>
             <rPr>
@@ -6459,30 +6445,16 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>
-</t>
+            <t xml:space="preserve">
+▸ [200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666</t>
           </r>
           <r>
             <rPr>
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>▸ [200] https://cuaca.bmkg.go.id/api/presentwx/coord?lat=-6.2&amp;lon=106.816666</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://cuaca.bmkg.go.id/api/v1/sunset/json?lat=-6.2&amp;lng=106.816666</t>
+            <t xml:space="preserve">
+▸ [200] https://cuaca.bmkg.go.id/api/v1/sunset/json?lat=-6.2&amp;lng=106.816666</t>
           </r>
         </is>
       </c>
@@ -6567,15 +6539,8 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ Open Data RESMI: prakiraan-cuaca (adm4) — (belum terekam saat capture)</t>
+            <t xml:space="preserve">
+▸ Open Data RESMI: prakiraan-cuaca (adm4) — (belum terekam saat capture)</t>
           </r>
         </is>
       </c>
@@ -6649,30 +6614,16 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>
-</t>
+            <t xml:space="preserve">
+▸ Public API: peringatan siklon — (belum terekam saat capture)</t>
           </r>
           <r>
             <rPr>
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>▸ Public API: peringatan siklon — (belum terekam saat capture)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://www.bmkg.go.id/alerts/nowcast/id</t>
+            <t xml:space="preserve">
+▸ [200] https://www.bmkg.go.id/alerts/nowcast/id</t>
           </r>
           <r>
             <rPr>
@@ -6759,15 +6710,8 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://cuaca.bmkg.go.id/api/public/weather/video-latest?hashtag=infobmkgpws</t>
+            <t xml:space="preserve">
+▸ [200] https://cuaca.bmkg.go.id/api/public/weather/video-latest?hashtag=infobmkgpws</t>
           </r>
           <r>
             <rPr>
@@ -6982,9 +6926,541 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>
-</t>
+            <t xml:space="preserve">
+▸ [200] https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location?lat=-6.2&amp;long=106.816666</t>
           </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+▸ [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+          </r>
+        </is>
+      </c>
+      <c r="G13" s="62" t="inlineStr">
+        <is>
+          <t>▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+[["lampung","Kab. Lampung Tengah","Terusan Nunyai",-4.699604904679063,105.20665965569867,"5013584","2026-09-10 16:00:00",["78","26","1","SE","9.5"],"ndf"],["lampung","Kab. Lampung Tengah","Seputih Agung",-4.89787745875816,105.05458830281606,"5013578","2026-09-10 16:00:00",["80","26","3","SE","9.2"],"ndf"],["lampung","Kab. Lampung Utara","Kotabumi",-4.846956993233334,104.85804482373453,"501378","2026-09-10 16:00:00",["81","26","1","SE","11.7"],"ndf"],["lampung","Kab. Lampung Utara","Abung Barat",-4.865040896877758,104.69148255332641,"5013612","2026-09-10 16:00:00",["87","24","1","SE","5.5"],"nd …
+▸ ISDP v1: wilayah laut terdekat
+{"statusCode":200,"message":"OK!","data":{"code":"F.09","name":"Teluk Jakarta","wilpel":"Stamar Tanjung Priok - Jakarta","geometry":{"type":"Polygon","coordinates":[[[106.68448229697637,-6.015114864033774],[106.68448229697637,-5.910111585789263],[107.03498697202032,-5.910111585789263],[106.99055680194432,-5.931987268756869],[107.01030354420033,-5.940737541943912],[107.02017691532832,-5.960425656614758],[107.01030354420033,-5.984488907879126],[106.98562011638033,-6.004177022549971],[106.99055680194432,-6.023865137220817],[107.02017691532832,-6.03480297870462],[107.02017691532832,-6.078554344639 …
+▸ Maritim: detail cuaca/gelombang perairan
+{"code": "F.09", "name": "Teluk Jakarta", "issued": "2026-09-21 23:39 UTC", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "data": [{"valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "time_desc": "Hari ini", "weather": "Berawan", "weather_desc": "Hari ini untuk Teluk Jakarta diperkirakan berawan, dengan kecepatan angin pada umumnya 5 - 18 knot bertiup dari arah selatan, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": …</t>
+        </is>
+      </c>
+      <c r="H13" s="59" t="inlineStr">
+        <is>
+          <t>▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+  Dipakai: rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
+  → Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.
+▸ ISDP v1: wilayah laut terdekat
+  Dipakai: code / nama wilayah laut terdekat
+  → Anchor koordinat → wilayah perairan/pelabuhan resmi terdekat.
+▸ Maritim: detail cuaca/gelombang perairan
+  Dipakai: data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
+  → Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.</t>
+        </is>
+      </c>
+      <c r="I13" s="63" t="inlineStr">
+        <is>
+          <t>▸ Jalan Raya: DWT kecamatan terdekat — data asli dari API
+▸ Kereta: DWT stasiun terdekat (178 stasiun) — data asli dari API
+▸ Maritim: perairan resmi (fix currentSlot 15 Sep) — data asli dari API
+▸ Penerbangan: MOCK/PAUSED (menunggu data partner) — data statis (belum ada endpoint)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="409" customHeight="1">
+      <c r="A14" s="58" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="59" t="inlineStr">
+        <is>
+          <t>Panduan Aktivitas &amp; Analisis Cuaca
+(weather-activity)</t>
+        </is>
+      </c>
+      <c r="C14" s="60" t="n"/>
+      <c r="D14" s="65" t="inlineStr">
+        <is>
+          <t>⚠️ CAMPURAN</t>
+        </is>
+      </c>
+      <c r="E14" s="59" t="inlineStr">
+        <is>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+▸ ISDP v1: wilayah laut terdekat
+▸ Maritim: detail cuaca/gelombang perairan</t>
+        </is>
+      </c>
+      <c r="F14" s="62" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+▸ [200] https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location?lat=-6.2&amp;long=106.816666</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+▸ [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+          </r>
+        </is>
+      </c>
+      <c r="G14" s="62" t="inlineStr">
+        <is>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.82670735619568,"lat":-6.176384269281675,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.8267073562,"lat":-6.1763842693,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T09:00:00Z","t":28,"tcc":90,"tp":0,"weathe …
+▸ ISDP v1: wilayah laut terdekat
+{"statusCode":200,"message":"OK!","data":{"code":"F.09","name":"Teluk Jakarta","wilpel":"Stamar Tanjung Priok - Jakarta","geometry":{"type":"Polygon","coordinates":[[[106.68448229697637,-6.015114864033774],[106.68448229697637,-5.910111585789263],[107.03498697202032,-5.910111585789263],[106.99055680194432,-5.931987268756869],[107.01030354420033,-5.940737541943912],[107.02017691532832,-5.960425656614758],[107.01030354420033,-5.984488907879126],[106.98562011638033,-6.004177022549971],[106.99055680194432,-6.023865137220817],[107.02017691532832,-6.03480297870462],[107.02017691532832,-6.078554344639 …
+▸ Maritim: detail cuaca/gelombang perairan
+{"code": "F.09", "name": "Teluk Jakarta", "issued": "2026-09-21 23:39 UTC", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "data": [{"valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "time_desc": "Hari ini", "weather": "Berawan", "weather_desc": "Hari ini untuk Teluk Jakarta diperkirakan berawan, dengan kecepatan angin pada umumnya 5 - 18 knot bertiup dari arah selatan, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": …</t>
+        </is>
+      </c>
+      <c r="H14" s="59" t="inlineStr">
+        <is>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+  Dipakai: data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  → Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ ISDP v1: wilayah laut terdekat
+  Dipakai: code / nama wilayah laut terdekat
+  → Anchor koordinat → wilayah perairan/pelabuhan resmi terdekat.
+▸ Maritim: detail cuaca/gelombang perairan
+  Dipakai: data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
+  → Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.</t>
+        </is>
+      </c>
+      <c r="I14" s="63" t="inlineStr">
+        <is>
+          <t>▸ Aktivitas umum: forecast live — data asli dari API
+▸ Aktivitas pelayaran: gelombang perairan resmi — data asli dari API
+▸ ISPU/AQI: ESTIMASI sintetis (tidak ada sumber resmi) — estimasi/konversi dari API
+▸ Indeks kenyamanan: label statis — data statis (belum ada endpoint)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="294.5" customHeight="1">
+      <c r="A15" s="58" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="59" t="inlineStr">
+        <is>
+          <t>Peta Laut (Marine Map)
+(marine-map)</t>
+        </is>
+      </c>
+      <c r="C15" s="60" t="n"/>
+      <c r="D15" s="65" t="inlineStr">
+        <is>
+          <t>⚠️ CAMPURAN</t>
+        </is>
+      </c>
+      <c r="E15" s="59" t="inlineStr">
+        <is>
+          <t>▸ Maritim: overview tinggi gelombang (232 wilayah)
+▸ Maritim: polygon 232 wilayah perairan
+▸ Maritim: detail cuaca/gelombang perairan
+▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)</t>
+        </is>
+      </c>
+      <c r="F15" s="62" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>▸ Maritim: overview tinggi gelombang (232 wilayah) — (belum terekam saat capture)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+▸ Maritim: polygon 232 wilayah perairan — (belum terekam saat capture)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+▸ [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+▸ [200] https://publik.bmkg.go.id/event/source/dwt/apiDF_Darat/202609101600.json</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+        </is>
+      </c>
+      <c r="G15" s="62" t="inlineStr">
+        <is>
+          <t>▸ Maritim: overview tinggi gelombang (232 wilayah)
+(tidak ada response live)
+▸ Maritim: polygon 232 wilayah perairan
+(tidak ada response live)
+▸ Maritim: detail cuaca/gelombang perairan
+{"code": "F.09", "name": "Teluk Jakarta", "issued": "2026-09-21 23:39 UTC", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "data": [{"valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "time_desc": "Hari ini", "weather": "Berawan", "weather_desc": "Hari ini untuk Teluk Jakarta diperkirakan berawan, dengan kecepatan angin pada umumnya 5 - 18 knot bertiup dari arah selatan, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": …
+▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+[["lampung","Kab. Lampung Tengah","Terusan Nunyai",-4.699604904679063,105.20665965569867,"5013584","2026-09-10 16:00:00",["78","26","1","SE","9.5"],"ndf"],["lampung","Kab. Lampung Tengah","Seputih Agung",-4.89787745875816,105.05458830281606,"5013578","2026-09-10 16:00:00",["80","26","3","SE","9.2"],"ndf"],["lampung","Kab. Lampung Utara","Kotabumi",-4.846956993233334,104.85804482373453,"501378","2026-09-10 16:00:00",["81","26","1","SE","11.7"],"ndf"],["lampung","Kab. Lampung Utara","Abung Barat",-4.865040896877758,104.69148255332641,"5013612","2026-09-10 16:00:00",["87","24","1","SE","5.5"],"nd …</t>
+        </is>
+      </c>
+      <c r="H15" s="59" t="inlineStr">
+        <is>
+          <t>▸ Maritim: overview tinggi gelombang (232 wilayah)
+  Dipakai: {code: issued, today, tomorrow, wave_desc}
+  → Ringkasan 232 wilayah → warna peta laut + legend gelombang.
+▸ Maritim: polygon 232 wilayah perairan
+  Dipakai: features[].geometry (polygon 232 wilayah)
+  → Polygon GeoJSON → layer batas wilayah perairan di peta.
+▸ Maritim: detail cuaca/gelombang perairan
+  Dipakai: data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
+  → Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.
+▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+  Dipakai: rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
+  → Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.</t>
+        </is>
+      </c>
+      <c r="I15" s="63" t="inlineStr">
+        <is>
+          <t>▸ Gelombang: 232 wilayah resmi (warna/legend live), klik → detail live — data asli dari API
+▸ Layer angin/cuaca: SNAPSHOT statis (sectors.json) — data statis (belum ada endpoint)
+▸ Mode Pelabuhan: snapshot ports.json (294) — hanya pelabuhan TERDEKAT yang live — data statis (belum ada endpoint)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="287.75" customHeight="1">
+      <c r="A16" s="58" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="59" t="inlineStr">
+        <is>
+          <t>Pelabuhan &amp; Pasut
+(port-tide)</t>
+        </is>
+      </c>
+      <c r="C16" s="60" t="n"/>
+      <c r="D16" s="61" t="inlineStr">
+        <is>
+          <t>✅ LIVE</t>
+        </is>
+      </c>
+      <c r="E16" s="59" t="inlineStr">
+        <is>
+          <t>▸ Maritim: daftar pelabuhan (294)
+▸ Maritim: detail pelabuhan + pasut</t>
+        </is>
+      </c>
+      <c r="F16" s="62" t="inlineStr">
+        <is>
+          <t>▸ [200] https://maritim.bmkg.go.id/public_api/pelabuhan_list
+▸ [200] https://maritim.bmkg.go.id/public_api/pelabuhan/0101_Sunda%20Kelapa.json</t>
+        </is>
+      </c>
+      <c r="G16" s="62" t="inlineStr">
+        <is>
+          <t>▸ Maritim: daftar pelabuhan (294)
+{ "files": [ { "coor": [ 1.198331, 109.054462 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1720, "name": "0088_Sintete.json", "portname": "Sintete", "type": "utama" }, { "coor": [ 0.00214, 109.285391 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1713, "name": "0310_PPP Sungai Rengas.json", "portname": "PPP Sungai Rengas", "type": "utama" }, { "coor": [ -2.531535, 110.21588 ], "file_date": "2026-09-21 23:47 UTC", "kb": …
+▸ Maritim: detail pelabuhan + pasut
+{"port_id": "0101", "name": "Sunda Kelapa", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "latitude": -6.11664888, "longitude": 106.80830956, "type": "utama", "data": [{"issued": "2026-09-21 23:47 UTC", "valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "weather": "Berawan", "weather_desc": "Untuk area Sunda Kelapa diperkirakan berawan, dengan kecepatan angin pada umumnya 2 - 14 knot bertiup dari arah timur", "warning_desc": "NIL", "wind_from": "Timur", "wind_to": "Utara", "wind_speed_min": 2, "wind_speed_max": 1 …</t>
+        </is>
+      </c>
+      <c r="H16" s="59" t="inlineStr">
+        <is>
+          <t>▸ Maritim: daftar pelabuhan (294)
+  Dipakai: files[].coor, file
+  → Koordinat 294 pelabuhan → pilih terdekat → fetch detail.
+▸ Maritim: detail pelabuhan + pasut
+  Dipakai: detail pelabuhan + data pasut
+  → Pasut (UTC → zona waktu pelabuhan) → PortTideCard; pasut null → blok disembunyikan.</t>
+        </is>
+      </c>
+      <c r="I16" s="63" t="inlineStr">
+        <is>
+          <t>Pasut null di sebagian pelabuhan → blok disembunyikan. Kolom arus di-skip (satuan ambigu).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="126.5" customHeight="1">
+      <c r="A17" s="58" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="59" t="inlineStr">
+        <is>
+          <t>Aktivitas Sekitar (POI)
+(around-activity)</t>
+        </is>
+      </c>
+      <c r="C17" s="60" t="n"/>
+      <c r="D17" s="65" t="inlineStr">
+        <is>
+          <t>⚠️ CAMPURAN</t>
+        </is>
+      </c>
+      <c r="E17" s="59" t="inlineStr">
+        <is>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+▸ Overpass API: POI OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="F17" s="62" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+▸ Overpass API: POI OpenStreetMap — (belum terekam saat capture)</t>
+          </r>
+        </is>
+      </c>
+      <c r="G17" s="62" t="inlineStr">
+        <is>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.82670735619568,"lat":-6.176384269281675,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.8267073562,"lat":-6.1763842693,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T09:00:00Z","t":28,"tcc":90,"tp":0,"weathe …
+▸ Overpass API: POI OpenStreetMap
+(tidak ada response live)</t>
+        </is>
+      </c>
+      <c r="H17" s="59" t="inlineStr">
+        <is>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+  Dipakai: data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  → Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ Overpass API: POI OpenStreetMap
+  Dipakai: elements[].lat/lon/tags
+  → POI OpenStreetMap sekitar pengguna → AroundActivity.</t>
+        </is>
+      </c>
+      <c r="I17" s="63" t="inlineStr">
+        <is>
+          <t>Nilai cuaca per titik POI live (1 request df/coord per POI).
+▸ Daftar POI: kurasi statis (cityLandmarks) — data statis (belum ada endpoint)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="279" customHeight="1">
+      <c r="A18" s="58" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="59" t="inlineStr">
+        <is>
+          <t>Aktivitas Darat (Drawer)
+(land-based)</t>
+        </is>
+      </c>
+      <c r="C18" s="60" t="n"/>
+      <c r="D18" s="65" t="inlineStr">
+        <is>
+          <t>⚠️ CAMPURAN</t>
+        </is>
+      </c>
+      <c r="E18" s="59" t="inlineStr">
+        <is>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+▸ Overpass API: POI OpenStreetMap
+▸ Nominatim: geocode OSM
+▸ OSRM: routing</t>
+        </is>
+      </c>
+      <c r="F18" s="62" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t>▸ [200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+▸ [200] https://publik.bmkg.go.id/event/source/dwt/apiDF_Darat/202609101600.json</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <b val="1"/>
+              <color rgb="FFCC0000"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve"> *(proxy)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+▸ Overpass API: POI OpenStreetMap — (belum terekam saat capture)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+▸ Nominatim: geocode OSM — (belum terekam saat capture)</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Courier New"/>
+              <sz val="8"/>
+            </rPr>
+            <t xml:space="preserve">
+▸ OSRM: routing — (belum terekam saat capture)</t>
+          </r>
+        </is>
+      </c>
+      <c r="G18" s="62" t="inlineStr">
+        <is>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.82670735619568,"lat":-6.176384269281675,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.8267073562,"lat":-6.1763842693,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T09:00:00Z","t":28,"tcc":90,"tp":0,"weathe …
+▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+[["lampung","Kab. Lampung Tengah","Terusan Nunyai",-4.699604904679063,105.20665965569867,"5013584","2026-09-10 16:00:00",["78","26","1","SE","9.5"],"ndf"],["lampung","Kab. Lampung Tengah","Seputih Agung",-4.89787745875816,105.05458830281606,"5013578","2026-09-10 16:00:00",["80","26","3","SE","9.2"],"ndf"],["lampung","Kab. Lampung Utara","Kotabumi",-4.846956993233334,104.85804482373453,"501378","2026-09-10 16:00:00",["81","26","1","SE","11.7"],"ndf"],["lampung","Kab. Lampung Utara","Abung Barat",-4.865040896877758,104.69148255332641,"5013612","2026-09-10 16:00:00",["87","24","1","SE","5.5"],"nd …
+▸ Overpass API: POI OpenStreetMap
+(tidak ada response live)
+▸ Nominatim: geocode OSM
+(tidak ada response live)
+▸ OSRM: routing
+(tidak ada response live)</t>
+        </is>
+      </c>
+      <c r="H18" s="59" t="inlineStr">
+        <is>
+          <t>▸ DF Forecast: prakiraan 10 hari + per jam
+  Dipakai: data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
+  → Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
+▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
+  Dipakai: rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
+  → Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.
+▸ Overpass API: POI OpenStreetMap
+  Dipakai: elements[].lat/lon/tags
+  → POI OpenStreetMap sekitar pengguna → AroundActivity.
+▸ Nominatim: geocode OSM
+  Dipakai: [].lat/lon/display_name
+  → Geocode nama tempat → koordinat.
+▸ OSRM: routing
+  Dipakai: routes[].geometry, duration, distance
+  → Rute antar titik → panel aktivitas darat.</t>
+        </is>
+      </c>
+      <c r="I18" s="63" t="inlineStr">
+        <is>
+          <t>Forecast per titik rute live; fallback mock saat API gagal.
+▸ Pilihan lokasi awal: daftar statis — data statis (belum ada endpoint)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="271.25" customHeight="1">
+      <c r="A19" s="58" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="59" t="inlineStr">
+        <is>
+          <t>Konsultasi Pelayaran (Drawer)
+(maritime-advisor)</t>
+        </is>
+      </c>
+      <c r="C19" s="60" t="n"/>
+      <c r="D19" s="65" t="inlineStr">
+        <is>
+          <t>⚠️ CAMPURAN</t>
+        </is>
+      </c>
+      <c r="E19" s="59" t="inlineStr">
+        <is>
+          <t>▸ ISDP v1: wilayah laut terdekat
+▸ Maritim: detail cuaca/gelombang perairan</t>
+        </is>
+      </c>
+      <c r="F19" s="62" t="inlineStr">
+        <is>
           <r>
             <rPr>
               <rFont val="Courier New"/>
@@ -7006,631 +7482,8 @@
               <rFont val="Courier New"/>
               <sz val="8"/>
             </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
-          </r>
-        </is>
-      </c>
-      <c r="G13" s="62" t="inlineStr">
-        <is>
-          <t>▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
-[["lampung","Kab. Lampung Tengah","Terusan Nunyai",-4.699604904679063,105.20665965569867,"5013584","2026-09-10 16:00:00",["78","26","1","SE","9.5"],"ndf"],["lampung","Kab. Lampung Tengah","Seputih Agung",-4.89787745875816,105.05458830281606,"5013578","2026-09-10 16:00:00",["80","26","3","SE","9.2"],"ndf"],["lampung","Kab. Lampung Utara","Kotabumi",-4.846956993233334,104.85804482373453,"501378","2026-09-10 16:00:00",["81","26","1","SE","11.7"],"ndf"],["lampung","Kab. Lampung Utara","Abung Barat",-4.865040896877758,104.69148255332641,"5013612","2026-09-10 16:00:00",["87","24","1","SE","5.5"],"nd …
-▸ ISDP v1: wilayah laut terdekat
-{"statusCode":200,"message":"OK!","data":{"code":"F.09","name":"Teluk Jakarta","wilpel":"Stamar Tanjung Priok - Jakarta","geometry":{"type":"Polygon","coordinates":[[[106.68448229697637,-6.015114864033774],[106.68448229697637,-5.910111585789263],[107.03498697202032,-5.910111585789263],[106.99055680194432,-5.931987268756869],[107.01030354420033,-5.940737541943912],[107.02017691532832,-5.960425656614758],[107.01030354420033,-5.984488907879126],[106.98562011638033,-6.004177022549971],[106.99055680194432,-6.023865137220817],[107.02017691532832,-6.03480297870462],[107.02017691532832,-6.078554344639 …
-▸ Maritim: detail cuaca/gelombang perairan
-{"code": "F.09", "name": "Teluk Jakarta", "issued": "2026-09-21 23:39 UTC", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "data": [{"valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "time_desc": "Hari ini", "weather": "Berawan", "weather_desc": "Hari ini untuk Teluk Jakarta diperkirakan berawan, dengan kecepatan angin pada umumnya 5 - 18 knot bertiup dari arah selatan, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": …</t>
-        </is>
-      </c>
-      <c r="H13" s="59" t="inlineStr">
-        <is>
-          <t>▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
-  Dipakai: rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
-  → Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.
-▸ ISDP v1: wilayah laut terdekat
-  Dipakai: code / nama wilayah laut terdekat
-  → Anchor koordinat → wilayah perairan/pelabuhan resmi terdekat.
-▸ Maritim: detail cuaca/gelombang perairan
-  Dipakai: data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
-  → Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.</t>
-        </is>
-      </c>
-      <c r="I13" s="63" t="inlineStr">
-        <is>
-          <t>▸ Jalan Raya: DWT kecamatan terdekat — data asli dari API
-▸ Kereta: DWT stasiun terdekat (178 stasiun) — data asli dari API
-▸ Maritim: perairan resmi (fix currentSlot 15 Sep) — data asli dari API
-▸ Penerbangan: MOCK/PAUSED (menunggu data partner) — data statis (belum ada endpoint)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="409" customHeight="1">
-      <c r="A14" s="58" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="59" t="inlineStr">
-        <is>
-          <t>Panduan Aktivitas &amp; Analisis Cuaca
-(weather-activity)</t>
-        </is>
-      </c>
-      <c r="C14" s="60" t="n"/>
-      <c r="D14" s="65" t="inlineStr">
-        <is>
-          <t>⚠️ CAMPURAN</t>
-        </is>
-      </c>
-      <c r="E14" s="59" t="inlineStr">
-        <is>
-          <t>▸ DF Forecast: prakiraan 10 hari + per jam
-▸ ISDP v1: wilayah laut terdekat
-▸ Maritim: detail cuaca/gelombang perairan</t>
-        </is>
-      </c>
-      <c r="F14" s="62" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <b val="1"/>
-              <color rgb="FFCC0000"/>
-              <sz val="8"/>
-            </rPr>
-            <t xml:space="preserve"> *(proxy)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location?lat=-6.2&amp;long=106.816666</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <b val="1"/>
-              <color rgb="FFCC0000"/>
-              <sz val="8"/>
-            </rPr>
-            <t xml:space="preserve"> *(proxy)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
-          </r>
-        </is>
-      </c>
-      <c r="G14" s="62" t="inlineStr">
-        <is>
-          <t>▸ DF Forecast: prakiraan 10 hari + per jam
-{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.82670735619568,"lat":-6.176384269281675,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.8267073562,"lat":-6.1763842693,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T09:00:00Z","t":28,"tcc":90,"tp":0,"weathe …
-▸ ISDP v1: wilayah laut terdekat
-{"statusCode":200,"message":"OK!","data":{"code":"F.09","name":"Teluk Jakarta","wilpel":"Stamar Tanjung Priok - Jakarta","geometry":{"type":"Polygon","coordinates":[[[106.68448229697637,-6.015114864033774],[106.68448229697637,-5.910111585789263],[107.03498697202032,-5.910111585789263],[106.99055680194432,-5.931987268756869],[107.01030354420033,-5.940737541943912],[107.02017691532832,-5.960425656614758],[107.01030354420033,-5.984488907879126],[106.98562011638033,-6.004177022549971],[106.99055680194432,-6.023865137220817],[107.02017691532832,-6.03480297870462],[107.02017691532832,-6.078554344639 …
-▸ Maritim: detail cuaca/gelombang perairan
-{"code": "F.09", "name": "Teluk Jakarta", "issued": "2026-09-21 23:39 UTC", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "data": [{"valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "time_desc": "Hari ini", "weather": "Berawan", "weather_desc": "Hari ini untuk Teluk Jakarta diperkirakan berawan, dengan kecepatan angin pada umumnya 5 - 18 knot bertiup dari arah selatan, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": …</t>
-        </is>
-      </c>
-      <c r="H14" s="59" t="inlineStr">
-        <is>
-          <t>▸ DF Forecast: prakiraan 10 hari + per jam
-  Dipakai: data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
-  → Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
-▸ ISDP v1: wilayah laut terdekat
-  Dipakai: code / nama wilayah laut terdekat
-  → Anchor koordinat → wilayah perairan/pelabuhan resmi terdekat.
-▸ Maritim: detail cuaca/gelombang perairan
-  Dipakai: data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
-  → Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.</t>
-        </is>
-      </c>
-      <c r="I14" s="63" t="inlineStr">
-        <is>
-          <t>▸ Aktivitas umum: forecast live — data asli dari API
-▸ Aktivitas pelayaran: gelombang perairan resmi — data asli dari API
-▸ ISPU/AQI: ESTIMASI sintetis (tidak ada sumber resmi) — estimasi/konversi dari API
-▸ Indeks kenyamanan: label statis — data statis (belum ada endpoint)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="294.5" customHeight="1">
-      <c r="A15" s="58" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="59" t="inlineStr">
-        <is>
-          <t>Peta Laut (Marine Map)
-(marine-map)</t>
-        </is>
-      </c>
-      <c r="C15" s="60" t="n"/>
-      <c r="D15" s="65" t="inlineStr">
-        <is>
-          <t>⚠️ CAMPURAN</t>
-        </is>
-      </c>
-      <c r="E15" s="59" t="inlineStr">
-        <is>
-          <t>▸ Maritim: overview tinggi gelombang (232 wilayah)
-▸ Maritim: polygon 232 wilayah perairan
-▸ Maritim: detail cuaca/gelombang perairan
-▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)</t>
-        </is>
-      </c>
-      <c r="F15" s="62" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ Maritim: overview tinggi gelombang (232 wilayah) — (belum terekam saat capture)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ Maritim: polygon 232 wilayah perairan — (belum terekam saat capture)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://publik.bmkg.go.id/event/source/dwt/apiDF_Darat/202609101600.json</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <b val="1"/>
-              <color rgb="FFCC0000"/>
-              <sz val="8"/>
-            </rPr>
-            <t xml:space="preserve"> *(proxy)</t>
-          </r>
-        </is>
-      </c>
-      <c r="G15" s="62" t="inlineStr">
-        <is>
-          <t>▸ Maritim: overview tinggi gelombang (232 wilayah)
-(tidak ada response live)
-▸ Maritim: polygon 232 wilayah perairan
-(tidak ada response live)
-▸ Maritim: detail cuaca/gelombang perairan
-{"code": "F.09", "name": "Teluk Jakarta", "issued": "2026-09-21 23:39 UTC", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "data": [{"valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "time_desc": "Hari ini", "weather": "Berawan", "weather_desc": "Hari ini untuk Teluk Jakarta diperkirakan berawan, dengan kecepatan angin pada umumnya 5 - 18 knot bertiup dari arah selatan, tinggi gelombang laut berkisar 0.5 - 1.25 m", "warning_desc": "Waspada Angin Kencang", "station_remark": "Digital forecast by BMKG", "wave_cat": …
-▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
-[["lampung","Kab. Lampung Tengah","Terusan Nunyai",-4.699604904679063,105.20665965569867,"5013584","2026-09-10 16:00:00",["78","26","1","SE","9.5"],"ndf"],["lampung","Kab. Lampung Tengah","Seputih Agung",-4.89787745875816,105.05458830281606,"5013578","2026-09-10 16:00:00",["80","26","3","SE","9.2"],"ndf"],["lampung","Kab. Lampung Utara","Kotabumi",-4.846956993233334,104.85804482373453,"501378","2026-09-10 16:00:00",["81","26","1","SE","11.7"],"ndf"],["lampung","Kab. Lampung Utara","Abung Barat",-4.865040896877758,104.69148255332641,"5013612","2026-09-10 16:00:00",["87","24","1","SE","5.5"],"nd …</t>
-        </is>
-      </c>
-      <c r="H15" s="59" t="inlineStr">
-        <is>
-          <t>▸ Maritim: overview tinggi gelombang (232 wilayah)
-  Dipakai: {code: issued, today, tomorrow, wave_desc}
-  → Ringkasan 232 wilayah → warna peta laut + legend gelombang.
-▸ Maritim: polygon 232 wilayah perairan
-  Dipakai: features[].geometry (polygon 232 wilayah)
-  → Polygon GeoJSON → layer batas wilayah perairan di peta.
-▸ Maritim: detail cuaca/gelombang perairan
-  Dipakai: data[] → weather_desc, wave_desc, wind_speed_min/max, warning_desc, time_desc
-  → Slot perairan resmi (Hari ini…H+3) → kartu maritim &amp; aktivitas pelayaran; currentSlot = slot pertama yang masih berlaku.
-▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
-  Dipakai: rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
-  → Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.</t>
-        </is>
-      </c>
-      <c r="I15" s="63" t="inlineStr">
-        <is>
-          <t>▸ Gelombang: 232 wilayah resmi (warna/legend live), klik → detail live — data asli dari API
-▸ Layer angin/cuaca: SNAPSHOT statis (sectors.json) — data statis (belum ada endpoint)
-▸ Mode Pelabuhan: snapshot ports.json (294) — hanya pelabuhan TERDEKAT yang live — data statis (belum ada endpoint)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="287.75" customHeight="1">
-      <c r="A16" s="58" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="59" t="inlineStr">
-        <is>
-          <t>Pelabuhan &amp; Pasut
-(port-tide)</t>
-        </is>
-      </c>
-      <c r="C16" s="60" t="n"/>
-      <c r="D16" s="61" t="inlineStr">
-        <is>
-          <t>✅ LIVE</t>
-        </is>
-      </c>
-      <c r="E16" s="59" t="inlineStr">
-        <is>
-          <t>▸ Maritim: daftar pelabuhan (294)
-▸ Maritim: detail pelabuhan + pasut</t>
-        </is>
-      </c>
-      <c r="F16" s="62" t="inlineStr">
-        <is>
-          <t>▸ [200] https://maritim.bmkg.go.id/public_api/pelabuhan_list
-▸ [200] https://maritim.bmkg.go.id/public_api/pelabuhan/0101_Sunda%20Kelapa.json</t>
-        </is>
-      </c>
-      <c r="G16" s="62" t="inlineStr">
-        <is>
-          <t>▸ Maritim: daftar pelabuhan (294)
-{ "files": [ { "coor": [ 1.198331, 109.054462 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1720, "name": "0088_Sintete.json", "portname": "Sintete", "type": "utama" }, { "coor": [ 0.00214, 109.285391 ], "file_date": "2026-09-21 23:47 UTC", "kb": 1713, "name": "0310_PPP Sungai Rengas.json", "portname": "PPP Sungai Rengas", "type": "utama" }, { "coor": [ -2.531535, 110.21588 ], "file_date": "2026-09-21 23:47 UTC", "kb": …
-▸ Maritim: detail pelabuhan + pasut
-{"port_id": "0101", "name": "Sunda Kelapa", "info": "Per 17 Februari 2025 layanan API ini sepenuhnya menggunakan data digital hasil pemodelan BMKG", "latitude": -6.11664888, "longitude": 106.80830956, "type": "utama", "data": [{"issued": "2026-09-21 23:47 UTC", "valid_from": "2026-09-21 12:00 UTC", "valid_to": "2026-09-22 00:00 UTC", "weather": "Berawan", "weather_desc": "Untuk area Sunda Kelapa diperkirakan berawan, dengan kecepatan angin pada umumnya 2 - 14 knot bertiup dari arah timur", "warning_desc": "NIL", "wind_from": "Timur", "wind_to": "Utara", "wind_speed_min": 2, "wind_speed_max": 1 …</t>
-        </is>
-      </c>
-      <c r="H16" s="59" t="inlineStr">
-        <is>
-          <t>▸ Maritim: daftar pelabuhan (294)
-  Dipakai: files[].coor, file
-  → Koordinat 294 pelabuhan → pilih terdekat → fetch detail.
-▸ Maritim: detail pelabuhan + pasut
-  Dipakai: detail pelabuhan + data pasut
-  → Pasut (UTC → zona waktu pelabuhan) → PortTideCard; pasut null → blok disembunyikan.</t>
-        </is>
-      </c>
-      <c r="I16" s="63" t="inlineStr">
-        <is>
-          <t>Pasut null di sebagian pelabuhan → blok disembunyikan. Kolom arus di-skip (satuan ambigu).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="126.5" customHeight="1">
-      <c r="A17" s="58" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="59" t="inlineStr">
-        <is>
-          <t>Aktivitas Sekitar (POI)
-(around-activity)</t>
-        </is>
-      </c>
-      <c r="C17" s="60" t="n"/>
-      <c r="D17" s="65" t="inlineStr">
-        <is>
-          <t>⚠️ CAMPURAN</t>
-        </is>
-      </c>
-      <c r="E17" s="59" t="inlineStr">
-        <is>
-          <t>▸ DF Forecast: prakiraan 10 hari + per jam
-▸ Overpass API: POI OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="F17" s="62" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <b val="1"/>
-              <color rgb="FFCC0000"/>
-              <sz val="8"/>
-            </rPr>
-            <t xml:space="preserve"> *(proxy)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ Overpass API: POI OpenStreetMap — (belum terekam saat capture)</t>
-          </r>
-        </is>
-      </c>
-      <c r="G17" s="62" t="inlineStr">
-        <is>
-          <t>▸ DF Forecast: prakiraan 10 hari + per jam
-{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.82670735619568,"lat":-6.176384269281675,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.8267073562,"lat":-6.1763842693,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T09:00:00Z","t":28,"tcc":90,"tp":0,"weathe …
-▸ Overpass API: POI OpenStreetMap
-(tidak ada response live)</t>
-        </is>
-      </c>
-      <c r="H17" s="59" t="inlineStr">
-        <is>
-          <t>▸ DF Forecast: prakiraan 10 hari + per jam
-  Dipakai: data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
-  → Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
-▸ Overpass API: POI OpenStreetMap
-  Dipakai: elements[].lat/lon/tags
-  → POI OpenStreetMap sekitar pengguna → AroundActivity.</t>
-        </is>
-      </c>
-      <c r="I17" s="63" t="inlineStr">
-        <is>
-          <t>Nilai cuaca per titik POI live (1 request df/coord per POI).
-▸ Daftar POI: kurasi statis (cityLandmarks) — data statis (belum ada endpoint)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="279" customHeight="1">
-      <c r="A18" s="58" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="59" t="inlineStr">
-        <is>
-          <t>Aktivitas Darat (Drawer)
-(land-based)</t>
-        </is>
-      </c>
-      <c r="C18" s="60" t="n"/>
-      <c r="D18" s="65" t="inlineStr">
-        <is>
-          <t>⚠️ CAMPURAN</t>
-        </is>
-      </c>
-      <c r="E18" s="59" t="inlineStr">
-        <is>
-          <t>▸ DF Forecast: prakiraan 10 hari + per jam
-▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
-▸ Overpass API: POI OpenStreetMap
-▸ Nominatim: geocode OSM
-▸ OSRM: routing</t>
-        </is>
-      </c>
-      <c r="F18" s="62" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://cuaca.bmkg.go.id/api/df/v1/forecast/coord?lat=-6.1754&amp;lon=106.8272</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <b val="1"/>
-              <color rgb="FFCC0000"/>
-              <sz val="8"/>
-            </rPr>
-            <t xml:space="preserve"> *(proxy)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://publik.bmkg.go.id/event/source/dwt/apiDF_Darat/202609101600.json</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <b val="1"/>
-              <color rgb="FFCC0000"/>
-              <sz val="8"/>
-            </rPr>
-            <t xml:space="preserve"> *(proxy)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ Overpass API: POI OpenStreetMap — (belum terekam saat capture)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ Nominatim: geocode OSM — (belum terekam saat capture)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ OSRM: routing — (belum terekam saat capture)</t>
-          </r>
-        </is>
-      </c>
-      <c r="G18" s="62" t="inlineStr">
-        <is>
-          <t>▸ DF Forecast: prakiraan 10 hari + per jam
-{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.82670735619568,"lat":-6.176384269281675,"distance":0,"timezone":"Asia/Jakarta"},"data":[{"lokasi":{"adm1":"31","adm2":"31.71","adm3":"31.71.01","adm4":"31.71.01.1001","provinsi":"DKI Jakarta","kotkab":"Kota Adm. Jakarta Pusat","kecamatan":"Gambir","desa":"Gambir","lon":106.8267073562,"lat":-6.1763842693,"timezone":"+0700","type":"adm4"},"cuaca":[[{"datetime":"2026-09-22T09:00:00Z","t":28,"tcc":90,"tp":0,"weathe …
-▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
-[["lampung","Kab. Lampung Tengah","Terusan Nunyai",-4.699604904679063,105.20665965569867,"5013584","2026-09-10 16:00:00",["78","26","1","SE","9.5"],"ndf"],["lampung","Kab. Lampung Tengah","Seputih Agung",-4.89787745875816,105.05458830281606,"5013578","2026-09-10 16:00:00",["80","26","3","SE","9.2"],"ndf"],["lampung","Kab. Lampung Utara","Kotabumi",-4.846956993233334,104.85804482373453,"501378","2026-09-10 16:00:00",["81","26","1","SE","11.7"],"ndf"],["lampung","Kab. Lampung Utara","Abung Barat",-4.865040896877758,104.69148255332641,"5013612","2026-09-10 16:00:00",["87","24","1","SE","5.5"],"nd …
-▸ Overpass API: POI OpenStreetMap
-(tidak ada response live)
-▸ Nominatim: geocode OSM
-(tidak ada response live)
-▸ OSRM: routing
-(tidak ada response live)</t>
-        </is>
-      </c>
-      <c r="H18" s="59" t="inlineStr">
-        <is>
-          <t>▸ DF Forecast: prakiraan 10 hari + per jam
-  Dipakai: data[0].cuaca[][] → t, hu, weather_desc, tp, ws, tcc, local_datetime
-  → Suhu &amp; kelembapan; weather_desc → ikon lucide (descToIcon); hujan mm → % (tp×20, aproksimasi); local_datetime → urutan jam &amp; strip 7 hari (slot pertama tiap grup). API tidak punya tmin/tmax/UV → diestimasi.
-▸ DWT: cuaca kecamatan/stasiun (jalan+kereta)
-  Dipakai: rows [kota, kecamatan/stasiun, lat, lng, id, waktu, slots cuaca[]]
-  → Cuaca kecamatan (jalan raya) &amp; stasiun (kereta) terdekat ≤2° → kartu transportasi.
-▸ Overpass API: POI OpenStreetMap
-  Dipakai: elements[].lat/lon/tags
-  → POI OpenStreetMap sekitar pengguna → AroundActivity.
-▸ Nominatim: geocode OSM
-  Dipakai: [].lat/lon/display_name
-  → Geocode nama tempat → koordinat.
-▸ OSRM: routing
-  Dipakai: routes[].geometry, duration, distance
-  → Rute antar titik → panel aktivitas darat.</t>
-        </is>
-      </c>
-      <c r="I18" s="63" t="inlineStr">
-        <is>
-          <t>Forecast per titik rute live; fallback mock saat API gagal.
-▸ Pilihan lokasi awal: daftar statis — data statis (belum ada endpoint)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="271.25" customHeight="1">
-      <c r="A19" s="58" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="59" t="inlineStr">
-        <is>
-          <t>Konsultasi Pelayaran (Drawer)
-(maritime-advisor)</t>
-        </is>
-      </c>
-      <c r="C19" s="60" t="n"/>
-      <c r="D19" s="65" t="inlineStr">
-        <is>
-          <t>⚠️ CAMPURAN</t>
-        </is>
-      </c>
-      <c r="E19" s="59" t="inlineStr">
-        <is>
-          <t>▸ ISDP v1: wilayah laut terdekat
-▸ Maritim: detail cuaca/gelombang perairan</t>
-        </is>
-      </c>
-      <c r="F19" s="62" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://cuaca.bmkg.go.id/api/v1/public/maritim/nearest-location?lat=-6.2&amp;long=106.816666</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <b val="1"/>
-              <color rgb="FFCC0000"/>
-              <sz val="8"/>
-            </rPr>
-            <t xml:space="preserve"> *(proxy)</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Courier New"/>
-              <sz val="8"/>
-            </rPr>
-            <t>▸ [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
+            <t xml:space="preserve">
+▸ [200] https://maritim.bmkg.go.id/public_api/perairan/F.09_Teluk%20Jakarta.json</t>
           </r>
         </is>
       </c>

</xml_diff>